<commit_message>
them giao dien cho mobile va tablet, fix 1 so loi giao dien
</commit_message>
<xml_diff>
--- a/backend/public/lichmau.xlsx
+++ b/backend/public/lichmau.xlsx
@@ -13,6 +13,7 @@
     <sheet sheetId="4" name="19_01-25_01" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="26_01-01_02" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="02_02-08_02" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="09_02-15_02" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'29_12-04_01'!$6:$6</definedName>
@@ -21,13 +22,14 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'19_01-25_01'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'26_01-01_02'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'02_02-08_02'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'09_02-15_02'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="248">
   <si>
     <t>TRƯỜNG ĐẠI HỌC THÁI BÌNH</t>
   </si>
@@ -862,6 +864,37 @@
   </si>
   <si>
     <t>Unit A</t>
+  </si>
+  <si>
+    <t>(Từ ngày 09/02/2026 đến ngày 15/02/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Hai
+ ngày 09/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba
+ ngày 10/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Tư
+ ngày 11/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Năm
+ ngày 12/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Sáu
+ ngày 13/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Bảy
+ ngày 14/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ Nhật
+ ngày 15/02</t>
   </si>
 </sst>
 </file>
@@ -8051,4 +8084,753 @@
   <pageMargins left="0.2362204724409449" right="0" top="0.2362204724409449" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="37.44140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="41.109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" style="5" customWidth="1"/>
+    <col min="9" max="256" width="9" style="1" customWidth="1"/>
+    <col min="257" max="257" width="9.33203125" style="1" customWidth="1"/>
+    <col min="258" max="258" width="6.33203125" style="1" customWidth="1"/>
+    <col min="259" max="259" width="47" style="1" customWidth="1"/>
+    <col min="260" max="260" width="43.33203125" style="1" customWidth="1"/>
+    <col min="261" max="261" width="13.33203125" style="1" customWidth="1"/>
+    <col min="262" max="262" width="10.6640625" style="1" customWidth="1"/>
+    <col min="263" max="263" width="12.44140625" style="1" customWidth="1"/>
+    <col min="264" max="264" width="12.109375" style="1" customWidth="1"/>
+    <col min="265" max="512" width="9" style="1" customWidth="1"/>
+    <col min="513" max="513" width="9.33203125" style="1" customWidth="1"/>
+    <col min="514" max="514" width="6.33203125" style="1" customWidth="1"/>
+    <col min="515" max="515" width="47" style="1" customWidth="1"/>
+    <col min="516" max="516" width="43.33203125" style="1" customWidth="1"/>
+    <col min="517" max="517" width="13.33203125" style="1" customWidth="1"/>
+    <col min="518" max="518" width="10.6640625" style="1" customWidth="1"/>
+    <col min="519" max="519" width="12.44140625" style="1" customWidth="1"/>
+    <col min="520" max="520" width="12.109375" style="1" customWidth="1"/>
+    <col min="521" max="768" width="9" style="1" customWidth="1"/>
+    <col min="769" max="769" width="9.33203125" style="1" customWidth="1"/>
+    <col min="770" max="770" width="6.33203125" style="1" customWidth="1"/>
+    <col min="771" max="771" width="47" style="1" customWidth="1"/>
+    <col min="772" max="772" width="43.33203125" style="1" customWidth="1"/>
+    <col min="773" max="773" width="13.33203125" style="1" customWidth="1"/>
+    <col min="774" max="774" width="10.6640625" style="1" customWidth="1"/>
+    <col min="775" max="775" width="12.44140625" style="1" customWidth="1"/>
+    <col min="776" max="776" width="12.109375" style="1" customWidth="1"/>
+    <col min="777" max="1024" width="9" style="1" customWidth="1"/>
+    <col min="1025" max="1025" width="9.33203125" style="1" customWidth="1"/>
+    <col min="1026" max="1026" width="6.33203125" style="1" customWidth="1"/>
+    <col min="1027" max="1027" width="47" style="1" customWidth="1"/>
+    <col min="1028" max="1028" width="43.33203125" style="1" customWidth="1"/>
+    <col min="1029" max="1029" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1030" max="1030" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1031" max="1031" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1032" max="1032" width="12.109375" style="1" customWidth="1"/>
+    <col min="1033" max="1280" width="9" style="1" customWidth="1"/>
+    <col min="1281" max="1281" width="9.33203125" style="1" customWidth="1"/>
+    <col min="1282" max="1282" width="6.33203125" style="1" customWidth="1"/>
+    <col min="1283" max="1283" width="47" style="1" customWidth="1"/>
+    <col min="1284" max="1284" width="43.33203125" style="1" customWidth="1"/>
+    <col min="1285" max="1285" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1286" max="1286" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1287" max="1287" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1288" max="1288" width="12.109375" style="1" customWidth="1"/>
+    <col min="1289" max="1536" width="9" style="1" customWidth="1"/>
+    <col min="1537" max="1537" width="9.33203125" style="1" customWidth="1"/>
+    <col min="1538" max="1538" width="6.33203125" style="1" customWidth="1"/>
+    <col min="1539" max="1539" width="47" style="1" customWidth="1"/>
+    <col min="1540" max="1540" width="43.33203125" style="1" customWidth="1"/>
+    <col min="1541" max="1541" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1542" max="1542" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1543" max="1543" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1544" max="1544" width="12.109375" style="1" customWidth="1"/>
+    <col min="1545" max="1792" width="9" style="1" customWidth="1"/>
+    <col min="1793" max="1793" width="9.33203125" style="1" customWidth="1"/>
+    <col min="1794" max="1794" width="6.33203125" style="1" customWidth="1"/>
+    <col min="1795" max="1795" width="47" style="1" customWidth="1"/>
+    <col min="1796" max="1796" width="43.33203125" style="1" customWidth="1"/>
+    <col min="1797" max="1797" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1798" max="1798" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1799" max="1799" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1800" max="1800" width="12.109375" style="1" customWidth="1"/>
+    <col min="1801" max="2048" width="9" style="1" customWidth="1"/>
+    <col min="2049" max="2049" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2050" max="2050" width="6.33203125" style="1" customWidth="1"/>
+    <col min="2051" max="2051" width="47" style="1" customWidth="1"/>
+    <col min="2052" max="2052" width="43.33203125" style="1" customWidth="1"/>
+    <col min="2053" max="2053" width="13.33203125" style="1" customWidth="1"/>
+    <col min="2054" max="2054" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2055" max="2055" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2056" max="2056" width="12.109375" style="1" customWidth="1"/>
+    <col min="2057" max="2304" width="9" style="1" customWidth="1"/>
+    <col min="2305" max="2305" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2306" max="2306" width="6.33203125" style="1" customWidth="1"/>
+    <col min="2307" max="2307" width="47" style="1" customWidth="1"/>
+    <col min="2308" max="2308" width="43.33203125" style="1" customWidth="1"/>
+    <col min="2309" max="2309" width="13.33203125" style="1" customWidth="1"/>
+    <col min="2310" max="2310" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2311" max="2311" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2312" max="2312" width="12.109375" style="1" customWidth="1"/>
+    <col min="2313" max="2560" width="9" style="1" customWidth="1"/>
+    <col min="2561" max="2561" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2562" max="2562" width="6.33203125" style="1" customWidth="1"/>
+    <col min="2563" max="2563" width="47" style="1" customWidth="1"/>
+    <col min="2564" max="2564" width="43.33203125" style="1" customWidth="1"/>
+    <col min="2565" max="2565" width="13.33203125" style="1" customWidth="1"/>
+    <col min="2566" max="2566" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2567" max="2567" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2568" max="2568" width="12.109375" style="1" customWidth="1"/>
+    <col min="2569" max="2816" width="9" style="1" customWidth="1"/>
+    <col min="2817" max="2817" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2818" max="2818" width="6.33203125" style="1" customWidth="1"/>
+    <col min="2819" max="2819" width="47" style="1" customWidth="1"/>
+    <col min="2820" max="2820" width="43.33203125" style="1" customWidth="1"/>
+    <col min="2821" max="2821" width="13.33203125" style="1" customWidth="1"/>
+    <col min="2822" max="2822" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2823" max="2823" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2824" max="2824" width="12.109375" style="1" customWidth="1"/>
+    <col min="2825" max="3072" width="9" style="1" customWidth="1"/>
+    <col min="3073" max="3073" width="9.33203125" style="1" customWidth="1"/>
+    <col min="3074" max="3074" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3075" max="3075" width="47" style="1" customWidth="1"/>
+    <col min="3076" max="3076" width="43.33203125" style="1" customWidth="1"/>
+    <col min="3077" max="3077" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3078" max="3078" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3079" max="3079" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3080" max="3080" width="12.109375" style="1" customWidth="1"/>
+    <col min="3081" max="3328" width="9" style="1" customWidth="1"/>
+    <col min="3329" max="3329" width="9.33203125" style="1" customWidth="1"/>
+    <col min="3330" max="3330" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3331" max="3331" width="47" style="1" customWidth="1"/>
+    <col min="3332" max="3332" width="43.33203125" style="1" customWidth="1"/>
+    <col min="3333" max="3333" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3334" max="3334" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3335" max="3335" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3336" max="3336" width="12.109375" style="1" customWidth="1"/>
+    <col min="3337" max="3584" width="9" style="1" customWidth="1"/>
+    <col min="3585" max="3585" width="9.33203125" style="1" customWidth="1"/>
+    <col min="3586" max="3586" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3587" max="3587" width="47" style="1" customWidth="1"/>
+    <col min="3588" max="3588" width="43.33203125" style="1" customWidth="1"/>
+    <col min="3589" max="3589" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3590" max="3590" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3591" max="3591" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3592" max="3592" width="12.109375" style="1" customWidth="1"/>
+    <col min="3593" max="3840" width="9" style="1" customWidth="1"/>
+    <col min="3841" max="3841" width="9.33203125" style="1" customWidth="1"/>
+    <col min="3842" max="3842" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3843" max="3843" width="47" style="1" customWidth="1"/>
+    <col min="3844" max="3844" width="43.33203125" style="1" customWidth="1"/>
+    <col min="3845" max="3845" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3846" max="3846" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3847" max="3847" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3848" max="3848" width="12.109375" style="1" customWidth="1"/>
+    <col min="3849" max="4096" width="9" style="1" customWidth="1"/>
+    <col min="4097" max="4097" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4098" max="4098" width="6.33203125" style="1" customWidth="1"/>
+    <col min="4099" max="4099" width="47" style="1" customWidth="1"/>
+    <col min="4100" max="4100" width="43.33203125" style="1" customWidth="1"/>
+    <col min="4101" max="4101" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4102" max="4102" width="10.6640625" style="1" customWidth="1"/>
+    <col min="4103" max="4103" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4104" max="4104" width="12.109375" style="1" customWidth="1"/>
+    <col min="4105" max="4352" width="9" style="1" customWidth="1"/>
+    <col min="4353" max="4353" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4354" max="4354" width="6.33203125" style="1" customWidth="1"/>
+    <col min="4355" max="4355" width="47" style="1" customWidth="1"/>
+    <col min="4356" max="4356" width="43.33203125" style="1" customWidth="1"/>
+    <col min="4357" max="4357" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4358" max="4358" width="10.6640625" style="1" customWidth="1"/>
+    <col min="4359" max="4359" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4360" max="4360" width="12.109375" style="1" customWidth="1"/>
+    <col min="4361" max="4608" width="9" style="1" customWidth="1"/>
+    <col min="4609" max="4609" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4610" max="4610" width="6.33203125" style="1" customWidth="1"/>
+    <col min="4611" max="4611" width="47" style="1" customWidth="1"/>
+    <col min="4612" max="4612" width="43.33203125" style="1" customWidth="1"/>
+    <col min="4613" max="4613" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4614" max="4614" width="10.6640625" style="1" customWidth="1"/>
+    <col min="4615" max="4615" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4616" max="4616" width="12.109375" style="1" customWidth="1"/>
+    <col min="4617" max="4864" width="9" style="1" customWidth="1"/>
+    <col min="4865" max="4865" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4866" max="4866" width="6.33203125" style="1" customWidth="1"/>
+    <col min="4867" max="4867" width="47" style="1" customWidth="1"/>
+    <col min="4868" max="4868" width="43.33203125" style="1" customWidth="1"/>
+    <col min="4869" max="4869" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4870" max="4870" width="10.6640625" style="1" customWidth="1"/>
+    <col min="4871" max="4871" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4872" max="4872" width="12.109375" style="1" customWidth="1"/>
+    <col min="4873" max="5120" width="9" style="1" customWidth="1"/>
+    <col min="5121" max="5121" width="9.33203125" style="1" customWidth="1"/>
+    <col min="5122" max="5122" width="6.33203125" style="1" customWidth="1"/>
+    <col min="5123" max="5123" width="47" style="1" customWidth="1"/>
+    <col min="5124" max="5124" width="43.33203125" style="1" customWidth="1"/>
+    <col min="5125" max="5125" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5126" max="5126" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5127" max="5127" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5128" max="5128" width="12.109375" style="1" customWidth="1"/>
+    <col min="5129" max="5376" width="9" style="1" customWidth="1"/>
+    <col min="5377" max="5377" width="9.33203125" style="1" customWidth="1"/>
+    <col min="5378" max="5378" width="6.33203125" style="1" customWidth="1"/>
+    <col min="5379" max="5379" width="47" style="1" customWidth="1"/>
+    <col min="5380" max="5380" width="43.33203125" style="1" customWidth="1"/>
+    <col min="5381" max="5381" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5382" max="5382" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5383" max="5383" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5384" max="5384" width="12.109375" style="1" customWidth="1"/>
+    <col min="5385" max="5632" width="9" style="1" customWidth="1"/>
+    <col min="5633" max="5633" width="9.33203125" style="1" customWidth="1"/>
+    <col min="5634" max="5634" width="6.33203125" style="1" customWidth="1"/>
+    <col min="5635" max="5635" width="47" style="1" customWidth="1"/>
+    <col min="5636" max="5636" width="43.33203125" style="1" customWidth="1"/>
+    <col min="5637" max="5637" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5638" max="5638" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5639" max="5639" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5640" max="5640" width="12.109375" style="1" customWidth="1"/>
+    <col min="5641" max="5888" width="9" style="1" customWidth="1"/>
+    <col min="5889" max="5889" width="9.33203125" style="1" customWidth="1"/>
+    <col min="5890" max="5890" width="6.33203125" style="1" customWidth="1"/>
+    <col min="5891" max="5891" width="47" style="1" customWidth="1"/>
+    <col min="5892" max="5892" width="43.33203125" style="1" customWidth="1"/>
+    <col min="5893" max="5893" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5894" max="5894" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5895" max="5895" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5896" max="5896" width="12.109375" style="1" customWidth="1"/>
+    <col min="5897" max="6144" width="9" style="1" customWidth="1"/>
+    <col min="6145" max="6145" width="9.33203125" style="1" customWidth="1"/>
+    <col min="6146" max="6146" width="6.33203125" style="1" customWidth="1"/>
+    <col min="6147" max="6147" width="47" style="1" customWidth="1"/>
+    <col min="6148" max="6148" width="43.33203125" style="1" customWidth="1"/>
+    <col min="6149" max="6149" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6150" max="6150" width="10.6640625" style="1" customWidth="1"/>
+    <col min="6151" max="6151" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6152" max="6152" width="12.109375" style="1" customWidth="1"/>
+    <col min="6153" max="6400" width="9" style="1" customWidth="1"/>
+    <col min="6401" max="6401" width="9.33203125" style="1" customWidth="1"/>
+    <col min="6402" max="6402" width="6.33203125" style="1" customWidth="1"/>
+    <col min="6403" max="6403" width="47" style="1" customWidth="1"/>
+    <col min="6404" max="6404" width="43.33203125" style="1" customWidth="1"/>
+    <col min="6405" max="6405" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6406" max="6406" width="10.6640625" style="1" customWidth="1"/>
+    <col min="6407" max="6407" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6408" max="6408" width="12.109375" style="1" customWidth="1"/>
+    <col min="6409" max="6656" width="9" style="1" customWidth="1"/>
+    <col min="6657" max="6657" width="9.33203125" style="1" customWidth="1"/>
+    <col min="6658" max="6658" width="6.33203125" style="1" customWidth="1"/>
+    <col min="6659" max="6659" width="47" style="1" customWidth="1"/>
+    <col min="6660" max="6660" width="43.33203125" style="1" customWidth="1"/>
+    <col min="6661" max="6661" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6662" max="6662" width="10.6640625" style="1" customWidth="1"/>
+    <col min="6663" max="6663" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6664" max="6664" width="12.109375" style="1" customWidth="1"/>
+    <col min="6665" max="6912" width="9" style="1" customWidth="1"/>
+    <col min="6913" max="6913" width="9.33203125" style="1" customWidth="1"/>
+    <col min="6914" max="6914" width="6.33203125" style="1" customWidth="1"/>
+    <col min="6915" max="6915" width="47" style="1" customWidth="1"/>
+    <col min="6916" max="6916" width="43.33203125" style="1" customWidth="1"/>
+    <col min="6917" max="6917" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6918" max="6918" width="10.6640625" style="1" customWidth="1"/>
+    <col min="6919" max="6919" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6920" max="6920" width="12.109375" style="1" customWidth="1"/>
+    <col min="6921" max="7168" width="9" style="1" customWidth="1"/>
+    <col min="7169" max="7169" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7170" max="7170" width="6.33203125" style="1" customWidth="1"/>
+    <col min="7171" max="7171" width="47" style="1" customWidth="1"/>
+    <col min="7172" max="7172" width="43.33203125" style="1" customWidth="1"/>
+    <col min="7173" max="7173" width="13.33203125" style="1" customWidth="1"/>
+    <col min="7174" max="7174" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7175" max="7175" width="12.44140625" style="1" customWidth="1"/>
+    <col min="7176" max="7176" width="12.109375" style="1" customWidth="1"/>
+    <col min="7177" max="7424" width="9" style="1" customWidth="1"/>
+    <col min="7425" max="7425" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7426" max="7426" width="6.33203125" style="1" customWidth="1"/>
+    <col min="7427" max="7427" width="47" style="1" customWidth="1"/>
+    <col min="7428" max="7428" width="43.33203125" style="1" customWidth="1"/>
+    <col min="7429" max="7429" width="13.33203125" style="1" customWidth="1"/>
+    <col min="7430" max="7430" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7431" max="7431" width="12.44140625" style="1" customWidth="1"/>
+    <col min="7432" max="7432" width="12.109375" style="1" customWidth="1"/>
+    <col min="7433" max="7680" width="9" style="1" customWidth="1"/>
+    <col min="7681" max="7681" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7682" max="7682" width="6.33203125" style="1" customWidth="1"/>
+    <col min="7683" max="7683" width="47" style="1" customWidth="1"/>
+    <col min="7684" max="7684" width="43.33203125" style="1" customWidth="1"/>
+    <col min="7685" max="7685" width="13.33203125" style="1" customWidth="1"/>
+    <col min="7686" max="7686" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7687" max="7687" width="12.44140625" style="1" customWidth="1"/>
+    <col min="7688" max="7688" width="12.109375" style="1" customWidth="1"/>
+    <col min="7689" max="7936" width="9" style="1" customWidth="1"/>
+    <col min="7937" max="7937" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7938" max="7938" width="6.33203125" style="1" customWidth="1"/>
+    <col min="7939" max="7939" width="47" style="1" customWidth="1"/>
+    <col min="7940" max="7940" width="43.33203125" style="1" customWidth="1"/>
+    <col min="7941" max="7941" width="13.33203125" style="1" customWidth="1"/>
+    <col min="7942" max="7942" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7943" max="7943" width="12.44140625" style="1" customWidth="1"/>
+    <col min="7944" max="7944" width="12.109375" style="1" customWidth="1"/>
+    <col min="7945" max="8192" width="9" style="1" customWidth="1"/>
+    <col min="8193" max="8193" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8194" max="8194" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8195" max="8195" width="47" style="1" customWidth="1"/>
+    <col min="8196" max="8196" width="43.33203125" style="1" customWidth="1"/>
+    <col min="8197" max="8197" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8198" max="8198" width="10.6640625" style="1" customWidth="1"/>
+    <col min="8199" max="8199" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8200" max="8200" width="12.109375" style="1" customWidth="1"/>
+    <col min="8201" max="8448" width="9" style="1" customWidth="1"/>
+    <col min="8449" max="8449" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8450" max="8450" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8451" max="8451" width="47" style="1" customWidth="1"/>
+    <col min="8452" max="8452" width="43.33203125" style="1" customWidth="1"/>
+    <col min="8453" max="8453" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8454" max="8454" width="10.6640625" style="1" customWidth="1"/>
+    <col min="8455" max="8455" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8456" max="8456" width="12.109375" style="1" customWidth="1"/>
+    <col min="8457" max="8704" width="9" style="1" customWidth="1"/>
+    <col min="8705" max="8705" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8706" max="8706" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8707" max="8707" width="47" style="1" customWidth="1"/>
+    <col min="8708" max="8708" width="43.33203125" style="1" customWidth="1"/>
+    <col min="8709" max="8709" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8710" max="8710" width="10.6640625" style="1" customWidth="1"/>
+    <col min="8711" max="8711" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8712" max="8712" width="12.109375" style="1" customWidth="1"/>
+    <col min="8713" max="8960" width="9" style="1" customWidth="1"/>
+    <col min="8961" max="8961" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8962" max="8962" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8963" max="8963" width="47" style="1" customWidth="1"/>
+    <col min="8964" max="8964" width="43.33203125" style="1" customWidth="1"/>
+    <col min="8965" max="8965" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8966" max="8966" width="10.6640625" style="1" customWidth="1"/>
+    <col min="8967" max="8967" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8968" max="8968" width="12.109375" style="1" customWidth="1"/>
+    <col min="8969" max="9216" width="9" style="1" customWidth="1"/>
+    <col min="9217" max="9217" width="9.33203125" style="1" customWidth="1"/>
+    <col min="9218" max="9218" width="6.33203125" style="1" customWidth="1"/>
+    <col min="9219" max="9219" width="47" style="1" customWidth="1"/>
+    <col min="9220" max="9220" width="43.33203125" style="1" customWidth="1"/>
+    <col min="9221" max="9221" width="13.33203125" style="1" customWidth="1"/>
+    <col min="9222" max="9222" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9223" max="9223" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9224" max="9224" width="12.109375" style="1" customWidth="1"/>
+    <col min="9225" max="9472" width="9" style="1" customWidth="1"/>
+    <col min="9473" max="9473" width="9.33203125" style="1" customWidth="1"/>
+    <col min="9474" max="9474" width="6.33203125" style="1" customWidth="1"/>
+    <col min="9475" max="9475" width="47" style="1" customWidth="1"/>
+    <col min="9476" max="9476" width="43.33203125" style="1" customWidth="1"/>
+    <col min="9477" max="9477" width="13.33203125" style="1" customWidth="1"/>
+    <col min="9478" max="9478" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9479" max="9479" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9480" max="9480" width="12.109375" style="1" customWidth="1"/>
+    <col min="9481" max="9728" width="9" style="1" customWidth="1"/>
+    <col min="9729" max="9729" width="9.33203125" style="1" customWidth="1"/>
+    <col min="9730" max="9730" width="6.33203125" style="1" customWidth="1"/>
+    <col min="9731" max="9731" width="47" style="1" customWidth="1"/>
+    <col min="9732" max="9732" width="43.33203125" style="1" customWidth="1"/>
+    <col min="9733" max="9733" width="13.33203125" style="1" customWidth="1"/>
+    <col min="9734" max="9734" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9735" max="9735" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9736" max="9736" width="12.109375" style="1" customWidth="1"/>
+    <col min="9737" max="9984" width="9" style="1" customWidth="1"/>
+    <col min="9985" max="9985" width="9.33203125" style="1" customWidth="1"/>
+    <col min="9986" max="9986" width="6.33203125" style="1" customWidth="1"/>
+    <col min="9987" max="9987" width="47" style="1" customWidth="1"/>
+    <col min="9988" max="9988" width="43.33203125" style="1" customWidth="1"/>
+    <col min="9989" max="9989" width="13.33203125" style="1" customWidth="1"/>
+    <col min="9990" max="9990" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9991" max="9991" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9992" max="9992" width="12.109375" style="1" customWidth="1"/>
+    <col min="9993" max="10240" width="9" style="1" customWidth="1"/>
+    <col min="10241" max="10241" width="9.33203125" style="1" customWidth="1"/>
+    <col min="10242" max="10242" width="6.33203125" style="1" customWidth="1"/>
+    <col min="10243" max="10243" width="47" style="1" customWidth="1"/>
+    <col min="10244" max="10244" width="43.33203125" style="1" customWidth="1"/>
+    <col min="10245" max="10245" width="13.33203125" style="1" customWidth="1"/>
+    <col min="10246" max="10246" width="10.6640625" style="1" customWidth="1"/>
+    <col min="10247" max="10247" width="12.44140625" style="1" customWidth="1"/>
+    <col min="10248" max="10248" width="12.109375" style="1" customWidth="1"/>
+    <col min="10249" max="10496" width="9" style="1" customWidth="1"/>
+    <col min="10497" max="10497" width="9.33203125" style="1" customWidth="1"/>
+    <col min="10498" max="10498" width="6.33203125" style="1" customWidth="1"/>
+    <col min="10499" max="10499" width="47" style="1" customWidth="1"/>
+    <col min="10500" max="10500" width="43.33203125" style="1" customWidth="1"/>
+    <col min="10501" max="10501" width="13.33203125" style="1" customWidth="1"/>
+    <col min="10502" max="10502" width="10.6640625" style="1" customWidth="1"/>
+    <col min="10503" max="10503" width="12.44140625" style="1" customWidth="1"/>
+    <col min="10504" max="10504" width="12.109375" style="1" customWidth="1"/>
+    <col min="10505" max="10752" width="9" style="1" customWidth="1"/>
+    <col min="10753" max="10753" width="9.33203125" style="1" customWidth="1"/>
+    <col min="10754" max="10754" width="6.33203125" style="1" customWidth="1"/>
+    <col min="10755" max="10755" width="47" style="1" customWidth="1"/>
+    <col min="10756" max="10756" width="43.33203125" style="1" customWidth="1"/>
+    <col min="10757" max="10757" width="13.33203125" style="1" customWidth="1"/>
+    <col min="10758" max="10758" width="10.6640625" style="1" customWidth="1"/>
+    <col min="10759" max="10759" width="12.44140625" style="1" customWidth="1"/>
+    <col min="10760" max="10760" width="12.109375" style="1" customWidth="1"/>
+    <col min="10761" max="11008" width="9" style="1" customWidth="1"/>
+    <col min="11009" max="11009" width="9.33203125" style="1" customWidth="1"/>
+    <col min="11010" max="11010" width="6.33203125" style="1" customWidth="1"/>
+    <col min="11011" max="11011" width="47" style="1" customWidth="1"/>
+    <col min="11012" max="11012" width="43.33203125" style="1" customWidth="1"/>
+    <col min="11013" max="11013" width="13.33203125" style="1" customWidth="1"/>
+    <col min="11014" max="11014" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11015" max="11015" width="12.44140625" style="1" customWidth="1"/>
+    <col min="11016" max="11016" width="12.109375" style="1" customWidth="1"/>
+    <col min="11017" max="11264" width="9" style="1" customWidth="1"/>
+    <col min="11265" max="11265" width="9.33203125" style="1" customWidth="1"/>
+    <col min="11266" max="11266" width="6.33203125" style="1" customWidth="1"/>
+    <col min="11267" max="11267" width="47" style="1" customWidth="1"/>
+    <col min="11268" max="11268" width="43.33203125" style="1" customWidth="1"/>
+    <col min="11269" max="11269" width="13.33203125" style="1" customWidth="1"/>
+    <col min="11270" max="11270" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11271" max="11271" width="12.44140625" style="1" customWidth="1"/>
+    <col min="11272" max="11272" width="12.109375" style="1" customWidth="1"/>
+    <col min="11273" max="11520" width="9" style="1" customWidth="1"/>
+    <col min="11521" max="11521" width="9.33203125" style="1" customWidth="1"/>
+    <col min="11522" max="11522" width="6.33203125" style="1" customWidth="1"/>
+    <col min="11523" max="11523" width="47" style="1" customWidth="1"/>
+    <col min="11524" max="11524" width="43.33203125" style="1" customWidth="1"/>
+    <col min="11525" max="11525" width="13.33203125" style="1" customWidth="1"/>
+    <col min="11526" max="11526" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11527" max="11527" width="12.44140625" style="1" customWidth="1"/>
+    <col min="11528" max="11528" width="12.109375" style="1" customWidth="1"/>
+    <col min="11529" max="11776" width="9" style="1" customWidth="1"/>
+    <col min="11777" max="11777" width="9.33203125" style="1" customWidth="1"/>
+    <col min="11778" max="11778" width="6.33203125" style="1" customWidth="1"/>
+    <col min="11779" max="11779" width="47" style="1" customWidth="1"/>
+    <col min="11780" max="11780" width="43.33203125" style="1" customWidth="1"/>
+    <col min="11781" max="11781" width="13.33203125" style="1" customWidth="1"/>
+    <col min="11782" max="11782" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11783" max="11783" width="12.44140625" style="1" customWidth="1"/>
+    <col min="11784" max="11784" width="12.109375" style="1" customWidth="1"/>
+    <col min="11785" max="12032" width="9" style="1" customWidth="1"/>
+    <col min="12033" max="12033" width="9.33203125" style="1" customWidth="1"/>
+    <col min="12034" max="12034" width="6.33203125" style="1" customWidth="1"/>
+    <col min="12035" max="12035" width="47" style="1" customWidth="1"/>
+    <col min="12036" max="12036" width="43.33203125" style="1" customWidth="1"/>
+    <col min="12037" max="12037" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12038" max="12038" width="10.6640625" style="1" customWidth="1"/>
+    <col min="12039" max="12039" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12040" max="12040" width="12.109375" style="1" customWidth="1"/>
+    <col min="12041" max="12288" width="9" style="1" customWidth="1"/>
+    <col min="12289" max="12289" width="9.33203125" style="1" customWidth="1"/>
+    <col min="12290" max="12290" width="6.33203125" style="1" customWidth="1"/>
+    <col min="12291" max="12291" width="47" style="1" customWidth="1"/>
+    <col min="12292" max="12292" width="43.33203125" style="1" customWidth="1"/>
+    <col min="12293" max="12293" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12294" max="12294" width="10.6640625" style="1" customWidth="1"/>
+    <col min="12295" max="12295" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12296" max="12296" width="12.109375" style="1" customWidth="1"/>
+    <col min="12297" max="12544" width="9" style="1" customWidth="1"/>
+    <col min="12545" max="12545" width="9.33203125" style="1" customWidth="1"/>
+    <col min="12546" max="12546" width="6.33203125" style="1" customWidth="1"/>
+    <col min="12547" max="12547" width="47" style="1" customWidth="1"/>
+    <col min="12548" max="12548" width="43.33203125" style="1" customWidth="1"/>
+    <col min="12549" max="12549" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12550" max="12550" width="10.6640625" style="1" customWidth="1"/>
+    <col min="12551" max="12551" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12552" max="12552" width="12.109375" style="1" customWidth="1"/>
+    <col min="12553" max="12800" width="9" style="1" customWidth="1"/>
+    <col min="12801" max="12801" width="9.33203125" style="1" customWidth="1"/>
+    <col min="12802" max="12802" width="6.33203125" style="1" customWidth="1"/>
+    <col min="12803" max="12803" width="47" style="1" customWidth="1"/>
+    <col min="12804" max="12804" width="43.33203125" style="1" customWidth="1"/>
+    <col min="12805" max="12805" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12806" max="12806" width="10.6640625" style="1" customWidth="1"/>
+    <col min="12807" max="12807" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12808" max="12808" width="12.109375" style="1" customWidth="1"/>
+    <col min="12809" max="13056" width="9" style="1" customWidth="1"/>
+    <col min="13057" max="13057" width="9.33203125" style="1" customWidth="1"/>
+    <col min="13058" max="13058" width="6.33203125" style="1" customWidth="1"/>
+    <col min="13059" max="13059" width="47" style="1" customWidth="1"/>
+    <col min="13060" max="13060" width="43.33203125" style="1" customWidth="1"/>
+    <col min="13061" max="13061" width="13.33203125" style="1" customWidth="1"/>
+    <col min="13062" max="13062" width="10.6640625" style="1" customWidth="1"/>
+    <col min="13063" max="13063" width="12.44140625" style="1" customWidth="1"/>
+    <col min="13064" max="13064" width="12.109375" style="1" customWidth="1"/>
+    <col min="13065" max="13312" width="9" style="1" customWidth="1"/>
+    <col min="13313" max="13313" width="9.33203125" style="1" customWidth="1"/>
+    <col min="13314" max="13314" width="6.33203125" style="1" customWidth="1"/>
+    <col min="13315" max="13315" width="47" style="1" customWidth="1"/>
+    <col min="13316" max="13316" width="43.33203125" style="1" customWidth="1"/>
+    <col min="13317" max="13317" width="13.33203125" style="1" customWidth="1"/>
+    <col min="13318" max="13318" width="10.6640625" style="1" customWidth="1"/>
+    <col min="13319" max="13319" width="12.44140625" style="1" customWidth="1"/>
+    <col min="13320" max="13320" width="12.109375" style="1" customWidth="1"/>
+    <col min="13321" max="13568" width="9" style="1" customWidth="1"/>
+    <col min="13569" max="13569" width="9.33203125" style="1" customWidth="1"/>
+    <col min="13570" max="13570" width="6.33203125" style="1" customWidth="1"/>
+    <col min="13571" max="13571" width="47" style="1" customWidth="1"/>
+    <col min="13572" max="13572" width="43.33203125" style="1" customWidth="1"/>
+    <col min="13573" max="13573" width="13.33203125" style="1" customWidth="1"/>
+    <col min="13574" max="13574" width="10.6640625" style="1" customWidth="1"/>
+    <col min="13575" max="13575" width="12.44140625" style="1" customWidth="1"/>
+    <col min="13576" max="13576" width="12.109375" style="1" customWidth="1"/>
+    <col min="13577" max="13824" width="9" style="1" customWidth="1"/>
+    <col min="13825" max="13825" width="9.33203125" style="1" customWidth="1"/>
+    <col min="13826" max="13826" width="6.33203125" style="1" customWidth="1"/>
+    <col min="13827" max="13827" width="47" style="1" customWidth="1"/>
+    <col min="13828" max="13828" width="43.33203125" style="1" customWidth="1"/>
+    <col min="13829" max="13829" width="13.33203125" style="1" customWidth="1"/>
+    <col min="13830" max="13830" width="10.6640625" style="1" customWidth="1"/>
+    <col min="13831" max="13831" width="12.44140625" style="1" customWidth="1"/>
+    <col min="13832" max="13832" width="12.109375" style="1" customWidth="1"/>
+    <col min="13833" max="14080" width="9" style="1" customWidth="1"/>
+    <col min="14081" max="14081" width="9.33203125" style="1" customWidth="1"/>
+    <col min="14082" max="14082" width="6.33203125" style="1" customWidth="1"/>
+    <col min="14083" max="14083" width="47" style="1" customWidth="1"/>
+    <col min="14084" max="14084" width="43.33203125" style="1" customWidth="1"/>
+    <col min="14085" max="14085" width="13.33203125" style="1" customWidth="1"/>
+    <col min="14086" max="14086" width="10.6640625" style="1" customWidth="1"/>
+    <col min="14087" max="14087" width="12.44140625" style="1" customWidth="1"/>
+    <col min="14088" max="14088" width="12.109375" style="1" customWidth="1"/>
+    <col min="14089" max="14336" width="9" style="1" customWidth="1"/>
+    <col min="14337" max="14337" width="9.33203125" style="1" customWidth="1"/>
+    <col min="14338" max="14338" width="6.33203125" style="1" customWidth="1"/>
+    <col min="14339" max="14339" width="47" style="1" customWidth="1"/>
+    <col min="14340" max="14340" width="43.33203125" style="1" customWidth="1"/>
+    <col min="14341" max="14341" width="13.33203125" style="1" customWidth="1"/>
+    <col min="14342" max="14342" width="10.6640625" style="1" customWidth="1"/>
+    <col min="14343" max="14343" width="12.44140625" style="1" customWidth="1"/>
+    <col min="14344" max="14344" width="12.109375" style="1" customWidth="1"/>
+    <col min="14345" max="14592" width="9" style="1" customWidth="1"/>
+    <col min="14593" max="14593" width="9.33203125" style="1" customWidth="1"/>
+    <col min="14594" max="14594" width="6.33203125" style="1" customWidth="1"/>
+    <col min="14595" max="14595" width="47" style="1" customWidth="1"/>
+    <col min="14596" max="14596" width="43.33203125" style="1" customWidth="1"/>
+    <col min="14597" max="14597" width="13.33203125" style="1" customWidth="1"/>
+    <col min="14598" max="14598" width="10.6640625" style="1" customWidth="1"/>
+    <col min="14599" max="14599" width="12.44140625" style="1" customWidth="1"/>
+    <col min="14600" max="14600" width="12.109375" style="1" customWidth="1"/>
+    <col min="14601" max="14848" width="9" style="1" customWidth="1"/>
+    <col min="14849" max="14849" width="9.33203125" style="1" customWidth="1"/>
+    <col min="14850" max="14850" width="6.33203125" style="1" customWidth="1"/>
+    <col min="14851" max="14851" width="47" style="1" customWidth="1"/>
+    <col min="14852" max="14852" width="43.33203125" style="1" customWidth="1"/>
+    <col min="14853" max="14853" width="13.33203125" style="1" customWidth="1"/>
+    <col min="14854" max="14854" width="10.6640625" style="1" customWidth="1"/>
+    <col min="14855" max="14855" width="12.44140625" style="1" customWidth="1"/>
+    <col min="14856" max="14856" width="12.109375" style="1" customWidth="1"/>
+    <col min="14857" max="15104" width="9" style="1" customWidth="1"/>
+    <col min="15105" max="15105" width="9.33203125" style="1" customWidth="1"/>
+    <col min="15106" max="15106" width="6.33203125" style="1" customWidth="1"/>
+    <col min="15107" max="15107" width="47" style="1" customWidth="1"/>
+    <col min="15108" max="15108" width="43.33203125" style="1" customWidth="1"/>
+    <col min="15109" max="15109" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15110" max="15110" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15111" max="15111" width="12.44140625" style="1" customWidth="1"/>
+    <col min="15112" max="15112" width="12.109375" style="1" customWidth="1"/>
+    <col min="15113" max="15360" width="9" style="1" customWidth="1"/>
+    <col min="15361" max="15361" width="9.33203125" style="1" customWidth="1"/>
+    <col min="15362" max="15362" width="6.33203125" style="1" customWidth="1"/>
+    <col min="15363" max="15363" width="47" style="1" customWidth="1"/>
+    <col min="15364" max="15364" width="43.33203125" style="1" customWidth="1"/>
+    <col min="15365" max="15365" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15366" max="15366" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15367" max="15367" width="12.44140625" style="1" customWidth="1"/>
+    <col min="15368" max="15368" width="12.109375" style="1" customWidth="1"/>
+    <col min="15369" max="15616" width="9" style="1" customWidth="1"/>
+    <col min="15617" max="15617" width="9.33203125" style="1" customWidth="1"/>
+    <col min="15618" max="15618" width="6.33203125" style="1" customWidth="1"/>
+    <col min="15619" max="15619" width="47" style="1" customWidth="1"/>
+    <col min="15620" max="15620" width="43.33203125" style="1" customWidth="1"/>
+    <col min="15621" max="15621" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15622" max="15622" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15623" max="15623" width="12.44140625" style="1" customWidth="1"/>
+    <col min="15624" max="15624" width="12.109375" style="1" customWidth="1"/>
+    <col min="15625" max="15872" width="9" style="1" customWidth="1"/>
+    <col min="15873" max="15873" width="9.33203125" style="1" customWidth="1"/>
+    <col min="15874" max="15874" width="6.33203125" style="1" customWidth="1"/>
+    <col min="15875" max="15875" width="47" style="1" customWidth="1"/>
+    <col min="15876" max="15876" width="43.33203125" style="1" customWidth="1"/>
+    <col min="15877" max="15877" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15878" max="15878" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15879" max="15879" width="12.44140625" style="1" customWidth="1"/>
+    <col min="15880" max="15880" width="12.109375" style="1" customWidth="1"/>
+    <col min="15881" max="16128" width="9" style="1" customWidth="1"/>
+    <col min="16129" max="16129" width="9.33203125" style="1" customWidth="1"/>
+    <col min="16130" max="16130" width="6.33203125" style="1" customWidth="1"/>
+    <col min="16131" max="16131" width="47" style="1" customWidth="1"/>
+    <col min="16132" max="16132" width="43.33203125" style="1" customWidth="1"/>
+    <col min="16133" max="16133" width="13.33203125" style="1" customWidth="1"/>
+    <col min="16134" max="16134" width="10.6640625" style="1" customWidth="1"/>
+    <col min="16135" max="16135" width="12.44140625" style="1" customWidth="1"/>
+    <col min="16136" max="16136" width="12.109375" style="1" customWidth="1"/>
+    <col min="16137" max="16384" width="9" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+    </row>
+    <row r="2" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" ht="8.1" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+    </row>
+    <row r="4" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" ht="20.25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="108" t="s">
+        <v>241</v>
+      </c>
+      <c r="B7" s="21"/>
+      <c r="C7" s="68"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="31"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="108" t="s">
+        <v>242</v>
+      </c>
+      <c r="B8" s="21"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="31"/>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="108" t="s">
+        <v>243</v>
+      </c>
+      <c r="B9" s="21"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="68"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="31"/>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="108" t="s">
+        <v>244</v>
+      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="68"/>
+      <c r="D10" s="68"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="31"/>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="108" t="s">
+        <v>245</v>
+      </c>
+      <c r="B11" s="21"/>
+      <c r="C11" s="68"/>
+      <c r="D11" s="68"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="31"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="108" t="s">
+        <v>246</v>
+      </c>
+      <c r="B12" s="21"/>
+      <c r="C12" s="68"/>
+      <c r="D12" s="68"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="31"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="108" t="s">
+        <v>247</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="68"/>
+      <c r="D13" s="68"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.2362204724409449" right="0" top="0.2362204724409449" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
sua mot so chuc nang
</commit_message>
<xml_diff>
--- a/backend/public/lichmau.xlsx
+++ b/backend/public/lichmau.xlsx
@@ -14,6 +14,7 @@
     <sheet sheetId="5" name="26_01-01_02" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="02_02-08_02" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="09_02-15_02" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="23_02-01_03" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'29_12-04_01'!$6:$6</definedName>
@@ -23,13 +24,14 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'26_01-01_02'!$7:$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'02_02-08_02'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'09_02-15_02'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'23_02-01_03'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="258">
   <si>
     <t>TRƯỜNG ĐẠI HỌC THÁI BÌNH</t>
   </si>
@@ -895,6 +897,43 @@
   <si>
     <t xml:space="preserve">Chủ Nhật
  ngày 15/02</t>
+  </si>
+  <si>
+    <t>(Từ ngày 23/02/2026 đến ngày 01/03/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Hai
+ ngày 23/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba
+ ngày 24/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Tư
+ ngày 25/02</t>
+  </si>
+  <si>
+    <t>1, từ 16h00</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Năm
+ ngày 26/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Sáu
+ ngày 27/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Bảy
+ ngày 28/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ Nhật
+ ngày 01/03</t>
   </si>
 </sst>
 </file>
@@ -8833,4 +8872,777 @@
   <pageMargins left="0.2362204724409449" right="0" top="0.2362204724409449" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="6.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="37.44140625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="41.109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.33203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" style="2" customWidth="1"/>
+    <col min="7" max="7" width="12.44140625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" style="5" customWidth="1"/>
+    <col min="9" max="256" width="9" style="1" customWidth="1"/>
+    <col min="257" max="257" width="9.33203125" style="1" customWidth="1"/>
+    <col min="258" max="258" width="6.33203125" style="1" customWidth="1"/>
+    <col min="259" max="259" width="47" style="1" customWidth="1"/>
+    <col min="260" max="260" width="43.33203125" style="1" customWidth="1"/>
+    <col min="261" max="261" width="13.33203125" style="1" customWidth="1"/>
+    <col min="262" max="262" width="10.6640625" style="1" customWidth="1"/>
+    <col min="263" max="263" width="12.44140625" style="1" customWidth="1"/>
+    <col min="264" max="264" width="12.109375" style="1" customWidth="1"/>
+    <col min="265" max="512" width="9" style="1" customWidth="1"/>
+    <col min="513" max="513" width="9.33203125" style="1" customWidth="1"/>
+    <col min="514" max="514" width="6.33203125" style="1" customWidth="1"/>
+    <col min="515" max="515" width="47" style="1" customWidth="1"/>
+    <col min="516" max="516" width="43.33203125" style="1" customWidth="1"/>
+    <col min="517" max="517" width="13.33203125" style="1" customWidth="1"/>
+    <col min="518" max="518" width="10.6640625" style="1" customWidth="1"/>
+    <col min="519" max="519" width="12.44140625" style="1" customWidth="1"/>
+    <col min="520" max="520" width="12.109375" style="1" customWidth="1"/>
+    <col min="521" max="768" width="9" style="1" customWidth="1"/>
+    <col min="769" max="769" width="9.33203125" style="1" customWidth="1"/>
+    <col min="770" max="770" width="6.33203125" style="1" customWidth="1"/>
+    <col min="771" max="771" width="47" style="1" customWidth="1"/>
+    <col min="772" max="772" width="43.33203125" style="1" customWidth="1"/>
+    <col min="773" max="773" width="13.33203125" style="1" customWidth="1"/>
+    <col min="774" max="774" width="10.6640625" style="1" customWidth="1"/>
+    <col min="775" max="775" width="12.44140625" style="1" customWidth="1"/>
+    <col min="776" max="776" width="12.109375" style="1" customWidth="1"/>
+    <col min="777" max="1024" width="9" style="1" customWidth="1"/>
+    <col min="1025" max="1025" width="9.33203125" style="1" customWidth="1"/>
+    <col min="1026" max="1026" width="6.33203125" style="1" customWidth="1"/>
+    <col min="1027" max="1027" width="47" style="1" customWidth="1"/>
+    <col min="1028" max="1028" width="43.33203125" style="1" customWidth="1"/>
+    <col min="1029" max="1029" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1030" max="1030" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1031" max="1031" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1032" max="1032" width="12.109375" style="1" customWidth="1"/>
+    <col min="1033" max="1280" width="9" style="1" customWidth="1"/>
+    <col min="1281" max="1281" width="9.33203125" style="1" customWidth="1"/>
+    <col min="1282" max="1282" width="6.33203125" style="1" customWidth="1"/>
+    <col min="1283" max="1283" width="47" style="1" customWidth="1"/>
+    <col min="1284" max="1284" width="43.33203125" style="1" customWidth="1"/>
+    <col min="1285" max="1285" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1286" max="1286" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1287" max="1287" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1288" max="1288" width="12.109375" style="1" customWidth="1"/>
+    <col min="1289" max="1536" width="9" style="1" customWidth="1"/>
+    <col min="1537" max="1537" width="9.33203125" style="1" customWidth="1"/>
+    <col min="1538" max="1538" width="6.33203125" style="1" customWidth="1"/>
+    <col min="1539" max="1539" width="47" style="1" customWidth="1"/>
+    <col min="1540" max="1540" width="43.33203125" style="1" customWidth="1"/>
+    <col min="1541" max="1541" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1542" max="1542" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1543" max="1543" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1544" max="1544" width="12.109375" style="1" customWidth="1"/>
+    <col min="1545" max="1792" width="9" style="1" customWidth="1"/>
+    <col min="1793" max="1793" width="9.33203125" style="1" customWidth="1"/>
+    <col min="1794" max="1794" width="6.33203125" style="1" customWidth="1"/>
+    <col min="1795" max="1795" width="47" style="1" customWidth="1"/>
+    <col min="1796" max="1796" width="43.33203125" style="1" customWidth="1"/>
+    <col min="1797" max="1797" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1798" max="1798" width="10.6640625" style="1" customWidth="1"/>
+    <col min="1799" max="1799" width="12.44140625" style="1" customWidth="1"/>
+    <col min="1800" max="1800" width="12.109375" style="1" customWidth="1"/>
+    <col min="1801" max="2048" width="9" style="1" customWidth="1"/>
+    <col min="2049" max="2049" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2050" max="2050" width="6.33203125" style="1" customWidth="1"/>
+    <col min="2051" max="2051" width="47" style="1" customWidth="1"/>
+    <col min="2052" max="2052" width="43.33203125" style="1" customWidth="1"/>
+    <col min="2053" max="2053" width="13.33203125" style="1" customWidth="1"/>
+    <col min="2054" max="2054" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2055" max="2055" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2056" max="2056" width="12.109375" style="1" customWidth="1"/>
+    <col min="2057" max="2304" width="9" style="1" customWidth="1"/>
+    <col min="2305" max="2305" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2306" max="2306" width="6.33203125" style="1" customWidth="1"/>
+    <col min="2307" max="2307" width="47" style="1" customWidth="1"/>
+    <col min="2308" max="2308" width="43.33203125" style="1" customWidth="1"/>
+    <col min="2309" max="2309" width="13.33203125" style="1" customWidth="1"/>
+    <col min="2310" max="2310" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2311" max="2311" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2312" max="2312" width="12.109375" style="1" customWidth="1"/>
+    <col min="2313" max="2560" width="9" style="1" customWidth="1"/>
+    <col min="2561" max="2561" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2562" max="2562" width="6.33203125" style="1" customWidth="1"/>
+    <col min="2563" max="2563" width="47" style="1" customWidth="1"/>
+    <col min="2564" max="2564" width="43.33203125" style="1" customWidth="1"/>
+    <col min="2565" max="2565" width="13.33203125" style="1" customWidth="1"/>
+    <col min="2566" max="2566" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2567" max="2567" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2568" max="2568" width="12.109375" style="1" customWidth="1"/>
+    <col min="2569" max="2816" width="9" style="1" customWidth="1"/>
+    <col min="2817" max="2817" width="9.33203125" style="1" customWidth="1"/>
+    <col min="2818" max="2818" width="6.33203125" style="1" customWidth="1"/>
+    <col min="2819" max="2819" width="47" style="1" customWidth="1"/>
+    <col min="2820" max="2820" width="43.33203125" style="1" customWidth="1"/>
+    <col min="2821" max="2821" width="13.33203125" style="1" customWidth="1"/>
+    <col min="2822" max="2822" width="10.6640625" style="1" customWidth="1"/>
+    <col min="2823" max="2823" width="12.44140625" style="1" customWidth="1"/>
+    <col min="2824" max="2824" width="12.109375" style="1" customWidth="1"/>
+    <col min="2825" max="3072" width="9" style="1" customWidth="1"/>
+    <col min="3073" max="3073" width="9.33203125" style="1" customWidth="1"/>
+    <col min="3074" max="3074" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3075" max="3075" width="47" style="1" customWidth="1"/>
+    <col min="3076" max="3076" width="43.33203125" style="1" customWidth="1"/>
+    <col min="3077" max="3077" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3078" max="3078" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3079" max="3079" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3080" max="3080" width="12.109375" style="1" customWidth="1"/>
+    <col min="3081" max="3328" width="9" style="1" customWidth="1"/>
+    <col min="3329" max="3329" width="9.33203125" style="1" customWidth="1"/>
+    <col min="3330" max="3330" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3331" max="3331" width="47" style="1" customWidth="1"/>
+    <col min="3332" max="3332" width="43.33203125" style="1" customWidth="1"/>
+    <col min="3333" max="3333" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3334" max="3334" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3335" max="3335" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3336" max="3336" width="12.109375" style="1" customWidth="1"/>
+    <col min="3337" max="3584" width="9" style="1" customWidth="1"/>
+    <col min="3585" max="3585" width="9.33203125" style="1" customWidth="1"/>
+    <col min="3586" max="3586" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3587" max="3587" width="47" style="1" customWidth="1"/>
+    <col min="3588" max="3588" width="43.33203125" style="1" customWidth="1"/>
+    <col min="3589" max="3589" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3590" max="3590" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3591" max="3591" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3592" max="3592" width="12.109375" style="1" customWidth="1"/>
+    <col min="3593" max="3840" width="9" style="1" customWidth="1"/>
+    <col min="3841" max="3841" width="9.33203125" style="1" customWidth="1"/>
+    <col min="3842" max="3842" width="6.33203125" style="1" customWidth="1"/>
+    <col min="3843" max="3843" width="47" style="1" customWidth="1"/>
+    <col min="3844" max="3844" width="43.33203125" style="1" customWidth="1"/>
+    <col min="3845" max="3845" width="13.33203125" style="1" customWidth="1"/>
+    <col min="3846" max="3846" width="10.6640625" style="1" customWidth="1"/>
+    <col min="3847" max="3847" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3848" max="3848" width="12.109375" style="1" customWidth="1"/>
+    <col min="3849" max="4096" width="9" style="1" customWidth="1"/>
+    <col min="4097" max="4097" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4098" max="4098" width="6.33203125" style="1" customWidth="1"/>
+    <col min="4099" max="4099" width="47" style="1" customWidth="1"/>
+    <col min="4100" max="4100" width="43.33203125" style="1" customWidth="1"/>
+    <col min="4101" max="4101" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4102" max="4102" width="10.6640625" style="1" customWidth="1"/>
+    <col min="4103" max="4103" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4104" max="4104" width="12.109375" style="1" customWidth="1"/>
+    <col min="4105" max="4352" width="9" style="1" customWidth="1"/>
+    <col min="4353" max="4353" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4354" max="4354" width="6.33203125" style="1" customWidth="1"/>
+    <col min="4355" max="4355" width="47" style="1" customWidth="1"/>
+    <col min="4356" max="4356" width="43.33203125" style="1" customWidth="1"/>
+    <col min="4357" max="4357" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4358" max="4358" width="10.6640625" style="1" customWidth="1"/>
+    <col min="4359" max="4359" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4360" max="4360" width="12.109375" style="1" customWidth="1"/>
+    <col min="4361" max="4608" width="9" style="1" customWidth="1"/>
+    <col min="4609" max="4609" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4610" max="4610" width="6.33203125" style="1" customWidth="1"/>
+    <col min="4611" max="4611" width="47" style="1" customWidth="1"/>
+    <col min="4612" max="4612" width="43.33203125" style="1" customWidth="1"/>
+    <col min="4613" max="4613" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4614" max="4614" width="10.6640625" style="1" customWidth="1"/>
+    <col min="4615" max="4615" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4616" max="4616" width="12.109375" style="1" customWidth="1"/>
+    <col min="4617" max="4864" width="9" style="1" customWidth="1"/>
+    <col min="4865" max="4865" width="9.33203125" style="1" customWidth="1"/>
+    <col min="4866" max="4866" width="6.33203125" style="1" customWidth="1"/>
+    <col min="4867" max="4867" width="47" style="1" customWidth="1"/>
+    <col min="4868" max="4868" width="43.33203125" style="1" customWidth="1"/>
+    <col min="4869" max="4869" width="13.33203125" style="1" customWidth="1"/>
+    <col min="4870" max="4870" width="10.6640625" style="1" customWidth="1"/>
+    <col min="4871" max="4871" width="12.44140625" style="1" customWidth="1"/>
+    <col min="4872" max="4872" width="12.109375" style="1" customWidth="1"/>
+    <col min="4873" max="5120" width="9" style="1" customWidth="1"/>
+    <col min="5121" max="5121" width="9.33203125" style="1" customWidth="1"/>
+    <col min="5122" max="5122" width="6.33203125" style="1" customWidth="1"/>
+    <col min="5123" max="5123" width="47" style="1" customWidth="1"/>
+    <col min="5124" max="5124" width="43.33203125" style="1" customWidth="1"/>
+    <col min="5125" max="5125" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5126" max="5126" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5127" max="5127" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5128" max="5128" width="12.109375" style="1" customWidth="1"/>
+    <col min="5129" max="5376" width="9" style="1" customWidth="1"/>
+    <col min="5377" max="5377" width="9.33203125" style="1" customWidth="1"/>
+    <col min="5378" max="5378" width="6.33203125" style="1" customWidth="1"/>
+    <col min="5379" max="5379" width="47" style="1" customWidth="1"/>
+    <col min="5380" max="5380" width="43.33203125" style="1" customWidth="1"/>
+    <col min="5381" max="5381" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5382" max="5382" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5383" max="5383" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5384" max="5384" width="12.109375" style="1" customWidth="1"/>
+    <col min="5385" max="5632" width="9" style="1" customWidth="1"/>
+    <col min="5633" max="5633" width="9.33203125" style="1" customWidth="1"/>
+    <col min="5634" max="5634" width="6.33203125" style="1" customWidth="1"/>
+    <col min="5635" max="5635" width="47" style="1" customWidth="1"/>
+    <col min="5636" max="5636" width="43.33203125" style="1" customWidth="1"/>
+    <col min="5637" max="5637" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5638" max="5638" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5639" max="5639" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5640" max="5640" width="12.109375" style="1" customWidth="1"/>
+    <col min="5641" max="5888" width="9" style="1" customWidth="1"/>
+    <col min="5889" max="5889" width="9.33203125" style="1" customWidth="1"/>
+    <col min="5890" max="5890" width="6.33203125" style="1" customWidth="1"/>
+    <col min="5891" max="5891" width="47" style="1" customWidth="1"/>
+    <col min="5892" max="5892" width="43.33203125" style="1" customWidth="1"/>
+    <col min="5893" max="5893" width="13.33203125" style="1" customWidth="1"/>
+    <col min="5894" max="5894" width="10.6640625" style="1" customWidth="1"/>
+    <col min="5895" max="5895" width="12.44140625" style="1" customWidth="1"/>
+    <col min="5896" max="5896" width="12.109375" style="1" customWidth="1"/>
+    <col min="5897" max="6144" width="9" style="1" customWidth="1"/>
+    <col min="6145" max="6145" width="9.33203125" style="1" customWidth="1"/>
+    <col min="6146" max="6146" width="6.33203125" style="1" customWidth="1"/>
+    <col min="6147" max="6147" width="47" style="1" customWidth="1"/>
+    <col min="6148" max="6148" width="43.33203125" style="1" customWidth="1"/>
+    <col min="6149" max="6149" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6150" max="6150" width="10.6640625" style="1" customWidth="1"/>
+    <col min="6151" max="6151" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6152" max="6152" width="12.109375" style="1" customWidth="1"/>
+    <col min="6153" max="6400" width="9" style="1" customWidth="1"/>
+    <col min="6401" max="6401" width="9.33203125" style="1" customWidth="1"/>
+    <col min="6402" max="6402" width="6.33203125" style="1" customWidth="1"/>
+    <col min="6403" max="6403" width="47" style="1" customWidth="1"/>
+    <col min="6404" max="6404" width="43.33203125" style="1" customWidth="1"/>
+    <col min="6405" max="6405" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6406" max="6406" width="10.6640625" style="1" customWidth="1"/>
+    <col min="6407" max="6407" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6408" max="6408" width="12.109375" style="1" customWidth="1"/>
+    <col min="6409" max="6656" width="9" style="1" customWidth="1"/>
+    <col min="6657" max="6657" width="9.33203125" style="1" customWidth="1"/>
+    <col min="6658" max="6658" width="6.33203125" style="1" customWidth="1"/>
+    <col min="6659" max="6659" width="47" style="1" customWidth="1"/>
+    <col min="6660" max="6660" width="43.33203125" style="1" customWidth="1"/>
+    <col min="6661" max="6661" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6662" max="6662" width="10.6640625" style="1" customWidth="1"/>
+    <col min="6663" max="6663" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6664" max="6664" width="12.109375" style="1" customWidth="1"/>
+    <col min="6665" max="6912" width="9" style="1" customWidth="1"/>
+    <col min="6913" max="6913" width="9.33203125" style="1" customWidth="1"/>
+    <col min="6914" max="6914" width="6.33203125" style="1" customWidth="1"/>
+    <col min="6915" max="6915" width="47" style="1" customWidth="1"/>
+    <col min="6916" max="6916" width="43.33203125" style="1" customWidth="1"/>
+    <col min="6917" max="6917" width="13.33203125" style="1" customWidth="1"/>
+    <col min="6918" max="6918" width="10.6640625" style="1" customWidth="1"/>
+    <col min="6919" max="6919" width="12.44140625" style="1" customWidth="1"/>
+    <col min="6920" max="6920" width="12.109375" style="1" customWidth="1"/>
+    <col min="6921" max="7168" width="9" style="1" customWidth="1"/>
+    <col min="7169" max="7169" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7170" max="7170" width="6.33203125" style="1" customWidth="1"/>
+    <col min="7171" max="7171" width="47" style="1" customWidth="1"/>
+    <col min="7172" max="7172" width="43.33203125" style="1" customWidth="1"/>
+    <col min="7173" max="7173" width="13.33203125" style="1" customWidth="1"/>
+    <col min="7174" max="7174" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7175" max="7175" width="12.44140625" style="1" customWidth="1"/>
+    <col min="7176" max="7176" width="12.109375" style="1" customWidth="1"/>
+    <col min="7177" max="7424" width="9" style="1" customWidth="1"/>
+    <col min="7425" max="7425" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7426" max="7426" width="6.33203125" style="1" customWidth="1"/>
+    <col min="7427" max="7427" width="47" style="1" customWidth="1"/>
+    <col min="7428" max="7428" width="43.33203125" style="1" customWidth="1"/>
+    <col min="7429" max="7429" width="13.33203125" style="1" customWidth="1"/>
+    <col min="7430" max="7430" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7431" max="7431" width="12.44140625" style="1" customWidth="1"/>
+    <col min="7432" max="7432" width="12.109375" style="1" customWidth="1"/>
+    <col min="7433" max="7680" width="9" style="1" customWidth="1"/>
+    <col min="7681" max="7681" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7682" max="7682" width="6.33203125" style="1" customWidth="1"/>
+    <col min="7683" max="7683" width="47" style="1" customWidth="1"/>
+    <col min="7684" max="7684" width="43.33203125" style="1" customWidth="1"/>
+    <col min="7685" max="7685" width="13.33203125" style="1" customWidth="1"/>
+    <col min="7686" max="7686" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7687" max="7687" width="12.44140625" style="1" customWidth="1"/>
+    <col min="7688" max="7688" width="12.109375" style="1" customWidth="1"/>
+    <col min="7689" max="7936" width="9" style="1" customWidth="1"/>
+    <col min="7937" max="7937" width="9.33203125" style="1" customWidth="1"/>
+    <col min="7938" max="7938" width="6.33203125" style="1" customWidth="1"/>
+    <col min="7939" max="7939" width="47" style="1" customWidth="1"/>
+    <col min="7940" max="7940" width="43.33203125" style="1" customWidth="1"/>
+    <col min="7941" max="7941" width="13.33203125" style="1" customWidth="1"/>
+    <col min="7942" max="7942" width="10.6640625" style="1" customWidth="1"/>
+    <col min="7943" max="7943" width="12.44140625" style="1" customWidth="1"/>
+    <col min="7944" max="7944" width="12.109375" style="1" customWidth="1"/>
+    <col min="7945" max="8192" width="9" style="1" customWidth="1"/>
+    <col min="8193" max="8193" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8194" max="8194" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8195" max="8195" width="47" style="1" customWidth="1"/>
+    <col min="8196" max="8196" width="43.33203125" style="1" customWidth="1"/>
+    <col min="8197" max="8197" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8198" max="8198" width="10.6640625" style="1" customWidth="1"/>
+    <col min="8199" max="8199" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8200" max="8200" width="12.109375" style="1" customWidth="1"/>
+    <col min="8201" max="8448" width="9" style="1" customWidth="1"/>
+    <col min="8449" max="8449" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8450" max="8450" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8451" max="8451" width="47" style="1" customWidth="1"/>
+    <col min="8452" max="8452" width="43.33203125" style="1" customWidth="1"/>
+    <col min="8453" max="8453" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8454" max="8454" width="10.6640625" style="1" customWidth="1"/>
+    <col min="8455" max="8455" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8456" max="8456" width="12.109375" style="1" customWidth="1"/>
+    <col min="8457" max="8704" width="9" style="1" customWidth="1"/>
+    <col min="8705" max="8705" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8706" max="8706" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8707" max="8707" width="47" style="1" customWidth="1"/>
+    <col min="8708" max="8708" width="43.33203125" style="1" customWidth="1"/>
+    <col min="8709" max="8709" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8710" max="8710" width="10.6640625" style="1" customWidth="1"/>
+    <col min="8711" max="8711" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8712" max="8712" width="12.109375" style="1" customWidth="1"/>
+    <col min="8713" max="8960" width="9" style="1" customWidth="1"/>
+    <col min="8961" max="8961" width="9.33203125" style="1" customWidth="1"/>
+    <col min="8962" max="8962" width="6.33203125" style="1" customWidth="1"/>
+    <col min="8963" max="8963" width="47" style="1" customWidth="1"/>
+    <col min="8964" max="8964" width="43.33203125" style="1" customWidth="1"/>
+    <col min="8965" max="8965" width="13.33203125" style="1" customWidth="1"/>
+    <col min="8966" max="8966" width="10.6640625" style="1" customWidth="1"/>
+    <col min="8967" max="8967" width="12.44140625" style="1" customWidth="1"/>
+    <col min="8968" max="8968" width="12.109375" style="1" customWidth="1"/>
+    <col min="8969" max="9216" width="9" style="1" customWidth="1"/>
+    <col min="9217" max="9217" width="9.33203125" style="1" customWidth="1"/>
+    <col min="9218" max="9218" width="6.33203125" style="1" customWidth="1"/>
+    <col min="9219" max="9219" width="47" style="1" customWidth="1"/>
+    <col min="9220" max="9220" width="43.33203125" style="1" customWidth="1"/>
+    <col min="9221" max="9221" width="13.33203125" style="1" customWidth="1"/>
+    <col min="9222" max="9222" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9223" max="9223" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9224" max="9224" width="12.109375" style="1" customWidth="1"/>
+    <col min="9225" max="9472" width="9" style="1" customWidth="1"/>
+    <col min="9473" max="9473" width="9.33203125" style="1" customWidth="1"/>
+    <col min="9474" max="9474" width="6.33203125" style="1" customWidth="1"/>
+    <col min="9475" max="9475" width="47" style="1" customWidth="1"/>
+    <col min="9476" max="9476" width="43.33203125" style="1" customWidth="1"/>
+    <col min="9477" max="9477" width="13.33203125" style="1" customWidth="1"/>
+    <col min="9478" max="9478" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9479" max="9479" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9480" max="9480" width="12.109375" style="1" customWidth="1"/>
+    <col min="9481" max="9728" width="9" style="1" customWidth="1"/>
+    <col min="9729" max="9729" width="9.33203125" style="1" customWidth="1"/>
+    <col min="9730" max="9730" width="6.33203125" style="1" customWidth="1"/>
+    <col min="9731" max="9731" width="47" style="1" customWidth="1"/>
+    <col min="9732" max="9732" width="43.33203125" style="1" customWidth="1"/>
+    <col min="9733" max="9733" width="13.33203125" style="1" customWidth="1"/>
+    <col min="9734" max="9734" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9735" max="9735" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9736" max="9736" width="12.109375" style="1" customWidth="1"/>
+    <col min="9737" max="9984" width="9" style="1" customWidth="1"/>
+    <col min="9985" max="9985" width="9.33203125" style="1" customWidth="1"/>
+    <col min="9986" max="9986" width="6.33203125" style="1" customWidth="1"/>
+    <col min="9987" max="9987" width="47" style="1" customWidth="1"/>
+    <col min="9988" max="9988" width="43.33203125" style="1" customWidth="1"/>
+    <col min="9989" max="9989" width="13.33203125" style="1" customWidth="1"/>
+    <col min="9990" max="9990" width="10.6640625" style="1" customWidth="1"/>
+    <col min="9991" max="9991" width="12.44140625" style="1" customWidth="1"/>
+    <col min="9992" max="9992" width="12.109375" style="1" customWidth="1"/>
+    <col min="9993" max="10240" width="9" style="1" customWidth="1"/>
+    <col min="10241" max="10241" width="9.33203125" style="1" customWidth="1"/>
+    <col min="10242" max="10242" width="6.33203125" style="1" customWidth="1"/>
+    <col min="10243" max="10243" width="47" style="1" customWidth="1"/>
+    <col min="10244" max="10244" width="43.33203125" style="1" customWidth="1"/>
+    <col min="10245" max="10245" width="13.33203125" style="1" customWidth="1"/>
+    <col min="10246" max="10246" width="10.6640625" style="1" customWidth="1"/>
+    <col min="10247" max="10247" width="12.44140625" style="1" customWidth="1"/>
+    <col min="10248" max="10248" width="12.109375" style="1" customWidth="1"/>
+    <col min="10249" max="10496" width="9" style="1" customWidth="1"/>
+    <col min="10497" max="10497" width="9.33203125" style="1" customWidth="1"/>
+    <col min="10498" max="10498" width="6.33203125" style="1" customWidth="1"/>
+    <col min="10499" max="10499" width="47" style="1" customWidth="1"/>
+    <col min="10500" max="10500" width="43.33203125" style="1" customWidth="1"/>
+    <col min="10501" max="10501" width="13.33203125" style="1" customWidth="1"/>
+    <col min="10502" max="10502" width="10.6640625" style="1" customWidth="1"/>
+    <col min="10503" max="10503" width="12.44140625" style="1" customWidth="1"/>
+    <col min="10504" max="10504" width="12.109375" style="1" customWidth="1"/>
+    <col min="10505" max="10752" width="9" style="1" customWidth="1"/>
+    <col min="10753" max="10753" width="9.33203125" style="1" customWidth="1"/>
+    <col min="10754" max="10754" width="6.33203125" style="1" customWidth="1"/>
+    <col min="10755" max="10755" width="47" style="1" customWidth="1"/>
+    <col min="10756" max="10756" width="43.33203125" style="1" customWidth="1"/>
+    <col min="10757" max="10757" width="13.33203125" style="1" customWidth="1"/>
+    <col min="10758" max="10758" width="10.6640625" style="1" customWidth="1"/>
+    <col min="10759" max="10759" width="12.44140625" style="1" customWidth="1"/>
+    <col min="10760" max="10760" width="12.109375" style="1" customWidth="1"/>
+    <col min="10761" max="11008" width="9" style="1" customWidth="1"/>
+    <col min="11009" max="11009" width="9.33203125" style="1" customWidth="1"/>
+    <col min="11010" max="11010" width="6.33203125" style="1" customWidth="1"/>
+    <col min="11011" max="11011" width="47" style="1" customWidth="1"/>
+    <col min="11012" max="11012" width="43.33203125" style="1" customWidth="1"/>
+    <col min="11013" max="11013" width="13.33203125" style="1" customWidth="1"/>
+    <col min="11014" max="11014" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11015" max="11015" width="12.44140625" style="1" customWidth="1"/>
+    <col min="11016" max="11016" width="12.109375" style="1" customWidth="1"/>
+    <col min="11017" max="11264" width="9" style="1" customWidth="1"/>
+    <col min="11265" max="11265" width="9.33203125" style="1" customWidth="1"/>
+    <col min="11266" max="11266" width="6.33203125" style="1" customWidth="1"/>
+    <col min="11267" max="11267" width="47" style="1" customWidth="1"/>
+    <col min="11268" max="11268" width="43.33203125" style="1" customWidth="1"/>
+    <col min="11269" max="11269" width="13.33203125" style="1" customWidth="1"/>
+    <col min="11270" max="11270" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11271" max="11271" width="12.44140625" style="1" customWidth="1"/>
+    <col min="11272" max="11272" width="12.109375" style="1" customWidth="1"/>
+    <col min="11273" max="11520" width="9" style="1" customWidth="1"/>
+    <col min="11521" max="11521" width="9.33203125" style="1" customWidth="1"/>
+    <col min="11522" max="11522" width="6.33203125" style="1" customWidth="1"/>
+    <col min="11523" max="11523" width="47" style="1" customWidth="1"/>
+    <col min="11524" max="11524" width="43.33203125" style="1" customWidth="1"/>
+    <col min="11525" max="11525" width="13.33203125" style="1" customWidth="1"/>
+    <col min="11526" max="11526" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11527" max="11527" width="12.44140625" style="1" customWidth="1"/>
+    <col min="11528" max="11528" width="12.109375" style="1" customWidth="1"/>
+    <col min="11529" max="11776" width="9" style="1" customWidth="1"/>
+    <col min="11777" max="11777" width="9.33203125" style="1" customWidth="1"/>
+    <col min="11778" max="11778" width="6.33203125" style="1" customWidth="1"/>
+    <col min="11779" max="11779" width="47" style="1" customWidth="1"/>
+    <col min="11780" max="11780" width="43.33203125" style="1" customWidth="1"/>
+    <col min="11781" max="11781" width="13.33203125" style="1" customWidth="1"/>
+    <col min="11782" max="11782" width="10.6640625" style="1" customWidth="1"/>
+    <col min="11783" max="11783" width="12.44140625" style="1" customWidth="1"/>
+    <col min="11784" max="11784" width="12.109375" style="1" customWidth="1"/>
+    <col min="11785" max="12032" width="9" style="1" customWidth="1"/>
+    <col min="12033" max="12033" width="9.33203125" style="1" customWidth="1"/>
+    <col min="12034" max="12034" width="6.33203125" style="1" customWidth="1"/>
+    <col min="12035" max="12035" width="47" style="1" customWidth="1"/>
+    <col min="12036" max="12036" width="43.33203125" style="1" customWidth="1"/>
+    <col min="12037" max="12037" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12038" max="12038" width="10.6640625" style="1" customWidth="1"/>
+    <col min="12039" max="12039" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12040" max="12040" width="12.109375" style="1" customWidth="1"/>
+    <col min="12041" max="12288" width="9" style="1" customWidth="1"/>
+    <col min="12289" max="12289" width="9.33203125" style="1" customWidth="1"/>
+    <col min="12290" max="12290" width="6.33203125" style="1" customWidth="1"/>
+    <col min="12291" max="12291" width="47" style="1" customWidth="1"/>
+    <col min="12292" max="12292" width="43.33203125" style="1" customWidth="1"/>
+    <col min="12293" max="12293" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12294" max="12294" width="10.6640625" style="1" customWidth="1"/>
+    <col min="12295" max="12295" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12296" max="12296" width="12.109375" style="1" customWidth="1"/>
+    <col min="12297" max="12544" width="9" style="1" customWidth="1"/>
+    <col min="12545" max="12545" width="9.33203125" style="1" customWidth="1"/>
+    <col min="12546" max="12546" width="6.33203125" style="1" customWidth="1"/>
+    <col min="12547" max="12547" width="47" style="1" customWidth="1"/>
+    <col min="12548" max="12548" width="43.33203125" style="1" customWidth="1"/>
+    <col min="12549" max="12549" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12550" max="12550" width="10.6640625" style="1" customWidth="1"/>
+    <col min="12551" max="12551" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12552" max="12552" width="12.109375" style="1" customWidth="1"/>
+    <col min="12553" max="12800" width="9" style="1" customWidth="1"/>
+    <col min="12801" max="12801" width="9.33203125" style="1" customWidth="1"/>
+    <col min="12802" max="12802" width="6.33203125" style="1" customWidth="1"/>
+    <col min="12803" max="12803" width="47" style="1" customWidth="1"/>
+    <col min="12804" max="12804" width="43.33203125" style="1" customWidth="1"/>
+    <col min="12805" max="12805" width="13.33203125" style="1" customWidth="1"/>
+    <col min="12806" max="12806" width="10.6640625" style="1" customWidth="1"/>
+    <col min="12807" max="12807" width="12.44140625" style="1" customWidth="1"/>
+    <col min="12808" max="12808" width="12.109375" style="1" customWidth="1"/>
+    <col min="12809" max="13056" width="9" style="1" customWidth="1"/>
+    <col min="13057" max="13057" width="9.33203125" style="1" customWidth="1"/>
+    <col min="13058" max="13058" width="6.33203125" style="1" customWidth="1"/>
+    <col min="13059" max="13059" width="47" style="1" customWidth="1"/>
+    <col min="13060" max="13060" width="43.33203125" style="1" customWidth="1"/>
+    <col min="13061" max="13061" width="13.33203125" style="1" customWidth="1"/>
+    <col min="13062" max="13062" width="10.6640625" style="1" customWidth="1"/>
+    <col min="13063" max="13063" width="12.44140625" style="1" customWidth="1"/>
+    <col min="13064" max="13064" width="12.109375" style="1" customWidth="1"/>
+    <col min="13065" max="13312" width="9" style="1" customWidth="1"/>
+    <col min="13313" max="13313" width="9.33203125" style="1" customWidth="1"/>
+    <col min="13314" max="13314" width="6.33203125" style="1" customWidth="1"/>
+    <col min="13315" max="13315" width="47" style="1" customWidth="1"/>
+    <col min="13316" max="13316" width="43.33203125" style="1" customWidth="1"/>
+    <col min="13317" max="13317" width="13.33203125" style="1" customWidth="1"/>
+    <col min="13318" max="13318" width="10.6640625" style="1" customWidth="1"/>
+    <col min="13319" max="13319" width="12.44140625" style="1" customWidth="1"/>
+    <col min="13320" max="13320" width="12.109375" style="1" customWidth="1"/>
+    <col min="13321" max="13568" width="9" style="1" customWidth="1"/>
+    <col min="13569" max="13569" width="9.33203125" style="1" customWidth="1"/>
+    <col min="13570" max="13570" width="6.33203125" style="1" customWidth="1"/>
+    <col min="13571" max="13571" width="47" style="1" customWidth="1"/>
+    <col min="13572" max="13572" width="43.33203125" style="1" customWidth="1"/>
+    <col min="13573" max="13573" width="13.33203125" style="1" customWidth="1"/>
+    <col min="13574" max="13574" width="10.6640625" style="1" customWidth="1"/>
+    <col min="13575" max="13575" width="12.44140625" style="1" customWidth="1"/>
+    <col min="13576" max="13576" width="12.109375" style="1" customWidth="1"/>
+    <col min="13577" max="13824" width="9" style="1" customWidth="1"/>
+    <col min="13825" max="13825" width="9.33203125" style="1" customWidth="1"/>
+    <col min="13826" max="13826" width="6.33203125" style="1" customWidth="1"/>
+    <col min="13827" max="13827" width="47" style="1" customWidth="1"/>
+    <col min="13828" max="13828" width="43.33203125" style="1" customWidth="1"/>
+    <col min="13829" max="13829" width="13.33203125" style="1" customWidth="1"/>
+    <col min="13830" max="13830" width="10.6640625" style="1" customWidth="1"/>
+    <col min="13831" max="13831" width="12.44140625" style="1" customWidth="1"/>
+    <col min="13832" max="13832" width="12.109375" style="1" customWidth="1"/>
+    <col min="13833" max="14080" width="9" style="1" customWidth="1"/>
+    <col min="14081" max="14081" width="9.33203125" style="1" customWidth="1"/>
+    <col min="14082" max="14082" width="6.33203125" style="1" customWidth="1"/>
+    <col min="14083" max="14083" width="47" style="1" customWidth="1"/>
+    <col min="14084" max="14084" width="43.33203125" style="1" customWidth="1"/>
+    <col min="14085" max="14085" width="13.33203125" style="1" customWidth="1"/>
+    <col min="14086" max="14086" width="10.6640625" style="1" customWidth="1"/>
+    <col min="14087" max="14087" width="12.44140625" style="1" customWidth="1"/>
+    <col min="14088" max="14088" width="12.109375" style="1" customWidth="1"/>
+    <col min="14089" max="14336" width="9" style="1" customWidth="1"/>
+    <col min="14337" max="14337" width="9.33203125" style="1" customWidth="1"/>
+    <col min="14338" max="14338" width="6.33203125" style="1" customWidth="1"/>
+    <col min="14339" max="14339" width="47" style="1" customWidth="1"/>
+    <col min="14340" max="14340" width="43.33203125" style="1" customWidth="1"/>
+    <col min="14341" max="14341" width="13.33203125" style="1" customWidth="1"/>
+    <col min="14342" max="14342" width="10.6640625" style="1" customWidth="1"/>
+    <col min="14343" max="14343" width="12.44140625" style="1" customWidth="1"/>
+    <col min="14344" max="14344" width="12.109375" style="1" customWidth="1"/>
+    <col min="14345" max="14592" width="9" style="1" customWidth="1"/>
+    <col min="14593" max="14593" width="9.33203125" style="1" customWidth="1"/>
+    <col min="14594" max="14594" width="6.33203125" style="1" customWidth="1"/>
+    <col min="14595" max="14595" width="47" style="1" customWidth="1"/>
+    <col min="14596" max="14596" width="43.33203125" style="1" customWidth="1"/>
+    <col min="14597" max="14597" width="13.33203125" style="1" customWidth="1"/>
+    <col min="14598" max="14598" width="10.6640625" style="1" customWidth="1"/>
+    <col min="14599" max="14599" width="12.44140625" style="1" customWidth="1"/>
+    <col min="14600" max="14600" width="12.109375" style="1" customWidth="1"/>
+    <col min="14601" max="14848" width="9" style="1" customWidth="1"/>
+    <col min="14849" max="14849" width="9.33203125" style="1" customWidth="1"/>
+    <col min="14850" max="14850" width="6.33203125" style="1" customWidth="1"/>
+    <col min="14851" max="14851" width="47" style="1" customWidth="1"/>
+    <col min="14852" max="14852" width="43.33203125" style="1" customWidth="1"/>
+    <col min="14853" max="14853" width="13.33203125" style="1" customWidth="1"/>
+    <col min="14854" max="14854" width="10.6640625" style="1" customWidth="1"/>
+    <col min="14855" max="14855" width="12.44140625" style="1" customWidth="1"/>
+    <col min="14856" max="14856" width="12.109375" style="1" customWidth="1"/>
+    <col min="14857" max="15104" width="9" style="1" customWidth="1"/>
+    <col min="15105" max="15105" width="9.33203125" style="1" customWidth="1"/>
+    <col min="15106" max="15106" width="6.33203125" style="1" customWidth="1"/>
+    <col min="15107" max="15107" width="47" style="1" customWidth="1"/>
+    <col min="15108" max="15108" width="43.33203125" style="1" customWidth="1"/>
+    <col min="15109" max="15109" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15110" max="15110" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15111" max="15111" width="12.44140625" style="1" customWidth="1"/>
+    <col min="15112" max="15112" width="12.109375" style="1" customWidth="1"/>
+    <col min="15113" max="15360" width="9" style="1" customWidth="1"/>
+    <col min="15361" max="15361" width="9.33203125" style="1" customWidth="1"/>
+    <col min="15362" max="15362" width="6.33203125" style="1" customWidth="1"/>
+    <col min="15363" max="15363" width="47" style="1" customWidth="1"/>
+    <col min="15364" max="15364" width="43.33203125" style="1" customWidth="1"/>
+    <col min="15365" max="15365" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15366" max="15366" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15367" max="15367" width="12.44140625" style="1" customWidth="1"/>
+    <col min="15368" max="15368" width="12.109375" style="1" customWidth="1"/>
+    <col min="15369" max="15616" width="9" style="1" customWidth="1"/>
+    <col min="15617" max="15617" width="9.33203125" style="1" customWidth="1"/>
+    <col min="15618" max="15618" width="6.33203125" style="1" customWidth="1"/>
+    <col min="15619" max="15619" width="47" style="1" customWidth="1"/>
+    <col min="15620" max="15620" width="43.33203125" style="1" customWidth="1"/>
+    <col min="15621" max="15621" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15622" max="15622" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15623" max="15623" width="12.44140625" style="1" customWidth="1"/>
+    <col min="15624" max="15624" width="12.109375" style="1" customWidth="1"/>
+    <col min="15625" max="15872" width="9" style="1" customWidth="1"/>
+    <col min="15873" max="15873" width="9.33203125" style="1" customWidth="1"/>
+    <col min="15874" max="15874" width="6.33203125" style="1" customWidth="1"/>
+    <col min="15875" max="15875" width="47" style="1" customWidth="1"/>
+    <col min="15876" max="15876" width="43.33203125" style="1" customWidth="1"/>
+    <col min="15877" max="15877" width="13.33203125" style="1" customWidth="1"/>
+    <col min="15878" max="15878" width="10.6640625" style="1" customWidth="1"/>
+    <col min="15879" max="15879" width="12.44140625" style="1" customWidth="1"/>
+    <col min="15880" max="15880" width="12.109375" style="1" customWidth="1"/>
+    <col min="15881" max="16128" width="9" style="1" customWidth="1"/>
+    <col min="16129" max="16129" width="9.33203125" style="1" customWidth="1"/>
+    <col min="16130" max="16130" width="6.33203125" style="1" customWidth="1"/>
+    <col min="16131" max="16131" width="47" style="1" customWidth="1"/>
+    <col min="16132" max="16132" width="43.33203125" style="1" customWidth="1"/>
+    <col min="16133" max="16133" width="13.33203125" style="1" customWidth="1"/>
+    <col min="16134" max="16134" width="10.6640625" style="1" customWidth="1"/>
+    <col min="16135" max="16135" width="12.44140625" style="1" customWidth="1"/>
+    <col min="16136" max="16136" width="12.109375" style="1" customWidth="1"/>
+    <col min="16137" max="16384" width="9" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+    </row>
+    <row r="2" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" ht="8.1" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+    </row>
+    <row r="4" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" ht="20.25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="108" t="s">
+        <v>249</v>
+      </c>
+      <c r="B7" s="21"/>
+      <c r="C7" s="68"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="31"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="108" t="s">
+        <v>250</v>
+      </c>
+      <c r="B8" s="21"/>
+      <c r="C8" s="68"/>
+      <c r="D8" s="68"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="31"/>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="108" t="s">
+        <v>251</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="68" t="s">
+        <v>252</v>
+      </c>
+      <c r="D9" s="68" t="s">
+        <v>253</v>
+      </c>
+      <c r="E9" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="F9" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="G9" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="H9" s="31"/>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="108" t="s">
+        <v>254</v>
+      </c>
+      <c r="B10" s="21"/>
+      <c r="C10" s="68"/>
+      <c r="D10" s="68"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="31"/>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="108" t="s">
+        <v>255</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="68" t="s">
+        <v>252</v>
+      </c>
+      <c r="D11" s="68" t="s">
+        <v>253</v>
+      </c>
+      <c r="E11" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="H11" s="31" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="108" t="s">
+        <v>256</v>
+      </c>
+      <c r="B12" s="21"/>
+      <c r="C12" s="68"/>
+      <c r="D12" s="68"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="31"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="108" t="s">
+        <v>257</v>
+      </c>
+      <c r="B13" s="21"/>
+      <c r="C13" s="68"/>
+      <c r="D13" s="68"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.2362204724409449" right="0" top="0.2362204724409449" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
them ai moi, sua excel
</commit_message>
<xml_diff>
--- a/backend/public/lichmau.xlsx
+++ b/backend/public/lichmau.xlsx
@@ -11,27 +11,27 @@
     <sheet sheetId="2" name="05_01-11_01" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="12_01-18_01" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="19_01-25_01" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="26_01-01_02" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="02_02-08_02" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="09_02-15_02" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="23_02-01_03" state="visible" r:id="rId11"/>
+    <sheet sheetId="6" name="02_02-08_02" state="visible" r:id="rId8"/>
+    <sheet sheetId="7" name="09_02-15_02" state="visible" r:id="rId9"/>
+    <sheet sheetId="8" name="23_02-01_03" state="visible" r:id="rId10"/>
+    <sheet sheetId="5" name="26_01-01_02" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'29_12-04_01'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'05_01-11_01'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'12_01-18_01'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'19_01-25_01'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'26_01-01_02'!$7:$7</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'02_02-08_02'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'09_02-15_02'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'23_02-01_03'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'02_02-08_02'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'09_02-15_02'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'23_02-01_03'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'26_01-01_02'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="266">
   <si>
     <t>TRƯỜNG ĐẠI HỌC THÁI BÌNH</t>
   </si>
@@ -702,6 +702,126 @@
     <t>Nhà F</t>
   </si>
   <si>
+    <t>(Từ ngày 02/02/2026 đến ngày 08/02/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Hai
+ ngày 02/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba
+ ngày 03/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Tư
+ ngày 04/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Năm
+ ngày 05/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Sáu
+ ngày 06/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Bảy
+ ngày 07/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ Nhật
+ ngày 08/02</t>
+  </si>
+  <si>
+    <t>KIỂM TRA LỊCH BỔ SUNG (MÀU VÀNG), từ 16h00</t>
+  </si>
+  <si>
+    <t>A, B</t>
+  </si>
+  <si>
+    <t>Leader</t>
+  </si>
+  <si>
+    <t>Unit A</t>
+  </si>
+  <si>
+    <t>(Từ ngày 09/02/2026 đến ngày 15/02/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Hai
+ ngày 09/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba
+ ngày 10/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Tư
+ ngày 11/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Năm
+ ngày 12/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Sáu
+ ngày 13/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Bảy
+ ngày 14/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ Nhật
+ ngày 15/02</t>
+  </si>
+  <si>
+    <t>(Từ ngày 23/02/2026 đến ngày 01/03/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Hai
+ ngày 23/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba
+ ngày 24/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Tư
+ ngày 25/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Năm
+ ngày 26/02</t>
+  </si>
+  <si>
+    <t>Họp giao ban, từ 8h00</t>
+  </si>
+  <si>
+    <t>Các ban ngành trong trường đại học</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Phòng F2-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Hiệu trưởng</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Văn Phòng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Sáu
+ ngày 27/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Bảy
+ ngày 28/02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ Nhật
+ ngày 01/03</t>
+  </si>
+  <si>
     <t>(Từ ngày 26/01/2026 đến ngày 01/02/2026)</t>
   </si>
   <si>
@@ -709,34 +829,48 @@
  ngày 26/01</t>
   </si>
   <si>
-    <t>Dự họp Ban chấp hành Hội Cựu giáo chức Trường Đại học Thái Bình, từ 8h30</t>
+    <t>Dự họp Ban chấp hành Hội Cựu giáo chức Trường Đại học Thái Bình, từ 8h30, từ 8h30</t>
   </si>
   <si>
     <t>SN 38, Đốc Nhưỡng, P. Trần Hưng Đạo</t>
   </si>
   <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Họp Ban Thường vụ mở rộng, từ 14h00, từ 14h00</t>
+  </si>
+  <si>
     <t>Ban Thường vụ, Ban Giám hiệu, VP. Đảng ủy</t>
   </si>
   <si>
-    <t>Họp Ban Chấp hành Đảng bộ, từ 15h00</t>
-  </si>
-  <si>
-    <t>Thứ Ba ngày 27/01</t>
+    <t>Họp Ban Chấp hành Đảng bộ, từ 15h00, từ 15h00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba
+ ngày 27/01</t>
+  </si>
+  <si>
+    <t>Họp Ban Giám hiệu, từ 8h00, từ 8h00</t>
   </si>
   <si>
     <t>Ban Giám hiệu, Chánh Văn phòng, đ/c Bắc (TCCB, TT&amp;KĐCL), đ/c Lệ (ĐT&amp;HSSV), đ/c Hương KHCN&amp;HTPT), TKHT, TLHT</t>
   </si>
   <si>
-    <t>Gặp mặt giảng viên (Nam từ 46, Nữ từ 44 tuổi trở xuống tính từ năm 2026), từ 14h00</t>
-  </si>
-  <si>
-    <t>Ban Giám hiệu,  Bí thư Chi bộ, Trưởng các đơn vị và giảng viên (Nam từ 46, Nữ từ 44 tuổi trở xuống)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Tư ngày 28/01 </t>
-  </si>
-  <si>
-    <t>Dự Đại hội đại biểu Hội Cựu chiến binh Khối 487, lần thứ Nhất, nhiệm kỳ 20225-2030, từ 8h00</t>
+    <t>Gặp mặt giảng viên (Nam từ 46, Nữ từ 44 tuổi trở xuống tính từ năm 2026), từ 14h00, từ 14h00</t>
+  </si>
+  <si>
+    <t>Ban Giám hiệu, Bí thư Chi bộ, Trưởng các đơn vị và giảng viên (Nam từ 46, Nữ từ 44 tuổi trở xuống)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Tư
+ ngày 28/01</t>
+  </si>
+  <si>
+    <t>Dự Hội nghị thông báo nhanh kết quả Đại hội đại biểu toàn quốc lần thứ XIV của Đảng, từ 8h00, từ 8h00</t>
+  </si>
+  <si>
+    <t>Dự Đại hội đại biểu Hội Cựu chiến binh Khối 487, lần thứ Nhất, nhiệm kỳ 20225-2030, từ 8h00, từ 8h00</t>
   </si>
   <si>
     <t>PHT Hà Văn Đổng, đ/c Thiện + đ/c Hữu Thúy + đ/c Liên (Hội CCB)</t>
@@ -745,195 +879,71 @@
     <t>Trường Chính trị Nguyễn Văn Linh</t>
   </si>
   <si>
-    <t>Dự Hội nghị thông báo nhanh kết quả Đại hội đại biểu toàn quốc lần thứ XIV của Đảng, từ 8h00</t>
-  </si>
-  <si>
-    <t>Dự Hội nghị báo cáo viên tháng 01 năm 2026, từ 8h00</t>
+    <t>Dự Hội nghị báo cáo viên tháng 01 năm 2026, từ 8h00, từ 8h00</t>
   </si>
   <si>
     <t>Đảng ủy UBND tỉnh</t>
   </si>
   <si>
-    <t>Họp thường trực Hội đồng Khoa học và Đào tạo cấp trường, từ 13h30</t>
-  </si>
-  <si>
-    <t>Nghe các Nghiên cứu sinh báo cáo tiến độ kế hoạch làm nghiên cứu sinh, từ 15h30</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Ban Giám hiệu, Chánh Văn phòng, Trưởng phòng </t>
-    </r>
-    <r>
-      <rPr>
-        <family val="1"/>
-        <sz val="10"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t>TTCB, TT&amp;KĐCL</t>
-    </r>
-    <r>
-      <rPr>
-        <family val="1"/>
-        <sz val="11"/>
-        <rFont val="Times New Roman"/>
-      </rPr>
-      <t xml:space="preserve"> và các Nghiên cứu sinh</t>
-    </r>
+    <t>Họp thường trực Hội đồng Khoa học và Đào tạo cấp trường, từ 13h30, từ 13h30</t>
+  </si>
+  <si>
+    <t>Nghe các Nghiên cứu sinh báo cáo tiến độ kế hoạch làm nghiên cứu sinh, từ 15h30, từ 15h30</t>
+  </si>
+  <si>
+    <t>Ban Giám hiệu, Chánh Văn phòng, Trưởng phòng TTCB, TT&amp;KĐCL và các Nghiên cứu sinh</t>
   </si>
   <si>
     <t xml:space="preserve">Thứ Năm
-ngày 29/01</t>
-  </si>
-  <si>
-    <t>Nghe phổ biến Quy chế chi tiêu nội bộ năm 2026, Quy định về chế độ làm việc của giảng viên, từ 8h00</t>
+ ngày 29/01</t>
+  </si>
+  <si>
+    <t>Tiếp công dân, từ 8h00, từ 8h00</t>
+  </si>
+  <si>
+    <t>Nghe phổ biến Quy chế chi tiêu nội bộ năm 2026, Quy định về chế độ làm việc của giảng viên, từ 8h00, từ 8h00</t>
   </si>
   <si>
     <t>Toàn thể viên chức, người lao động Trường  Đại học Thái Bình</t>
   </si>
   <si>
-    <t>Họp Hội đồng xét nâng lương và phụ cấp thâm niên nhà giáo 6 tháng đầu năm 2026, từ 15h00</t>
-  </si>
-  <si>
-    <t>Gặp mặt cán bộ, viên chức nghỉ hưu năm 2025, từ 16h00</t>
+    <t>Họp giao ban Khối Hiệu bộ, từ 13h30, từ 13h30</t>
+  </si>
+  <si>
+    <t>Họp Hội đồng xét nâng lương và phụ cấp thâm niên nhà giáo 6 tháng đầu năm 2026, từ 15h00, từ 15h00</t>
+  </si>
+  <si>
+    <t>Gặp mặt cán bộ, viên chức nghỉ hưu năm 2025, từ 16h00, từ 16h00</t>
   </si>
   <si>
     <t>Ban Giám hiệu, Trưởng các đơn vị, Trưởng đoàn thể, cán bộ, viên chức nghỉ hưu năm 2025</t>
   </si>
   <si>
-    <t>Thứ Sáu ngày 30/01</t>
-  </si>
-  <si>
-    <t>Khám sức khỏe cho sinh viên đầu khóa nhập học năm 2025, thời gian: sáng từ 7h30; chiều từ 13h15</t>
+    <t xml:space="preserve">Thứ Sáu
+ ngày 30/01</t>
+  </si>
+  <si>
+    <t>Khám sức khỏe cho sinh viên đầu khóa nhập học năm 2025, thời gian: sáng từ 7h30; chiều từ 13h15, từ 7h30</t>
   </si>
   <si>
     <t>Theo kế hoạch số 117/KH-ĐHTB, ngày 19/01/2026</t>
   </si>
   <si>
-    <t>Họp Ban Thường vụ mở rộng, từ 9h00</t>
-  </si>
-  <si>
-    <t>Họp Ban Chấp hành Đảng bộ mở rộng, từ 14h00</t>
+    <t>Họp Ban Thường vụ mở rộng, từ 9h00, từ 9h00</t>
+  </si>
+  <si>
+    <t>Họp Ban Chấp hành Đảng bộ mở rộng, từ 14h00, từ 14h00</t>
   </si>
   <si>
     <t>BCH Đảng bộ, Bí thư các chi bộ, VP. Đảng ủy</t>
   </si>
   <si>
     <t xml:space="preserve">Thứ Bảy
-ngày 31/01</t>
-  </si>
-  <si>
-    <t>Chủ Nhật ngày 01/02</t>
-  </si>
-  <si>
-    <t>(Từ ngày 02/02/2026 đến ngày 08/02/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Hai
- ngày 02/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Ba
- ngày 03/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Tư
- ngày 04/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Năm
- ngày 05/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Sáu
- ngày 06/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Bảy
- ngày 07/02</t>
+ ngày 31/01</t>
   </si>
   <si>
     <t xml:space="preserve">Chủ Nhật
- ngày 08/02</t>
-  </si>
-  <si>
-    <t>KIỂM TRA LỊCH BỔ SUNG (MÀU VÀNG), từ 16h00</t>
-  </si>
-  <si>
-    <t>A, B</t>
-  </si>
-  <si>
-    <t>Leader</t>
-  </si>
-  <si>
-    <t>Unit A</t>
-  </si>
-  <si>
-    <t>(Từ ngày 09/02/2026 đến ngày 15/02/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Hai
- ngày 09/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Ba
- ngày 10/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Tư
- ngày 11/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Năm
- ngày 12/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Sáu
- ngày 13/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Bảy
- ngày 14/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chủ Nhật
- ngày 15/02</t>
-  </si>
-  <si>
-    <t>(Từ ngày 23/02/2026 đến ngày 01/03/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Hai
- ngày 23/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Ba
- ngày 24/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Tư
- ngày 25/02</t>
-  </si>
-  <si>
-    <t>1, từ 16h00</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Năm
- ngày 26/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Sáu
- ngày 27/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thứ Bảy
- ngày 28/02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chủ Nhật
- ngày 01/03</t>
+ ngày 01/02</t>
   </si>
 </sst>
 </file>
@@ -943,7 +953,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* (#,##0.00);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1074,8 +1084,20 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1097,6 +1119,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEBF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1471,7 +1499,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1754,36 +1782,6 @@
     <xf numFmtId="0" fontId="17" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1797,6 +1795,57 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6243,600 +6292,31 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultRowHeight="13.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="9" customHeight="1"/>
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="38.5546875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="40.5546875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="12.109375" style="5" customWidth="1"/>
-    <col min="9" max="256" width="9" style="1" customWidth="1"/>
-    <col min="257" max="257" width="9.33203125" style="1" customWidth="1"/>
-    <col min="258" max="258" width="6.33203125" style="1" customWidth="1"/>
-    <col min="259" max="259" width="47" style="1" customWidth="1"/>
-    <col min="260" max="260" width="43.33203125" style="1" customWidth="1"/>
-    <col min="261" max="261" width="13.33203125" style="1" customWidth="1"/>
-    <col min="262" max="262" width="10.6640625" style="1" customWidth="1"/>
-    <col min="263" max="263" width="12.44140625" style="1" customWidth="1"/>
-    <col min="264" max="264" width="12.109375" style="1" customWidth="1"/>
-    <col min="265" max="512" width="9" style="1" customWidth="1"/>
-    <col min="513" max="513" width="9.33203125" style="1" customWidth="1"/>
-    <col min="514" max="514" width="6.33203125" style="1" customWidth="1"/>
-    <col min="515" max="515" width="47" style="1" customWidth="1"/>
-    <col min="516" max="516" width="43.33203125" style="1" customWidth="1"/>
-    <col min="517" max="517" width="13.33203125" style="1" customWidth="1"/>
-    <col min="518" max="518" width="10.6640625" style="1" customWidth="1"/>
-    <col min="519" max="519" width="12.44140625" style="1" customWidth="1"/>
-    <col min="520" max="520" width="12.109375" style="1" customWidth="1"/>
-    <col min="521" max="768" width="9" style="1" customWidth="1"/>
-    <col min="769" max="769" width="9.33203125" style="1" customWidth="1"/>
-    <col min="770" max="770" width="6.33203125" style="1" customWidth="1"/>
-    <col min="771" max="771" width="47" style="1" customWidth="1"/>
-    <col min="772" max="772" width="43.33203125" style="1" customWidth="1"/>
-    <col min="773" max="773" width="13.33203125" style="1" customWidth="1"/>
-    <col min="774" max="774" width="10.6640625" style="1" customWidth="1"/>
-    <col min="775" max="775" width="12.44140625" style="1" customWidth="1"/>
-    <col min="776" max="776" width="12.109375" style="1" customWidth="1"/>
-    <col min="777" max="1024" width="9" style="1" customWidth="1"/>
-    <col min="1025" max="1025" width="9.33203125" style="1" customWidth="1"/>
-    <col min="1026" max="1026" width="6.33203125" style="1" customWidth="1"/>
-    <col min="1027" max="1027" width="47" style="1" customWidth="1"/>
-    <col min="1028" max="1028" width="43.33203125" style="1" customWidth="1"/>
-    <col min="1029" max="1029" width="13.33203125" style="1" customWidth="1"/>
-    <col min="1030" max="1030" width="10.6640625" style="1" customWidth="1"/>
-    <col min="1031" max="1031" width="12.44140625" style="1" customWidth="1"/>
-    <col min="1032" max="1032" width="12.109375" style="1" customWidth="1"/>
-    <col min="1033" max="1280" width="9" style="1" customWidth="1"/>
-    <col min="1281" max="1281" width="9.33203125" style="1" customWidth="1"/>
-    <col min="1282" max="1282" width="6.33203125" style="1" customWidth="1"/>
-    <col min="1283" max="1283" width="47" style="1" customWidth="1"/>
-    <col min="1284" max="1284" width="43.33203125" style="1" customWidth="1"/>
-    <col min="1285" max="1285" width="13.33203125" style="1" customWidth="1"/>
-    <col min="1286" max="1286" width="10.6640625" style="1" customWidth="1"/>
-    <col min="1287" max="1287" width="12.44140625" style="1" customWidth="1"/>
-    <col min="1288" max="1288" width="12.109375" style="1" customWidth="1"/>
-    <col min="1289" max="1536" width="9" style="1" customWidth="1"/>
-    <col min="1537" max="1537" width="9.33203125" style="1" customWidth="1"/>
-    <col min="1538" max="1538" width="6.33203125" style="1" customWidth="1"/>
-    <col min="1539" max="1539" width="47" style="1" customWidth="1"/>
-    <col min="1540" max="1540" width="43.33203125" style="1" customWidth="1"/>
-    <col min="1541" max="1541" width="13.33203125" style="1" customWidth="1"/>
-    <col min="1542" max="1542" width="10.6640625" style="1" customWidth="1"/>
-    <col min="1543" max="1543" width="12.44140625" style="1" customWidth="1"/>
-    <col min="1544" max="1544" width="12.109375" style="1" customWidth="1"/>
-    <col min="1545" max="1792" width="9" style="1" customWidth="1"/>
-    <col min="1793" max="1793" width="9.33203125" style="1" customWidth="1"/>
-    <col min="1794" max="1794" width="6.33203125" style="1" customWidth="1"/>
-    <col min="1795" max="1795" width="47" style="1" customWidth="1"/>
-    <col min="1796" max="1796" width="43.33203125" style="1" customWidth="1"/>
-    <col min="1797" max="1797" width="13.33203125" style="1" customWidth="1"/>
-    <col min="1798" max="1798" width="10.6640625" style="1" customWidth="1"/>
-    <col min="1799" max="1799" width="12.44140625" style="1" customWidth="1"/>
-    <col min="1800" max="1800" width="12.109375" style="1" customWidth="1"/>
-    <col min="1801" max="2048" width="9" style="1" customWidth="1"/>
-    <col min="2049" max="2049" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2050" max="2050" width="6.33203125" style="1" customWidth="1"/>
-    <col min="2051" max="2051" width="47" style="1" customWidth="1"/>
-    <col min="2052" max="2052" width="43.33203125" style="1" customWidth="1"/>
-    <col min="2053" max="2053" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2054" max="2054" width="10.6640625" style="1" customWidth="1"/>
-    <col min="2055" max="2055" width="12.44140625" style="1" customWidth="1"/>
-    <col min="2056" max="2056" width="12.109375" style="1" customWidth="1"/>
-    <col min="2057" max="2304" width="9" style="1" customWidth="1"/>
-    <col min="2305" max="2305" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2306" max="2306" width="6.33203125" style="1" customWidth="1"/>
-    <col min="2307" max="2307" width="47" style="1" customWidth="1"/>
-    <col min="2308" max="2308" width="43.33203125" style="1" customWidth="1"/>
-    <col min="2309" max="2309" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2310" max="2310" width="10.6640625" style="1" customWidth="1"/>
-    <col min="2311" max="2311" width="12.44140625" style="1" customWidth="1"/>
-    <col min="2312" max="2312" width="12.109375" style="1" customWidth="1"/>
-    <col min="2313" max="2560" width="9" style="1" customWidth="1"/>
-    <col min="2561" max="2561" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2562" max="2562" width="6.33203125" style="1" customWidth="1"/>
-    <col min="2563" max="2563" width="47" style="1" customWidth="1"/>
-    <col min="2564" max="2564" width="43.33203125" style="1" customWidth="1"/>
-    <col min="2565" max="2565" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2566" max="2566" width="10.6640625" style="1" customWidth="1"/>
-    <col min="2567" max="2567" width="12.44140625" style="1" customWidth="1"/>
-    <col min="2568" max="2568" width="12.109375" style="1" customWidth="1"/>
-    <col min="2569" max="2816" width="9" style="1" customWidth="1"/>
-    <col min="2817" max="2817" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2818" max="2818" width="6.33203125" style="1" customWidth="1"/>
-    <col min="2819" max="2819" width="47" style="1" customWidth="1"/>
-    <col min="2820" max="2820" width="43.33203125" style="1" customWidth="1"/>
-    <col min="2821" max="2821" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2822" max="2822" width="10.6640625" style="1" customWidth="1"/>
-    <col min="2823" max="2823" width="12.44140625" style="1" customWidth="1"/>
-    <col min="2824" max="2824" width="12.109375" style="1" customWidth="1"/>
-    <col min="2825" max="3072" width="9" style="1" customWidth="1"/>
-    <col min="3073" max="3073" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3074" max="3074" width="6.33203125" style="1" customWidth="1"/>
-    <col min="3075" max="3075" width="47" style="1" customWidth="1"/>
-    <col min="3076" max="3076" width="43.33203125" style="1" customWidth="1"/>
-    <col min="3077" max="3077" width="13.33203125" style="1" customWidth="1"/>
-    <col min="3078" max="3078" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3079" max="3079" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3080" max="3080" width="12.109375" style="1" customWidth="1"/>
-    <col min="3081" max="3328" width="9" style="1" customWidth="1"/>
-    <col min="3329" max="3329" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3330" max="3330" width="6.33203125" style="1" customWidth="1"/>
-    <col min="3331" max="3331" width="47" style="1" customWidth="1"/>
-    <col min="3332" max="3332" width="43.33203125" style="1" customWidth="1"/>
-    <col min="3333" max="3333" width="13.33203125" style="1" customWidth="1"/>
-    <col min="3334" max="3334" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3335" max="3335" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3336" max="3336" width="12.109375" style="1" customWidth="1"/>
-    <col min="3337" max="3584" width="9" style="1" customWidth="1"/>
-    <col min="3585" max="3585" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3586" max="3586" width="6.33203125" style="1" customWidth="1"/>
-    <col min="3587" max="3587" width="47" style="1" customWidth="1"/>
-    <col min="3588" max="3588" width="43.33203125" style="1" customWidth="1"/>
-    <col min="3589" max="3589" width="13.33203125" style="1" customWidth="1"/>
-    <col min="3590" max="3590" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3591" max="3591" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3592" max="3592" width="12.109375" style="1" customWidth="1"/>
-    <col min="3593" max="3840" width="9" style="1" customWidth="1"/>
-    <col min="3841" max="3841" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3842" max="3842" width="6.33203125" style="1" customWidth="1"/>
-    <col min="3843" max="3843" width="47" style="1" customWidth="1"/>
-    <col min="3844" max="3844" width="43.33203125" style="1" customWidth="1"/>
-    <col min="3845" max="3845" width="13.33203125" style="1" customWidth="1"/>
-    <col min="3846" max="3846" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3847" max="3847" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3848" max="3848" width="12.109375" style="1" customWidth="1"/>
-    <col min="3849" max="4096" width="9" style="1" customWidth="1"/>
-    <col min="4097" max="4097" width="9.33203125" style="1" customWidth="1"/>
-    <col min="4098" max="4098" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4099" max="4099" width="47" style="1" customWidth="1"/>
-    <col min="4100" max="4100" width="43.33203125" style="1" customWidth="1"/>
-    <col min="4101" max="4101" width="13.33203125" style="1" customWidth="1"/>
-    <col min="4102" max="4102" width="10.6640625" style="1" customWidth="1"/>
-    <col min="4103" max="4103" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4104" max="4104" width="12.109375" style="1" customWidth="1"/>
-    <col min="4105" max="4352" width="9" style="1" customWidth="1"/>
-    <col min="4353" max="4353" width="9.33203125" style="1" customWidth="1"/>
-    <col min="4354" max="4354" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4355" max="4355" width="47" style="1" customWidth="1"/>
-    <col min="4356" max="4356" width="43.33203125" style="1" customWidth="1"/>
-    <col min="4357" max="4357" width="13.33203125" style="1" customWidth="1"/>
-    <col min="4358" max="4358" width="10.6640625" style="1" customWidth="1"/>
-    <col min="4359" max="4359" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4360" max="4360" width="12.109375" style="1" customWidth="1"/>
-    <col min="4361" max="4608" width="9" style="1" customWidth="1"/>
-    <col min="4609" max="4609" width="9.33203125" style="1" customWidth="1"/>
-    <col min="4610" max="4610" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4611" max="4611" width="47" style="1" customWidth="1"/>
-    <col min="4612" max="4612" width="43.33203125" style="1" customWidth="1"/>
-    <col min="4613" max="4613" width="13.33203125" style="1" customWidth="1"/>
-    <col min="4614" max="4614" width="10.6640625" style="1" customWidth="1"/>
-    <col min="4615" max="4615" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4616" max="4616" width="12.109375" style="1" customWidth="1"/>
-    <col min="4617" max="4864" width="9" style="1" customWidth="1"/>
-    <col min="4865" max="4865" width="9.33203125" style="1" customWidth="1"/>
-    <col min="4866" max="4866" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4867" max="4867" width="47" style="1" customWidth="1"/>
-    <col min="4868" max="4868" width="43.33203125" style="1" customWidth="1"/>
-    <col min="4869" max="4869" width="13.33203125" style="1" customWidth="1"/>
-    <col min="4870" max="4870" width="10.6640625" style="1" customWidth="1"/>
-    <col min="4871" max="4871" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4872" max="4872" width="12.109375" style="1" customWidth="1"/>
-    <col min="4873" max="5120" width="9" style="1" customWidth="1"/>
-    <col min="5121" max="5121" width="9.33203125" style="1" customWidth="1"/>
-    <col min="5122" max="5122" width="6.33203125" style="1" customWidth="1"/>
-    <col min="5123" max="5123" width="47" style="1" customWidth="1"/>
-    <col min="5124" max="5124" width="43.33203125" style="1" customWidth="1"/>
-    <col min="5125" max="5125" width="13.33203125" style="1" customWidth="1"/>
-    <col min="5126" max="5126" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5127" max="5127" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5128" max="5128" width="12.109375" style="1" customWidth="1"/>
-    <col min="5129" max="5376" width="9" style="1" customWidth="1"/>
-    <col min="5377" max="5377" width="9.33203125" style="1" customWidth="1"/>
-    <col min="5378" max="5378" width="6.33203125" style="1" customWidth="1"/>
-    <col min="5379" max="5379" width="47" style="1" customWidth="1"/>
-    <col min="5380" max="5380" width="43.33203125" style="1" customWidth="1"/>
-    <col min="5381" max="5381" width="13.33203125" style="1" customWidth="1"/>
-    <col min="5382" max="5382" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5383" max="5383" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5384" max="5384" width="12.109375" style="1" customWidth="1"/>
-    <col min="5385" max="5632" width="9" style="1" customWidth="1"/>
-    <col min="5633" max="5633" width="9.33203125" style="1" customWidth="1"/>
-    <col min="5634" max="5634" width="6.33203125" style="1" customWidth="1"/>
-    <col min="5635" max="5635" width="47" style="1" customWidth="1"/>
-    <col min="5636" max="5636" width="43.33203125" style="1" customWidth="1"/>
-    <col min="5637" max="5637" width="13.33203125" style="1" customWidth="1"/>
-    <col min="5638" max="5638" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5639" max="5639" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5640" max="5640" width="12.109375" style="1" customWidth="1"/>
-    <col min="5641" max="5888" width="9" style="1" customWidth="1"/>
-    <col min="5889" max="5889" width="9.33203125" style="1" customWidth="1"/>
-    <col min="5890" max="5890" width="6.33203125" style="1" customWidth="1"/>
-    <col min="5891" max="5891" width="47" style="1" customWidth="1"/>
-    <col min="5892" max="5892" width="43.33203125" style="1" customWidth="1"/>
-    <col min="5893" max="5893" width="13.33203125" style="1" customWidth="1"/>
-    <col min="5894" max="5894" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5895" max="5895" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5896" max="5896" width="12.109375" style="1" customWidth="1"/>
-    <col min="5897" max="6144" width="9" style="1" customWidth="1"/>
-    <col min="6145" max="6145" width="9.33203125" style="1" customWidth="1"/>
-    <col min="6146" max="6146" width="6.33203125" style="1" customWidth="1"/>
-    <col min="6147" max="6147" width="47" style="1" customWidth="1"/>
-    <col min="6148" max="6148" width="43.33203125" style="1" customWidth="1"/>
-    <col min="6149" max="6149" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6150" max="6150" width="10.6640625" style="1" customWidth="1"/>
-    <col min="6151" max="6151" width="12.44140625" style="1" customWidth="1"/>
-    <col min="6152" max="6152" width="12.109375" style="1" customWidth="1"/>
-    <col min="6153" max="6400" width="9" style="1" customWidth="1"/>
-    <col min="6401" max="6401" width="9.33203125" style="1" customWidth="1"/>
-    <col min="6402" max="6402" width="6.33203125" style="1" customWidth="1"/>
-    <col min="6403" max="6403" width="47" style="1" customWidth="1"/>
-    <col min="6404" max="6404" width="43.33203125" style="1" customWidth="1"/>
-    <col min="6405" max="6405" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6406" max="6406" width="10.6640625" style="1" customWidth="1"/>
-    <col min="6407" max="6407" width="12.44140625" style="1" customWidth="1"/>
-    <col min="6408" max="6408" width="12.109375" style="1" customWidth="1"/>
-    <col min="6409" max="6656" width="9" style="1" customWidth="1"/>
-    <col min="6657" max="6657" width="9.33203125" style="1" customWidth="1"/>
-    <col min="6658" max="6658" width="6.33203125" style="1" customWidth="1"/>
-    <col min="6659" max="6659" width="47" style="1" customWidth="1"/>
-    <col min="6660" max="6660" width="43.33203125" style="1" customWidth="1"/>
-    <col min="6661" max="6661" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6662" max="6662" width="10.6640625" style="1" customWidth="1"/>
-    <col min="6663" max="6663" width="12.44140625" style="1" customWidth="1"/>
-    <col min="6664" max="6664" width="12.109375" style="1" customWidth="1"/>
-    <col min="6665" max="6912" width="9" style="1" customWidth="1"/>
-    <col min="6913" max="6913" width="9.33203125" style="1" customWidth="1"/>
-    <col min="6914" max="6914" width="6.33203125" style="1" customWidth="1"/>
-    <col min="6915" max="6915" width="47" style="1" customWidth="1"/>
-    <col min="6916" max="6916" width="43.33203125" style="1" customWidth="1"/>
-    <col min="6917" max="6917" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6918" max="6918" width="10.6640625" style="1" customWidth="1"/>
-    <col min="6919" max="6919" width="12.44140625" style="1" customWidth="1"/>
-    <col min="6920" max="6920" width="12.109375" style="1" customWidth="1"/>
-    <col min="6921" max="7168" width="9" style="1" customWidth="1"/>
-    <col min="7169" max="7169" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7170" max="7170" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7171" max="7171" width="47" style="1" customWidth="1"/>
-    <col min="7172" max="7172" width="43.33203125" style="1" customWidth="1"/>
-    <col min="7173" max="7173" width="13.33203125" style="1" customWidth="1"/>
-    <col min="7174" max="7174" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7175" max="7175" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7176" max="7176" width="12.109375" style="1" customWidth="1"/>
-    <col min="7177" max="7424" width="9" style="1" customWidth="1"/>
-    <col min="7425" max="7425" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7426" max="7426" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7427" max="7427" width="47" style="1" customWidth="1"/>
-    <col min="7428" max="7428" width="43.33203125" style="1" customWidth="1"/>
-    <col min="7429" max="7429" width="13.33203125" style="1" customWidth="1"/>
-    <col min="7430" max="7430" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7431" max="7431" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7432" max="7432" width="12.109375" style="1" customWidth="1"/>
-    <col min="7433" max="7680" width="9" style="1" customWidth="1"/>
-    <col min="7681" max="7681" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7682" max="7682" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7683" max="7683" width="47" style="1" customWidth="1"/>
-    <col min="7684" max="7684" width="43.33203125" style="1" customWidth="1"/>
-    <col min="7685" max="7685" width="13.33203125" style="1" customWidth="1"/>
-    <col min="7686" max="7686" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7687" max="7687" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7688" max="7688" width="12.109375" style="1" customWidth="1"/>
-    <col min="7689" max="7936" width="9" style="1" customWidth="1"/>
-    <col min="7937" max="7937" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7938" max="7938" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7939" max="7939" width="47" style="1" customWidth="1"/>
-    <col min="7940" max="7940" width="43.33203125" style="1" customWidth="1"/>
-    <col min="7941" max="7941" width="13.33203125" style="1" customWidth="1"/>
-    <col min="7942" max="7942" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7943" max="7943" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7944" max="7944" width="12.109375" style="1" customWidth="1"/>
-    <col min="7945" max="8192" width="9" style="1" customWidth="1"/>
-    <col min="8193" max="8193" width="9.33203125" style="1" customWidth="1"/>
-    <col min="8194" max="8194" width="6.33203125" style="1" customWidth="1"/>
-    <col min="8195" max="8195" width="47" style="1" customWidth="1"/>
-    <col min="8196" max="8196" width="43.33203125" style="1" customWidth="1"/>
-    <col min="8197" max="8197" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8198" max="8198" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8199" max="8199" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8200" max="8200" width="12.109375" style="1" customWidth="1"/>
-    <col min="8201" max="8448" width="9" style="1" customWidth="1"/>
-    <col min="8449" max="8449" width="9.33203125" style="1" customWidth="1"/>
-    <col min="8450" max="8450" width="6.33203125" style="1" customWidth="1"/>
-    <col min="8451" max="8451" width="47" style="1" customWidth="1"/>
-    <col min="8452" max="8452" width="43.33203125" style="1" customWidth="1"/>
-    <col min="8453" max="8453" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8454" max="8454" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8455" max="8455" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8456" max="8456" width="12.109375" style="1" customWidth="1"/>
-    <col min="8457" max="8704" width="9" style="1" customWidth="1"/>
-    <col min="8705" max="8705" width="9.33203125" style="1" customWidth="1"/>
-    <col min="8706" max="8706" width="6.33203125" style="1" customWidth="1"/>
-    <col min="8707" max="8707" width="47" style="1" customWidth="1"/>
-    <col min="8708" max="8708" width="43.33203125" style="1" customWidth="1"/>
-    <col min="8709" max="8709" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8710" max="8710" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8711" max="8711" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8712" max="8712" width="12.109375" style="1" customWidth="1"/>
-    <col min="8713" max="8960" width="9" style="1" customWidth="1"/>
-    <col min="8961" max="8961" width="9.33203125" style="1" customWidth="1"/>
-    <col min="8962" max="8962" width="6.33203125" style="1" customWidth="1"/>
-    <col min="8963" max="8963" width="47" style="1" customWidth="1"/>
-    <col min="8964" max="8964" width="43.33203125" style="1" customWidth="1"/>
-    <col min="8965" max="8965" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8966" max="8966" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8967" max="8967" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8968" max="8968" width="12.109375" style="1" customWidth="1"/>
-    <col min="8969" max="9216" width="9" style="1" customWidth="1"/>
-    <col min="9217" max="9217" width="9.33203125" style="1" customWidth="1"/>
-    <col min="9218" max="9218" width="6.33203125" style="1" customWidth="1"/>
-    <col min="9219" max="9219" width="47" style="1" customWidth="1"/>
-    <col min="9220" max="9220" width="43.33203125" style="1" customWidth="1"/>
-    <col min="9221" max="9221" width="13.33203125" style="1" customWidth="1"/>
-    <col min="9222" max="9222" width="10.6640625" style="1" customWidth="1"/>
-    <col min="9223" max="9223" width="12.44140625" style="1" customWidth="1"/>
-    <col min="9224" max="9224" width="12.109375" style="1" customWidth="1"/>
-    <col min="9225" max="9472" width="9" style="1" customWidth="1"/>
-    <col min="9473" max="9473" width="9.33203125" style="1" customWidth="1"/>
-    <col min="9474" max="9474" width="6.33203125" style="1" customWidth="1"/>
-    <col min="9475" max="9475" width="47" style="1" customWidth="1"/>
-    <col min="9476" max="9476" width="43.33203125" style="1" customWidth="1"/>
-    <col min="9477" max="9477" width="13.33203125" style="1" customWidth="1"/>
-    <col min="9478" max="9478" width="10.6640625" style="1" customWidth="1"/>
-    <col min="9479" max="9479" width="12.44140625" style="1" customWidth="1"/>
-    <col min="9480" max="9480" width="12.109375" style="1" customWidth="1"/>
-    <col min="9481" max="9728" width="9" style="1" customWidth="1"/>
-    <col min="9729" max="9729" width="9.33203125" style="1" customWidth="1"/>
-    <col min="9730" max="9730" width="6.33203125" style="1" customWidth="1"/>
-    <col min="9731" max="9731" width="47" style="1" customWidth="1"/>
-    <col min="9732" max="9732" width="43.33203125" style="1" customWidth="1"/>
-    <col min="9733" max="9733" width="13.33203125" style="1" customWidth="1"/>
-    <col min="9734" max="9734" width="10.6640625" style="1" customWidth="1"/>
-    <col min="9735" max="9735" width="12.44140625" style="1" customWidth="1"/>
-    <col min="9736" max="9736" width="12.109375" style="1" customWidth="1"/>
-    <col min="9737" max="9984" width="9" style="1" customWidth="1"/>
-    <col min="9985" max="9985" width="9.33203125" style="1" customWidth="1"/>
-    <col min="9986" max="9986" width="6.33203125" style="1" customWidth="1"/>
-    <col min="9987" max="9987" width="47" style="1" customWidth="1"/>
-    <col min="9988" max="9988" width="43.33203125" style="1" customWidth="1"/>
-    <col min="9989" max="9989" width="13.33203125" style="1" customWidth="1"/>
-    <col min="9990" max="9990" width="10.6640625" style="1" customWidth="1"/>
-    <col min="9991" max="9991" width="12.44140625" style="1" customWidth="1"/>
-    <col min="9992" max="9992" width="12.109375" style="1" customWidth="1"/>
-    <col min="9993" max="10240" width="9" style="1" customWidth="1"/>
-    <col min="10241" max="10241" width="9.33203125" style="1" customWidth="1"/>
-    <col min="10242" max="10242" width="6.33203125" style="1" customWidth="1"/>
-    <col min="10243" max="10243" width="47" style="1" customWidth="1"/>
-    <col min="10244" max="10244" width="43.33203125" style="1" customWidth="1"/>
-    <col min="10245" max="10245" width="13.33203125" style="1" customWidth="1"/>
-    <col min="10246" max="10246" width="10.6640625" style="1" customWidth="1"/>
-    <col min="10247" max="10247" width="12.44140625" style="1" customWidth="1"/>
-    <col min="10248" max="10248" width="12.109375" style="1" customWidth="1"/>
-    <col min="10249" max="10496" width="9" style="1" customWidth="1"/>
-    <col min="10497" max="10497" width="9.33203125" style="1" customWidth="1"/>
-    <col min="10498" max="10498" width="6.33203125" style="1" customWidth="1"/>
-    <col min="10499" max="10499" width="47" style="1" customWidth="1"/>
-    <col min="10500" max="10500" width="43.33203125" style="1" customWidth="1"/>
-    <col min="10501" max="10501" width="13.33203125" style="1" customWidth="1"/>
-    <col min="10502" max="10502" width="10.6640625" style="1" customWidth="1"/>
-    <col min="10503" max="10503" width="12.44140625" style="1" customWidth="1"/>
-    <col min="10504" max="10504" width="12.109375" style="1" customWidth="1"/>
-    <col min="10505" max="10752" width="9" style="1" customWidth="1"/>
-    <col min="10753" max="10753" width="9.33203125" style="1" customWidth="1"/>
-    <col min="10754" max="10754" width="6.33203125" style="1" customWidth="1"/>
-    <col min="10755" max="10755" width="47" style="1" customWidth="1"/>
-    <col min="10756" max="10756" width="43.33203125" style="1" customWidth="1"/>
-    <col min="10757" max="10757" width="13.33203125" style="1" customWidth="1"/>
-    <col min="10758" max="10758" width="10.6640625" style="1" customWidth="1"/>
-    <col min="10759" max="10759" width="12.44140625" style="1" customWidth="1"/>
-    <col min="10760" max="10760" width="12.109375" style="1" customWidth="1"/>
-    <col min="10761" max="11008" width="9" style="1" customWidth="1"/>
-    <col min="11009" max="11009" width="9.33203125" style="1" customWidth="1"/>
-    <col min="11010" max="11010" width="6.33203125" style="1" customWidth="1"/>
-    <col min="11011" max="11011" width="47" style="1" customWidth="1"/>
-    <col min="11012" max="11012" width="43.33203125" style="1" customWidth="1"/>
-    <col min="11013" max="11013" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11014" max="11014" width="10.6640625" style="1" customWidth="1"/>
-    <col min="11015" max="11015" width="12.44140625" style="1" customWidth="1"/>
-    <col min="11016" max="11016" width="12.109375" style="1" customWidth="1"/>
-    <col min="11017" max="11264" width="9" style="1" customWidth="1"/>
-    <col min="11265" max="11265" width="9.33203125" style="1" customWidth="1"/>
-    <col min="11266" max="11266" width="6.33203125" style="1" customWidth="1"/>
-    <col min="11267" max="11267" width="47" style="1" customWidth="1"/>
-    <col min="11268" max="11268" width="43.33203125" style="1" customWidth="1"/>
-    <col min="11269" max="11269" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11270" max="11270" width="10.6640625" style="1" customWidth="1"/>
-    <col min="11271" max="11271" width="12.44140625" style="1" customWidth="1"/>
-    <col min="11272" max="11272" width="12.109375" style="1" customWidth="1"/>
-    <col min="11273" max="11520" width="9" style="1" customWidth="1"/>
-    <col min="11521" max="11521" width="9.33203125" style="1" customWidth="1"/>
-    <col min="11522" max="11522" width="6.33203125" style="1" customWidth="1"/>
-    <col min="11523" max="11523" width="47" style="1" customWidth="1"/>
-    <col min="11524" max="11524" width="43.33203125" style="1" customWidth="1"/>
-    <col min="11525" max="11525" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11526" max="11526" width="10.6640625" style="1" customWidth="1"/>
-    <col min="11527" max="11527" width="12.44140625" style="1" customWidth="1"/>
-    <col min="11528" max="11528" width="12.109375" style="1" customWidth="1"/>
-    <col min="11529" max="11776" width="9" style="1" customWidth="1"/>
-    <col min="11777" max="11777" width="9.33203125" style="1" customWidth="1"/>
-    <col min="11778" max="11778" width="6.33203125" style="1" customWidth="1"/>
-    <col min="11779" max="11779" width="47" style="1" customWidth="1"/>
-    <col min="11780" max="11780" width="43.33203125" style="1" customWidth="1"/>
-    <col min="11781" max="11781" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11782" max="11782" width="10.6640625" style="1" customWidth="1"/>
-    <col min="11783" max="11783" width="12.44140625" style="1" customWidth="1"/>
-    <col min="11784" max="11784" width="12.109375" style="1" customWidth="1"/>
-    <col min="11785" max="12032" width="9" style="1" customWidth="1"/>
-    <col min="12033" max="12033" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12034" max="12034" width="6.33203125" style="1" customWidth="1"/>
-    <col min="12035" max="12035" width="47" style="1" customWidth="1"/>
-    <col min="12036" max="12036" width="43.33203125" style="1" customWidth="1"/>
-    <col min="12037" max="12037" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12038" max="12038" width="10.6640625" style="1" customWidth="1"/>
-    <col min="12039" max="12039" width="12.44140625" style="1" customWidth="1"/>
-    <col min="12040" max="12040" width="12.109375" style="1" customWidth="1"/>
-    <col min="12041" max="12288" width="9" style="1" customWidth="1"/>
-    <col min="12289" max="12289" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12290" max="12290" width="6.33203125" style="1" customWidth="1"/>
-    <col min="12291" max="12291" width="47" style="1" customWidth="1"/>
-    <col min="12292" max="12292" width="43.33203125" style="1" customWidth="1"/>
-    <col min="12293" max="12293" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12294" max="12294" width="10.6640625" style="1" customWidth="1"/>
-    <col min="12295" max="12295" width="12.44140625" style="1" customWidth="1"/>
-    <col min="12296" max="12296" width="12.109375" style="1" customWidth="1"/>
-    <col min="12297" max="12544" width="9" style="1" customWidth="1"/>
-    <col min="12545" max="12545" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12546" max="12546" width="6.33203125" style="1" customWidth="1"/>
-    <col min="12547" max="12547" width="47" style="1" customWidth="1"/>
-    <col min="12548" max="12548" width="43.33203125" style="1" customWidth="1"/>
-    <col min="12549" max="12549" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12550" max="12550" width="10.6640625" style="1" customWidth="1"/>
-    <col min="12551" max="12551" width="12.44140625" style="1" customWidth="1"/>
-    <col min="12552" max="12552" width="12.109375" style="1" customWidth="1"/>
-    <col min="12553" max="12800" width="9" style="1" customWidth="1"/>
-    <col min="12801" max="12801" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12802" max="12802" width="6.33203125" style="1" customWidth="1"/>
-    <col min="12803" max="12803" width="47" style="1" customWidth="1"/>
-    <col min="12804" max="12804" width="43.33203125" style="1" customWidth="1"/>
-    <col min="12805" max="12805" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12806" max="12806" width="10.6640625" style="1" customWidth="1"/>
-    <col min="12807" max="12807" width="12.44140625" style="1" customWidth="1"/>
-    <col min="12808" max="12808" width="12.109375" style="1" customWidth="1"/>
-    <col min="12809" max="13056" width="9" style="1" customWidth="1"/>
-    <col min="13057" max="13057" width="9.33203125" style="1" customWidth="1"/>
-    <col min="13058" max="13058" width="6.33203125" style="1" customWidth="1"/>
-    <col min="13059" max="13059" width="47" style="1" customWidth="1"/>
-    <col min="13060" max="13060" width="43.33203125" style="1" customWidth="1"/>
-    <col min="13061" max="13061" width="13.33203125" style="1" customWidth="1"/>
-    <col min="13062" max="13062" width="10.6640625" style="1" customWidth="1"/>
-    <col min="13063" max="13063" width="12.44140625" style="1" customWidth="1"/>
-    <col min="13064" max="13064" width="12.109375" style="1" customWidth="1"/>
-    <col min="13065" max="13312" width="9" style="1" customWidth="1"/>
-    <col min="13313" max="13313" width="9.33203125" style="1" customWidth="1"/>
-    <col min="13314" max="13314" width="6.33203125" style="1" customWidth="1"/>
-    <col min="13315" max="13315" width="47" style="1" customWidth="1"/>
-    <col min="13316" max="13316" width="43.33203125" style="1" customWidth="1"/>
-    <col min="13317" max="13317" width="13.33203125" style="1" customWidth="1"/>
-    <col min="13318" max="13318" width="10.6640625" style="1" customWidth="1"/>
-    <col min="13319" max="13319" width="12.44140625" style="1" customWidth="1"/>
-    <col min="13320" max="13320" width="12.109375" style="1" customWidth="1"/>
-    <col min="13321" max="13568" width="9" style="1" customWidth="1"/>
-    <col min="13569" max="13569" width="9.33203125" style="1" customWidth="1"/>
-    <col min="13570" max="13570" width="6.33203125" style="1" customWidth="1"/>
-    <col min="13571" max="13571" width="47" style="1" customWidth="1"/>
-    <col min="13572" max="13572" width="43.33203125" style="1" customWidth="1"/>
-    <col min="13573" max="13573" width="13.33203125" style="1" customWidth="1"/>
-    <col min="13574" max="13574" width="10.6640625" style="1" customWidth="1"/>
-    <col min="13575" max="13575" width="12.44140625" style="1" customWidth="1"/>
-    <col min="13576" max="13576" width="12.109375" style="1" customWidth="1"/>
-    <col min="13577" max="13824" width="9" style="1" customWidth="1"/>
-    <col min="13825" max="13825" width="9.33203125" style="1" customWidth="1"/>
-    <col min="13826" max="13826" width="6.33203125" style="1" customWidth="1"/>
-    <col min="13827" max="13827" width="47" style="1" customWidth="1"/>
-    <col min="13828" max="13828" width="43.33203125" style="1" customWidth="1"/>
-    <col min="13829" max="13829" width="13.33203125" style="1" customWidth="1"/>
-    <col min="13830" max="13830" width="10.6640625" style="1" customWidth="1"/>
-    <col min="13831" max="13831" width="12.44140625" style="1" customWidth="1"/>
-    <col min="13832" max="13832" width="12.109375" style="1" customWidth="1"/>
-    <col min="13833" max="14080" width="9" style="1" customWidth="1"/>
-    <col min="14081" max="14081" width="9.33203125" style="1" customWidth="1"/>
-    <col min="14082" max="14082" width="6.33203125" style="1" customWidth="1"/>
-    <col min="14083" max="14083" width="47" style="1" customWidth="1"/>
-    <col min="14084" max="14084" width="43.33203125" style="1" customWidth="1"/>
-    <col min="14085" max="14085" width="13.33203125" style="1" customWidth="1"/>
-    <col min="14086" max="14086" width="10.6640625" style="1" customWidth="1"/>
-    <col min="14087" max="14087" width="12.44140625" style="1" customWidth="1"/>
-    <col min="14088" max="14088" width="12.109375" style="1" customWidth="1"/>
-    <col min="14089" max="14336" width="9" style="1" customWidth="1"/>
-    <col min="14337" max="14337" width="9.33203125" style="1" customWidth="1"/>
-    <col min="14338" max="14338" width="6.33203125" style="1" customWidth="1"/>
-    <col min="14339" max="14339" width="47" style="1" customWidth="1"/>
-    <col min="14340" max="14340" width="43.33203125" style="1" customWidth="1"/>
-    <col min="14341" max="14341" width="13.33203125" style="1" customWidth="1"/>
-    <col min="14342" max="14342" width="10.6640625" style="1" customWidth="1"/>
-    <col min="14343" max="14343" width="12.44140625" style="1" customWidth="1"/>
-    <col min="14344" max="14344" width="12.109375" style="1" customWidth="1"/>
-    <col min="14345" max="14592" width="9" style="1" customWidth="1"/>
-    <col min="14593" max="14593" width="9.33203125" style="1" customWidth="1"/>
-    <col min="14594" max="14594" width="6.33203125" style="1" customWidth="1"/>
-    <col min="14595" max="14595" width="47" style="1" customWidth="1"/>
-    <col min="14596" max="14596" width="43.33203125" style="1" customWidth="1"/>
-    <col min="14597" max="14597" width="13.33203125" style="1" customWidth="1"/>
-    <col min="14598" max="14598" width="10.6640625" style="1" customWidth="1"/>
-    <col min="14599" max="14599" width="12.44140625" style="1" customWidth="1"/>
-    <col min="14600" max="14600" width="12.109375" style="1" customWidth="1"/>
-    <col min="14601" max="14848" width="9" style="1" customWidth="1"/>
-    <col min="14849" max="14849" width="9.33203125" style="1" customWidth="1"/>
-    <col min="14850" max="14850" width="6.33203125" style="1" customWidth="1"/>
-    <col min="14851" max="14851" width="47" style="1" customWidth="1"/>
-    <col min="14852" max="14852" width="43.33203125" style="1" customWidth="1"/>
-    <col min="14853" max="14853" width="13.33203125" style="1" customWidth="1"/>
-    <col min="14854" max="14854" width="10.6640625" style="1" customWidth="1"/>
-    <col min="14855" max="14855" width="12.44140625" style="1" customWidth="1"/>
-    <col min="14856" max="14856" width="12.109375" style="1" customWidth="1"/>
-    <col min="14857" max="15104" width="9" style="1" customWidth="1"/>
-    <col min="15105" max="15105" width="9.33203125" style="1" customWidth="1"/>
-    <col min="15106" max="15106" width="6.33203125" style="1" customWidth="1"/>
-    <col min="15107" max="15107" width="47" style="1" customWidth="1"/>
-    <col min="15108" max="15108" width="43.33203125" style="1" customWidth="1"/>
-    <col min="15109" max="15109" width="13.33203125" style="1" customWidth="1"/>
-    <col min="15110" max="15110" width="10.6640625" style="1" customWidth="1"/>
-    <col min="15111" max="15111" width="12.44140625" style="1" customWidth="1"/>
-    <col min="15112" max="15112" width="12.109375" style="1" customWidth="1"/>
-    <col min="15113" max="15360" width="9" style="1" customWidth="1"/>
-    <col min="15361" max="15361" width="9.33203125" style="1" customWidth="1"/>
-    <col min="15362" max="15362" width="6.33203125" style="1" customWidth="1"/>
-    <col min="15363" max="15363" width="47" style="1" customWidth="1"/>
-    <col min="15364" max="15364" width="43.33203125" style="1" customWidth="1"/>
-    <col min="15365" max="15365" width="13.33203125" style="1" customWidth="1"/>
-    <col min="15366" max="15366" width="10.6640625" style="1" customWidth="1"/>
-    <col min="15367" max="15367" width="12.44140625" style="1" customWidth="1"/>
-    <col min="15368" max="15368" width="12.109375" style="1" customWidth="1"/>
-    <col min="15369" max="15616" width="9" style="1" customWidth="1"/>
-    <col min="15617" max="15617" width="9.33203125" style="1" customWidth="1"/>
-    <col min="15618" max="15618" width="6.33203125" style="1" customWidth="1"/>
-    <col min="15619" max="15619" width="47" style="1" customWidth="1"/>
-    <col min="15620" max="15620" width="43.33203125" style="1" customWidth="1"/>
-    <col min="15621" max="15621" width="13.33203125" style="1" customWidth="1"/>
-    <col min="15622" max="15622" width="10.6640625" style="1" customWidth="1"/>
-    <col min="15623" max="15623" width="12.44140625" style="1" customWidth="1"/>
-    <col min="15624" max="15624" width="12.109375" style="1" customWidth="1"/>
-    <col min="15625" max="15872" width="9" style="1" customWidth="1"/>
-    <col min="15873" max="15873" width="9.33203125" style="1" customWidth="1"/>
-    <col min="15874" max="15874" width="6.33203125" style="1" customWidth="1"/>
-    <col min="15875" max="15875" width="47" style="1" customWidth="1"/>
-    <col min="15876" max="15876" width="43.33203125" style="1" customWidth="1"/>
-    <col min="15877" max="15877" width="13.33203125" style="1" customWidth="1"/>
-    <col min="15878" max="15878" width="10.6640625" style="1" customWidth="1"/>
-    <col min="15879" max="15879" width="12.44140625" style="1" customWidth="1"/>
-    <col min="15880" max="15880" width="12.109375" style="1" customWidth="1"/>
-    <col min="15881" max="16128" width="9" style="1" customWidth="1"/>
-    <col min="16129" max="16129" width="9.33203125" style="1" customWidth="1"/>
-    <col min="16130" max="16130" width="6.33203125" style="1" customWidth="1"/>
-    <col min="16131" max="16131" width="47" style="1" customWidth="1"/>
-    <col min="16132" max="16132" width="43.33203125" style="1" customWidth="1"/>
-    <col min="16133" max="16133" width="13.33203125" style="1" customWidth="1"/>
-    <col min="16134" max="16134" width="10.6640625" style="1" customWidth="1"/>
-    <col min="16135" max="16135" width="12.44140625" style="1" customWidth="1"/>
-    <col min="16136" max="16136" width="12.109375" style="1" customWidth="1"/>
-    <col min="16137" max="16384" width="9" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33" customWidth="1"/>
+    <col min="2" max="2" width="6.33" customWidth="1"/>
+    <col min="3" max="3" width="37.44" customWidth="1"/>
+    <col min="4" max="4" width="41.11" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="70" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
     </row>
     <row r="3" ht="8.1" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="8"/>
@@ -6855,9 +6335,9 @@
       <c r="G4" s="9"/>
       <c r="H4" s="9"/>
     </row>
-    <row r="5" ht="19.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" ht="20.25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>194</v>
+        <v>227</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -6867,477 +6347,472 @@
       <c r="G5" s="10"/>
       <c r="H5" s="10"/>
     </row>
-    <row r="6" ht="12" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="10"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-    </row>
-    <row r="7" ht="27.9" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+    <row r="6" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B6" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C6" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D6" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E6" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F6" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G6" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="H6" s="15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" ht="39.9" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="B8" s="17" t="s">
+    <row r="7" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="103" t="s">
+        <v>228</v>
+      </c>
+      <c r="B7" s="104" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>196</v>
-      </c>
-      <c r="D8" s="19" t="s">
+      <c r="C7" s="105" t="s">
+        <v>229</v>
+      </c>
+      <c r="D7" s="106" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="20" t="s">
-        <v>197</v>
-      </c>
-      <c r="F8" s="20"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="30"/>
-    </row>
-    <row r="9" ht="24.9" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="23"/>
-      <c r="B9" s="17" t="s">
+      <c r="E7" s="107" t="s">
+        <v>230</v>
+      </c>
+      <c r="F7" s="107" t="s">
+        <v>231</v>
+      </c>
+      <c r="G7" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="H7" s="108"/>
+    </row>
+    <row r="8" ht="41" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="103"/>
+      <c r="B8" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>198</v>
-      </c>
-      <c r="E9" s="20" t="s">
+      <c r="C8" s="105" t="s">
+        <v>232</v>
+      </c>
+      <c r="D8" s="106" t="s">
+        <v>233</v>
+      </c>
+      <c r="E8" s="107" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="20" t="s">
+      <c r="F8" s="107" t="s">
         <v>24</v>
       </c>
-      <c r="G9" s="21" t="s">
+      <c r="G8" s="104" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="30"/>
-    </row>
-    <row r="10" ht="24.9" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="25"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="D10" s="19" t="s">
+      <c r="H8" s="108"/>
+    </row>
+    <row r="9" ht="41" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="103"/>
+      <c r="B9" s="104"/>
+      <c r="C9" s="105" t="s">
+        <v>234</v>
+      </c>
+      <c r="D9" s="106" t="s">
         <v>143</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E9" s="107" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="20" t="s">
+      <c r="F9" s="107" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="21" t="s">
+      <c r="G9" s="104" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="30"/>
-    </row>
-    <row r="11" ht="44.1" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="26" t="s">
-        <v>200</v>
-      </c>
-      <c r="B11" s="28" t="s">
+      <c r="H9" s="108"/>
+    </row>
+    <row r="10" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="103" t="s">
+        <v>235</v>
+      </c>
+      <c r="B10" s="104" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>201</v>
-      </c>
-      <c r="E11" s="20" t="s">
+      <c r="C10" s="105" t="s">
+        <v>236</v>
+      </c>
+      <c r="D10" s="106" t="s">
+        <v>237</v>
+      </c>
+      <c r="E10" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="20" t="s">
+      <c r="F10" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="G11" s="21"/>
-      <c r="H11" s="30"/>
-    </row>
-    <row r="12" ht="44.1" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="29"/>
-      <c r="B12" s="17" t="s">
+      <c r="G10" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="H10" s="108"/>
+    </row>
+    <row r="11" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="103"/>
+      <c r="B11" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>202</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>203</v>
-      </c>
-      <c r="E12" s="20" t="s">
+      <c r="C11" s="105" t="s">
+        <v>238</v>
+      </c>
+      <c r="D11" s="106" t="s">
+        <v>239</v>
+      </c>
+      <c r="E11" s="107" t="s">
         <v>44</v>
       </c>
-      <c r="F12" s="20" t="s">
+      <c r="F11" s="107" t="s">
         <v>87</v>
       </c>
-      <c r="G12" s="21" t="s">
+      <c r="G11" s="104" t="s">
         <v>61</v>
       </c>
-      <c r="H12" s="30"/>
-    </row>
-    <row r="13" ht="45" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
-        <v>204</v>
-      </c>
-      <c r="B13" s="17" t="s">
+      <c r="H11" s="108"/>
+    </row>
+    <row r="12" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="103" t="s">
+        <v>240</v>
+      </c>
+      <c r="B12" s="104" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>205</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>206</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>207</v>
-      </c>
-      <c r="F13" s="20"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="30"/>
-    </row>
-    <row r="14" ht="45" customHeight="1" spans="1:8" s="75" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="27"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="98" t="s">
-        <v>208</v>
-      </c>
-      <c r="D14" s="99" t="s">
+      <c r="C12" s="105" t="s">
+        <v>241</v>
+      </c>
+      <c r="D12" s="106" t="s">
         <v>153</v>
       </c>
-      <c r="E14" s="100" t="s">
+      <c r="E12" s="107" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="100"/>
-      <c r="G14" s="79"/>
-      <c r="H14" s="101"/>
-    </row>
-    <row r="15" ht="30" customHeight="1" spans="1:8" s="75" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="27"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="98" t="s">
-        <v>209</v>
-      </c>
-      <c r="D15" s="99" t="s">
+      <c r="F12" s="107" t="s">
+        <v>231</v>
+      </c>
+      <c r="G12" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="H12" s="108"/>
+    </row>
+    <row r="13" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="103"/>
+      <c r="B13" s="104"/>
+      <c r="C13" s="105" t="s">
+        <v>242</v>
+      </c>
+      <c r="D13" s="106" t="s">
+        <v>243</v>
+      </c>
+      <c r="E13" s="107" t="s">
+        <v>244</v>
+      </c>
+      <c r="F13" s="107" t="s">
+        <v>231</v>
+      </c>
+      <c r="G13" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="H13" s="108"/>
+    </row>
+    <row r="14" ht="41" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="103"/>
+      <c r="B14" s="104"/>
+      <c r="C14" s="105" t="s">
+        <v>245</v>
+      </c>
+      <c r="D14" s="106" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="100" t="s">
-        <v>210</v>
-      </c>
-      <c r="F15" s="100"/>
-      <c r="G15" s="79"/>
-      <c r="H15" s="101"/>
-    </row>
-    <row r="16" ht="32.1" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="27"/>
-      <c r="B16" s="17" t="s">
+      <c r="E14" s="107" t="s">
+        <v>246</v>
+      </c>
+      <c r="F14" s="107" t="s">
+        <v>231</v>
+      </c>
+      <c r="G14" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="H14" s="108"/>
+    </row>
+    <row r="15" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="103"/>
+      <c r="B15" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="60" t="s">
-        <v>211</v>
-      </c>
-      <c r="D16" s="19" t="s">
+      <c r="C15" s="105" t="s">
+        <v>247</v>
+      </c>
+      <c r="D15" s="106" t="s">
         <v>174</v>
       </c>
-      <c r="E16" s="20" t="s">
+      <c r="E15" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="F15" s="107" t="s">
         <v>175</v>
       </c>
-      <c r="G16" s="24" t="s">
+      <c r="G15" s="104" t="s">
         <v>114</v>
       </c>
-      <c r="H16" s="30"/>
-    </row>
-    <row r="17" ht="30" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="29"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="18" t="s">
-        <v>212</v>
-      </c>
-      <c r="D17" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="E17" s="20" t="s">
+      <c r="H15" s="108"/>
+    </row>
+    <row r="16" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="103"/>
+      <c r="B16" s="104"/>
+      <c r="C16" s="105" t="s">
+        <v>248</v>
+      </c>
+      <c r="D16" s="106" t="s">
+        <v>249</v>
+      </c>
+      <c r="E16" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="20" t="s">
+      <c r="F16" s="107" t="s">
         <v>87</v>
       </c>
-      <c r="G17" s="21"/>
-      <c r="H17" s="30"/>
-    </row>
-    <row r="18" ht="20.1" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
-        <v>214</v>
-      </c>
-      <c r="B18" s="59" t="s">
+      <c r="G16" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="H16" s="108"/>
+    </row>
+    <row r="17" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="103" t="s">
+        <v>250</v>
+      </c>
+      <c r="B17" s="104" t="s">
         <v>13</v>
       </c>
-      <c r="C18" s="60" t="s">
-        <v>171</v>
-      </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="20" t="s">
+      <c r="C17" s="105" t="s">
+        <v>251</v>
+      </c>
+      <c r="D17" s="106"/>
+      <c r="E17" s="107" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F17" s="107" t="s">
         <v>24</v>
       </c>
-      <c r="G18" s="21"/>
-      <c r="H18" s="42"/>
-    </row>
-    <row r="19" ht="42.9" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="23"/>
-      <c r="B19" s="43"/>
-      <c r="C19" s="60" t="s">
-        <v>215</v>
-      </c>
-      <c r="D19" s="19" t="s">
-        <v>216</v>
-      </c>
-      <c r="E19" s="20" t="s">
+      <c r="G17" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="H17" s="108"/>
+    </row>
+    <row r="18" ht="72" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="103"/>
+      <c r="B18" s="104"/>
+      <c r="C18" s="105" t="s">
+        <v>252</v>
+      </c>
+      <c r="D18" s="106" t="s">
+        <v>253</v>
+      </c>
+      <c r="E18" s="107" t="s">
         <v>136</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="F18" s="107" t="s">
         <v>87</v>
       </c>
-      <c r="G19" s="21"/>
-      <c r="H19" s="42" t="s">
+      <c r="G18" s="104" t="s">
+        <v>231</v>
+      </c>
+      <c r="H18" s="108" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="20" ht="29.1" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="23"/>
-      <c r="B20" s="59" t="s">
+    <row r="19" ht="41" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="103"/>
+      <c r="B19" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="19" t="s">
-        <v>72</v>
-      </c>
-      <c r="D20" s="19" t="s">
+      <c r="C19" s="105" t="s">
+        <v>254</v>
+      </c>
+      <c r="D19" s="106" t="s">
         <v>73</v>
       </c>
-      <c r="E20" s="20" t="s">
+      <c r="E19" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="F20" s="20" t="s">
+      <c r="F19" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="G20" s="21" t="s">
+      <c r="G19" s="104" t="s">
         <v>49</v>
       </c>
-      <c r="H20" s="42"/>
-    </row>
-    <row r="21" ht="30" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="23"/>
-      <c r="B21" s="61"/>
-      <c r="C21" s="74" t="s">
-        <v>217</v>
-      </c>
-      <c r="D21" s="19" t="s">
+      <c r="H19" s="108"/>
+    </row>
+    <row r="20" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="103"/>
+      <c r="B20" s="104"/>
+      <c r="C20" s="105" t="s">
+        <v>255</v>
+      </c>
+      <c r="D20" s="106" t="s">
         <v>173</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E20" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="20" t="s">
+      <c r="F20" s="107" t="s">
         <v>181</v>
       </c>
-      <c r="G21" s="21" t="s">
+      <c r="G20" s="104" t="s">
         <v>61</v>
       </c>
-      <c r="H21" s="42"/>
-    </row>
-    <row r="22" ht="32.1" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="25"/>
-      <c r="B22" s="43"/>
-      <c r="C22" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="D22" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="E22" s="20" t="s">
+      <c r="H20" s="108"/>
+    </row>
+    <row r="21" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="103"/>
+      <c r="B21" s="104"/>
+      <c r="C21" s="105" t="s">
+        <v>256</v>
+      </c>
+      <c r="D21" s="106" t="s">
+        <v>257</v>
+      </c>
+      <c r="E21" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="F22" s="20" t="s">
+      <c r="F21" s="107" t="s">
         <v>17</v>
       </c>
-      <c r="G22" s="21" t="s">
+      <c r="G21" s="104" t="s">
         <v>61</v>
       </c>
-      <c r="H22" s="42"/>
-    </row>
-    <row r="23" ht="45" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16" t="s">
-        <v>220</v>
-      </c>
-      <c r="B23" s="38"/>
-      <c r="C23" s="19" t="s">
-        <v>221</v>
-      </c>
-      <c r="D23" s="19" t="s">
-        <v>222</v>
-      </c>
-      <c r="E23" s="20" t="s">
+      <c r="H21" s="108"/>
+    </row>
+    <row r="22" ht="56.5" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="103" t="s">
+        <v>258</v>
+      </c>
+      <c r="B22" s="104" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="105" t="s">
+        <v>259</v>
+      </c>
+      <c r="D22" s="106" t="s">
+        <v>260</v>
+      </c>
+      <c r="E22" s="107" t="s">
         <v>136</v>
       </c>
-      <c r="F23" s="20" t="s">
+      <c r="F22" s="107" t="s">
         <v>40</v>
       </c>
-      <c r="G23" s="21" t="s">
+      <c r="G22" s="104" t="s">
         <v>35</v>
       </c>
-      <c r="H23" s="42" t="s">
+      <c r="H22" s="108" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="24" ht="27.9" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="23"/>
-      <c r="B24" s="43" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>223</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>198</v>
-      </c>
-      <c r="E24" s="20" t="s">
+    <row r="23" ht="41" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="103"/>
+      <c r="B23" s="104"/>
+      <c r="C23" s="105" t="s">
+        <v>261</v>
+      </c>
+      <c r="D23" s="106" t="s">
+        <v>233</v>
+      </c>
+      <c r="E23" s="107" t="s">
         <v>23</v>
       </c>
-      <c r="F24" s="20" t="s">
+      <c r="F23" s="107" t="s">
         <v>24</v>
       </c>
-      <c r="G24" s="21" t="s">
+      <c r="G23" s="104" t="s">
         <v>78</v>
       </c>
-      <c r="H24" s="42" t="s">
+      <c r="H23" s="108" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="25" ht="27.9" customHeight="1" spans="1:8" s="75" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="25"/>
-      <c r="B25" s="88" t="s">
+    <row r="24" ht="41" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="103"/>
+      <c r="B24" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="C25" s="98" t="s">
-        <v>224</v>
-      </c>
-      <c r="D25" s="99" t="s">
-        <v>225</v>
-      </c>
-      <c r="E25" s="100" t="s">
+      <c r="C24" s="105" t="s">
+        <v>262</v>
+      </c>
+      <c r="D24" s="106" t="s">
+        <v>263</v>
+      </c>
+      <c r="E24" s="107" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="100" t="s">
+      <c r="F24" s="107" t="s">
         <v>24</v>
       </c>
-      <c r="G25" s="89" t="s">
+      <c r="G24" s="104" t="s">
         <v>78</v>
       </c>
-      <c r="H25" s="80" t="s">
+      <c r="H24" s="108" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26" ht="39.9" customHeight="1" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="37" t="s">
-        <v>226</v>
-      </c>
-      <c r="B26" s="38" t="s">
-        <v>20</v>
-      </c>
-      <c r="C26" s="32"/>
-      <c r="D26" s="58"/>
-      <c r="E26" s="102"/>
-      <c r="F26" s="102"/>
-      <c r="G26" s="21"/>
-      <c r="H26" s="42"/>
-    </row>
-    <row r="27" ht="39.9" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="49" t="s">
-        <v>227</v>
-      </c>
-      <c r="B27" s="50" t="s">
-        <v>13</v>
-      </c>
-      <c r="C27" s="103"/>
-      <c r="D27" s="104"/>
-      <c r="E27" s="105"/>
-      <c r="F27" s="105"/>
-      <c r="G27" s="106"/>
-      <c r="H27" s="107"/>
-    </row>
-    <row r="28" ht="15.75" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B28" s="1"/>
-      <c r="C28" s="56"/>
-      <c r="E28" s="1"/>
-      <c r="F28" s="1"/>
-      <c r="G28" s="1"/>
-      <c r="H28" s="1"/>
-    </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B29" s="1"/>
-      <c r="C29" s="56"/>
-      <c r="E29" s="1"/>
-      <c r="F29" s="1"/>
-      <c r="G29" s="1"/>
-      <c r="H29" s="1"/>
+    <row r="25" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="103" t="s">
+        <v>264</v>
+      </c>
+      <c r="B25" s="104"/>
+      <c r="C25" s="105"/>
+      <c r="D25" s="106"/>
+      <c r="E25" s="107"/>
+      <c r="F25" s="107"/>
+      <c r="G25" s="104"/>
+      <c r="H25" s="108"/>
+    </row>
+    <row r="26" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="114" t="s">
+        <v>265</v>
+      </c>
+      <c r="B26" s="115"/>
+      <c r="C26" s="116"/>
+      <c r="D26" s="117"/>
+      <c r="E26" s="118"/>
+      <c r="F26" s="118"/>
+      <c r="G26" s="115"/>
+      <c r="H26" s="119"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A17"/>
-    <mergeCell ref="B13:B15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="A18:A22"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A12:A16"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="B19:B21"/>
+    <mergeCell ref="A22:A24"/>
+    <mergeCell ref="B22:B23"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
-  <pageMargins left="0.25" right="0" top="0.5" bottom="0.25" header="0.3" footer="0.3"/>
+  <pageMargins left="0.2362204724409449" right="0" top="0.2362204724409449" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
@@ -7958,7 +7433,7 @@
     </row>
     <row r="5" ht="20.25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>228</v>
+        <v>194</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -7995,8 +7470,8 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="108" t="s">
-        <v>229</v>
+      <c r="A7" s="98" t="s">
+        <v>195</v>
       </c>
       <c r="B7" s="21"/>
       <c r="C7" s="68"/>
@@ -8007,8 +7482,8 @@
       <c r="H7" s="31"/>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="108" t="s">
-        <v>230</v>
+      <c r="A8" s="98" t="s">
+        <v>196</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="68"/>
@@ -8019,8 +7494,8 @@
       <c r="H8" s="31"/>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="108" t="s">
-        <v>231</v>
+      <c r="A9" s="98" t="s">
+        <v>197</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="68"/>
@@ -8031,8 +7506,8 @@
       <c r="H9" s="31"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="108" t="s">
-        <v>232</v>
+      <c r="A10" s="98" t="s">
+        <v>198</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="68"/>
@@ -8043,8 +7518,8 @@
       <c r="H10" s="31"/>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="108" t="s">
-        <v>233</v>
+      <c r="A11" s="98" t="s">
+        <v>199</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="68"/>
@@ -8055,8 +7530,8 @@
       <c r="H11" s="31"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="108" t="s">
-        <v>234</v>
+      <c r="A12" s="98" t="s">
+        <v>200</v>
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="68"/>
@@ -8067,48 +7542,48 @@
       <c r="H12" s="31"/>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="109" t="s">
-        <v>235</v>
-      </c>
-      <c r="B13" s="110" t="s">
+      <c r="A13" s="99" t="s">
+        <v>201</v>
+      </c>
+      <c r="B13" s="100" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="111" t="s">
-        <v>236</v>
-      </c>
-      <c r="D13" s="111" t="s">
-        <v>237</v>
-      </c>
-      <c r="E13" s="110" t="s">
+      <c r="C13" s="101" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" s="101" t="s">
+        <v>203</v>
+      </c>
+      <c r="E13" s="100" t="s">
         <v>23</v>
       </c>
-      <c r="F13" s="110" t="s">
-        <v>238</v>
-      </c>
-      <c r="G13" s="110" t="s">
-        <v>239</v>
-      </c>
-      <c r="H13" s="112"/>
+      <c r="F13" s="100" t="s">
+        <v>204</v>
+      </c>
+      <c r="G13" s="100" t="s">
+        <v>205</v>
+      </c>
+      <c r="H13" s="102"/>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="109"/>
-      <c r="B14" s="110"/>
-      <c r="C14" s="111" t="s">
-        <v>236</v>
-      </c>
-      <c r="D14" s="111" t="s">
-        <v>237</v>
-      </c>
-      <c r="E14" s="110" t="s">
+      <c r="A14" s="99"/>
+      <c r="B14" s="100"/>
+      <c r="C14" s="101" t="s">
+        <v>202</v>
+      </c>
+      <c r="D14" s="101" t="s">
+        <v>203</v>
+      </c>
+      <c r="E14" s="100" t="s">
         <v>23</v>
       </c>
-      <c r="F14" s="110" t="s">
-        <v>238</v>
-      </c>
-      <c r="G14" s="110" t="s">
-        <v>239</v>
-      </c>
-      <c r="H14" s="112"/>
+      <c r="F14" s="100" t="s">
+        <v>204</v>
+      </c>
+      <c r="G14" s="100" t="s">
+        <v>205</v>
+      </c>
+      <c r="H14" s="102"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -8741,7 +8216,7 @@
     </row>
     <row r="5" ht="20.25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>240</v>
+        <v>206</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -8778,8 +8253,8 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="108" t="s">
-        <v>241</v>
+      <c r="A7" s="98" t="s">
+        <v>207</v>
       </c>
       <c r="B7" s="21"/>
       <c r="C7" s="68"/>
@@ -8790,8 +8265,8 @@
       <c r="H7" s="31"/>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="108" t="s">
-        <v>242</v>
+      <c r="A8" s="98" t="s">
+        <v>208</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="68"/>
@@ -8802,8 +8277,8 @@
       <c r="H8" s="31"/>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="108" t="s">
-        <v>243</v>
+      <c r="A9" s="98" t="s">
+        <v>209</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="68"/>
@@ -8814,8 +8289,8 @@
       <c r="H9" s="31"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="108" t="s">
-        <v>244</v>
+      <c r="A10" s="98" t="s">
+        <v>210</v>
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="68"/>
@@ -8826,8 +8301,8 @@
       <c r="H10" s="31"/>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="108" t="s">
-        <v>245</v>
+      <c r="A11" s="98" t="s">
+        <v>211</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="68"/>
@@ -8838,8 +8313,8 @@
       <c r="H11" s="31"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="108" t="s">
-        <v>246</v>
+      <c r="A12" s="98" t="s">
+        <v>212</v>
       </c>
       <c r="B12" s="21"/>
       <c r="C12" s="68"/>
@@ -8850,8 +8325,8 @@
       <c r="H12" s="31"/>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="108" t="s">
-        <v>247</v>
+      <c r="A13" s="98" t="s">
+        <v>213</v>
       </c>
       <c r="B13" s="21"/>
       <c r="C13" s="68"/>
@@ -8876,585 +8351,17 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.33203125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="37.44140625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="41.109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="13.33203125" style="2" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="12.44140625" style="4" customWidth="1"/>
-    <col min="8" max="8" width="12.109375" style="5" customWidth="1"/>
-    <col min="9" max="256" width="9" style="1" customWidth="1"/>
-    <col min="257" max="257" width="9.33203125" style="1" customWidth="1"/>
-    <col min="258" max="258" width="6.33203125" style="1" customWidth="1"/>
-    <col min="259" max="259" width="47" style="1" customWidth="1"/>
-    <col min="260" max="260" width="43.33203125" style="1" customWidth="1"/>
-    <col min="261" max="261" width="13.33203125" style="1" customWidth="1"/>
-    <col min="262" max="262" width="10.6640625" style="1" customWidth="1"/>
-    <col min="263" max="263" width="12.44140625" style="1" customWidth="1"/>
-    <col min="264" max="264" width="12.109375" style="1" customWidth="1"/>
-    <col min="265" max="512" width="9" style="1" customWidth="1"/>
-    <col min="513" max="513" width="9.33203125" style="1" customWidth="1"/>
-    <col min="514" max="514" width="6.33203125" style="1" customWidth="1"/>
-    <col min="515" max="515" width="47" style="1" customWidth="1"/>
-    <col min="516" max="516" width="43.33203125" style="1" customWidth="1"/>
-    <col min="517" max="517" width="13.33203125" style="1" customWidth="1"/>
-    <col min="518" max="518" width="10.6640625" style="1" customWidth="1"/>
-    <col min="519" max="519" width="12.44140625" style="1" customWidth="1"/>
-    <col min="520" max="520" width="12.109375" style="1" customWidth="1"/>
-    <col min="521" max="768" width="9" style="1" customWidth="1"/>
-    <col min="769" max="769" width="9.33203125" style="1" customWidth="1"/>
-    <col min="770" max="770" width="6.33203125" style="1" customWidth="1"/>
-    <col min="771" max="771" width="47" style="1" customWidth="1"/>
-    <col min="772" max="772" width="43.33203125" style="1" customWidth="1"/>
-    <col min="773" max="773" width="13.33203125" style="1" customWidth="1"/>
-    <col min="774" max="774" width="10.6640625" style="1" customWidth="1"/>
-    <col min="775" max="775" width="12.44140625" style="1" customWidth="1"/>
-    <col min="776" max="776" width="12.109375" style="1" customWidth="1"/>
-    <col min="777" max="1024" width="9" style="1" customWidth="1"/>
-    <col min="1025" max="1025" width="9.33203125" style="1" customWidth="1"/>
-    <col min="1026" max="1026" width="6.33203125" style="1" customWidth="1"/>
-    <col min="1027" max="1027" width="47" style="1" customWidth="1"/>
-    <col min="1028" max="1028" width="43.33203125" style="1" customWidth="1"/>
-    <col min="1029" max="1029" width="13.33203125" style="1" customWidth="1"/>
-    <col min="1030" max="1030" width="10.6640625" style="1" customWidth="1"/>
-    <col min="1031" max="1031" width="12.44140625" style="1" customWidth="1"/>
-    <col min="1032" max="1032" width="12.109375" style="1" customWidth="1"/>
-    <col min="1033" max="1280" width="9" style="1" customWidth="1"/>
-    <col min="1281" max="1281" width="9.33203125" style="1" customWidth="1"/>
-    <col min="1282" max="1282" width="6.33203125" style="1" customWidth="1"/>
-    <col min="1283" max="1283" width="47" style="1" customWidth="1"/>
-    <col min="1284" max="1284" width="43.33203125" style="1" customWidth="1"/>
-    <col min="1285" max="1285" width="13.33203125" style="1" customWidth="1"/>
-    <col min="1286" max="1286" width="10.6640625" style="1" customWidth="1"/>
-    <col min="1287" max="1287" width="12.44140625" style="1" customWidth="1"/>
-    <col min="1288" max="1288" width="12.109375" style="1" customWidth="1"/>
-    <col min="1289" max="1536" width="9" style="1" customWidth="1"/>
-    <col min="1537" max="1537" width="9.33203125" style="1" customWidth="1"/>
-    <col min="1538" max="1538" width="6.33203125" style="1" customWidth="1"/>
-    <col min="1539" max="1539" width="47" style="1" customWidth="1"/>
-    <col min="1540" max="1540" width="43.33203125" style="1" customWidth="1"/>
-    <col min="1541" max="1541" width="13.33203125" style="1" customWidth="1"/>
-    <col min="1542" max="1542" width="10.6640625" style="1" customWidth="1"/>
-    <col min="1543" max="1543" width="12.44140625" style="1" customWidth="1"/>
-    <col min="1544" max="1544" width="12.109375" style="1" customWidth="1"/>
-    <col min="1545" max="1792" width="9" style="1" customWidth="1"/>
-    <col min="1793" max="1793" width="9.33203125" style="1" customWidth="1"/>
-    <col min="1794" max="1794" width="6.33203125" style="1" customWidth="1"/>
-    <col min="1795" max="1795" width="47" style="1" customWidth="1"/>
-    <col min="1796" max="1796" width="43.33203125" style="1" customWidth="1"/>
-    <col min="1797" max="1797" width="13.33203125" style="1" customWidth="1"/>
-    <col min="1798" max="1798" width="10.6640625" style="1" customWidth="1"/>
-    <col min="1799" max="1799" width="12.44140625" style="1" customWidth="1"/>
-    <col min="1800" max="1800" width="12.109375" style="1" customWidth="1"/>
-    <col min="1801" max="2048" width="9" style="1" customWidth="1"/>
-    <col min="2049" max="2049" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2050" max="2050" width="6.33203125" style="1" customWidth="1"/>
-    <col min="2051" max="2051" width="47" style="1" customWidth="1"/>
-    <col min="2052" max="2052" width="43.33203125" style="1" customWidth="1"/>
-    <col min="2053" max="2053" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2054" max="2054" width="10.6640625" style="1" customWidth="1"/>
-    <col min="2055" max="2055" width="12.44140625" style="1" customWidth="1"/>
-    <col min="2056" max="2056" width="12.109375" style="1" customWidth="1"/>
-    <col min="2057" max="2304" width="9" style="1" customWidth="1"/>
-    <col min="2305" max="2305" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2306" max="2306" width="6.33203125" style="1" customWidth="1"/>
-    <col min="2307" max="2307" width="47" style="1" customWidth="1"/>
-    <col min="2308" max="2308" width="43.33203125" style="1" customWidth="1"/>
-    <col min="2309" max="2309" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2310" max="2310" width="10.6640625" style="1" customWidth="1"/>
-    <col min="2311" max="2311" width="12.44140625" style="1" customWidth="1"/>
-    <col min="2312" max="2312" width="12.109375" style="1" customWidth="1"/>
-    <col min="2313" max="2560" width="9" style="1" customWidth="1"/>
-    <col min="2561" max="2561" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2562" max="2562" width="6.33203125" style="1" customWidth="1"/>
-    <col min="2563" max="2563" width="47" style="1" customWidth="1"/>
-    <col min="2564" max="2564" width="43.33203125" style="1" customWidth="1"/>
-    <col min="2565" max="2565" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2566" max="2566" width="10.6640625" style="1" customWidth="1"/>
-    <col min="2567" max="2567" width="12.44140625" style="1" customWidth="1"/>
-    <col min="2568" max="2568" width="12.109375" style="1" customWidth="1"/>
-    <col min="2569" max="2816" width="9" style="1" customWidth="1"/>
-    <col min="2817" max="2817" width="9.33203125" style="1" customWidth="1"/>
-    <col min="2818" max="2818" width="6.33203125" style="1" customWidth="1"/>
-    <col min="2819" max="2819" width="47" style="1" customWidth="1"/>
-    <col min="2820" max="2820" width="43.33203125" style="1" customWidth="1"/>
-    <col min="2821" max="2821" width="13.33203125" style="1" customWidth="1"/>
-    <col min="2822" max="2822" width="10.6640625" style="1" customWidth="1"/>
-    <col min="2823" max="2823" width="12.44140625" style="1" customWidth="1"/>
-    <col min="2824" max="2824" width="12.109375" style="1" customWidth="1"/>
-    <col min="2825" max="3072" width="9" style="1" customWidth="1"/>
-    <col min="3073" max="3073" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3074" max="3074" width="6.33203125" style="1" customWidth="1"/>
-    <col min="3075" max="3075" width="47" style="1" customWidth="1"/>
-    <col min="3076" max="3076" width="43.33203125" style="1" customWidth="1"/>
-    <col min="3077" max="3077" width="13.33203125" style="1" customWidth="1"/>
-    <col min="3078" max="3078" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3079" max="3079" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3080" max="3080" width="12.109375" style="1" customWidth="1"/>
-    <col min="3081" max="3328" width="9" style="1" customWidth="1"/>
-    <col min="3329" max="3329" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3330" max="3330" width="6.33203125" style="1" customWidth="1"/>
-    <col min="3331" max="3331" width="47" style="1" customWidth="1"/>
-    <col min="3332" max="3332" width="43.33203125" style="1" customWidth="1"/>
-    <col min="3333" max="3333" width="13.33203125" style="1" customWidth="1"/>
-    <col min="3334" max="3334" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3335" max="3335" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3336" max="3336" width="12.109375" style="1" customWidth="1"/>
-    <col min="3337" max="3584" width="9" style="1" customWidth="1"/>
-    <col min="3585" max="3585" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3586" max="3586" width="6.33203125" style="1" customWidth="1"/>
-    <col min="3587" max="3587" width="47" style="1" customWidth="1"/>
-    <col min="3588" max="3588" width="43.33203125" style="1" customWidth="1"/>
-    <col min="3589" max="3589" width="13.33203125" style="1" customWidth="1"/>
-    <col min="3590" max="3590" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3591" max="3591" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3592" max="3592" width="12.109375" style="1" customWidth="1"/>
-    <col min="3593" max="3840" width="9" style="1" customWidth="1"/>
-    <col min="3841" max="3841" width="9.33203125" style="1" customWidth="1"/>
-    <col min="3842" max="3842" width="6.33203125" style="1" customWidth="1"/>
-    <col min="3843" max="3843" width="47" style="1" customWidth="1"/>
-    <col min="3844" max="3844" width="43.33203125" style="1" customWidth="1"/>
-    <col min="3845" max="3845" width="13.33203125" style="1" customWidth="1"/>
-    <col min="3846" max="3846" width="10.6640625" style="1" customWidth="1"/>
-    <col min="3847" max="3847" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3848" max="3848" width="12.109375" style="1" customWidth="1"/>
-    <col min="3849" max="4096" width="9" style="1" customWidth="1"/>
-    <col min="4097" max="4097" width="9.33203125" style="1" customWidth="1"/>
-    <col min="4098" max="4098" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4099" max="4099" width="47" style="1" customWidth="1"/>
-    <col min="4100" max="4100" width="43.33203125" style="1" customWidth="1"/>
-    <col min="4101" max="4101" width="13.33203125" style="1" customWidth="1"/>
-    <col min="4102" max="4102" width="10.6640625" style="1" customWidth="1"/>
-    <col min="4103" max="4103" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4104" max="4104" width="12.109375" style="1" customWidth="1"/>
-    <col min="4105" max="4352" width="9" style="1" customWidth="1"/>
-    <col min="4353" max="4353" width="9.33203125" style="1" customWidth="1"/>
-    <col min="4354" max="4354" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4355" max="4355" width="47" style="1" customWidth="1"/>
-    <col min="4356" max="4356" width="43.33203125" style="1" customWidth="1"/>
-    <col min="4357" max="4357" width="13.33203125" style="1" customWidth="1"/>
-    <col min="4358" max="4358" width="10.6640625" style="1" customWidth="1"/>
-    <col min="4359" max="4359" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4360" max="4360" width="12.109375" style="1" customWidth="1"/>
-    <col min="4361" max="4608" width="9" style="1" customWidth="1"/>
-    <col min="4609" max="4609" width="9.33203125" style="1" customWidth="1"/>
-    <col min="4610" max="4610" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4611" max="4611" width="47" style="1" customWidth="1"/>
-    <col min="4612" max="4612" width="43.33203125" style="1" customWidth="1"/>
-    <col min="4613" max="4613" width="13.33203125" style="1" customWidth="1"/>
-    <col min="4614" max="4614" width="10.6640625" style="1" customWidth="1"/>
-    <col min="4615" max="4615" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4616" max="4616" width="12.109375" style="1" customWidth="1"/>
-    <col min="4617" max="4864" width="9" style="1" customWidth="1"/>
-    <col min="4865" max="4865" width="9.33203125" style="1" customWidth="1"/>
-    <col min="4866" max="4866" width="6.33203125" style="1" customWidth="1"/>
-    <col min="4867" max="4867" width="47" style="1" customWidth="1"/>
-    <col min="4868" max="4868" width="43.33203125" style="1" customWidth="1"/>
-    <col min="4869" max="4869" width="13.33203125" style="1" customWidth="1"/>
-    <col min="4870" max="4870" width="10.6640625" style="1" customWidth="1"/>
-    <col min="4871" max="4871" width="12.44140625" style="1" customWidth="1"/>
-    <col min="4872" max="4872" width="12.109375" style="1" customWidth="1"/>
-    <col min="4873" max="5120" width="9" style="1" customWidth="1"/>
-    <col min="5121" max="5121" width="9.33203125" style="1" customWidth="1"/>
-    <col min="5122" max="5122" width="6.33203125" style="1" customWidth="1"/>
-    <col min="5123" max="5123" width="47" style="1" customWidth="1"/>
-    <col min="5124" max="5124" width="43.33203125" style="1" customWidth="1"/>
-    <col min="5125" max="5125" width="13.33203125" style="1" customWidth="1"/>
-    <col min="5126" max="5126" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5127" max="5127" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5128" max="5128" width="12.109375" style="1" customWidth="1"/>
-    <col min="5129" max="5376" width="9" style="1" customWidth="1"/>
-    <col min="5377" max="5377" width="9.33203125" style="1" customWidth="1"/>
-    <col min="5378" max="5378" width="6.33203125" style="1" customWidth="1"/>
-    <col min="5379" max="5379" width="47" style="1" customWidth="1"/>
-    <col min="5380" max="5380" width="43.33203125" style="1" customWidth="1"/>
-    <col min="5381" max="5381" width="13.33203125" style="1" customWidth="1"/>
-    <col min="5382" max="5382" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5383" max="5383" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5384" max="5384" width="12.109375" style="1" customWidth="1"/>
-    <col min="5385" max="5632" width="9" style="1" customWidth="1"/>
-    <col min="5633" max="5633" width="9.33203125" style="1" customWidth="1"/>
-    <col min="5634" max="5634" width="6.33203125" style="1" customWidth="1"/>
-    <col min="5635" max="5635" width="47" style="1" customWidth="1"/>
-    <col min="5636" max="5636" width="43.33203125" style="1" customWidth="1"/>
-    <col min="5637" max="5637" width="13.33203125" style="1" customWidth="1"/>
-    <col min="5638" max="5638" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5639" max="5639" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5640" max="5640" width="12.109375" style="1" customWidth="1"/>
-    <col min="5641" max="5888" width="9" style="1" customWidth="1"/>
-    <col min="5889" max="5889" width="9.33203125" style="1" customWidth="1"/>
-    <col min="5890" max="5890" width="6.33203125" style="1" customWidth="1"/>
-    <col min="5891" max="5891" width="47" style="1" customWidth="1"/>
-    <col min="5892" max="5892" width="43.33203125" style="1" customWidth="1"/>
-    <col min="5893" max="5893" width="13.33203125" style="1" customWidth="1"/>
-    <col min="5894" max="5894" width="10.6640625" style="1" customWidth="1"/>
-    <col min="5895" max="5895" width="12.44140625" style="1" customWidth="1"/>
-    <col min="5896" max="5896" width="12.109375" style="1" customWidth="1"/>
-    <col min="5897" max="6144" width="9" style="1" customWidth="1"/>
-    <col min="6145" max="6145" width="9.33203125" style="1" customWidth="1"/>
-    <col min="6146" max="6146" width="6.33203125" style="1" customWidth="1"/>
-    <col min="6147" max="6147" width="47" style="1" customWidth="1"/>
-    <col min="6148" max="6148" width="43.33203125" style="1" customWidth="1"/>
-    <col min="6149" max="6149" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6150" max="6150" width="10.6640625" style="1" customWidth="1"/>
-    <col min="6151" max="6151" width="12.44140625" style="1" customWidth="1"/>
-    <col min="6152" max="6152" width="12.109375" style="1" customWidth="1"/>
-    <col min="6153" max="6400" width="9" style="1" customWidth="1"/>
-    <col min="6401" max="6401" width="9.33203125" style="1" customWidth="1"/>
-    <col min="6402" max="6402" width="6.33203125" style="1" customWidth="1"/>
-    <col min="6403" max="6403" width="47" style="1" customWidth="1"/>
-    <col min="6404" max="6404" width="43.33203125" style="1" customWidth="1"/>
-    <col min="6405" max="6405" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6406" max="6406" width="10.6640625" style="1" customWidth="1"/>
-    <col min="6407" max="6407" width="12.44140625" style="1" customWidth="1"/>
-    <col min="6408" max="6408" width="12.109375" style="1" customWidth="1"/>
-    <col min="6409" max="6656" width="9" style="1" customWidth="1"/>
-    <col min="6657" max="6657" width="9.33203125" style="1" customWidth="1"/>
-    <col min="6658" max="6658" width="6.33203125" style="1" customWidth="1"/>
-    <col min="6659" max="6659" width="47" style="1" customWidth="1"/>
-    <col min="6660" max="6660" width="43.33203125" style="1" customWidth="1"/>
-    <col min="6661" max="6661" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6662" max="6662" width="10.6640625" style="1" customWidth="1"/>
-    <col min="6663" max="6663" width="12.44140625" style="1" customWidth="1"/>
-    <col min="6664" max="6664" width="12.109375" style="1" customWidth="1"/>
-    <col min="6665" max="6912" width="9" style="1" customWidth="1"/>
-    <col min="6913" max="6913" width="9.33203125" style="1" customWidth="1"/>
-    <col min="6914" max="6914" width="6.33203125" style="1" customWidth="1"/>
-    <col min="6915" max="6915" width="47" style="1" customWidth="1"/>
-    <col min="6916" max="6916" width="43.33203125" style="1" customWidth="1"/>
-    <col min="6917" max="6917" width="13.33203125" style="1" customWidth="1"/>
-    <col min="6918" max="6918" width="10.6640625" style="1" customWidth="1"/>
-    <col min="6919" max="6919" width="12.44140625" style="1" customWidth="1"/>
-    <col min="6920" max="6920" width="12.109375" style="1" customWidth="1"/>
-    <col min="6921" max="7168" width="9" style="1" customWidth="1"/>
-    <col min="7169" max="7169" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7170" max="7170" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7171" max="7171" width="47" style="1" customWidth="1"/>
-    <col min="7172" max="7172" width="43.33203125" style="1" customWidth="1"/>
-    <col min="7173" max="7173" width="13.33203125" style="1" customWidth="1"/>
-    <col min="7174" max="7174" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7175" max="7175" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7176" max="7176" width="12.109375" style="1" customWidth="1"/>
-    <col min="7177" max="7424" width="9" style="1" customWidth="1"/>
-    <col min="7425" max="7425" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7426" max="7426" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7427" max="7427" width="47" style="1" customWidth="1"/>
-    <col min="7428" max="7428" width="43.33203125" style="1" customWidth="1"/>
-    <col min="7429" max="7429" width="13.33203125" style="1" customWidth="1"/>
-    <col min="7430" max="7430" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7431" max="7431" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7432" max="7432" width="12.109375" style="1" customWidth="1"/>
-    <col min="7433" max="7680" width="9" style="1" customWidth="1"/>
-    <col min="7681" max="7681" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7682" max="7682" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7683" max="7683" width="47" style="1" customWidth="1"/>
-    <col min="7684" max="7684" width="43.33203125" style="1" customWidth="1"/>
-    <col min="7685" max="7685" width="13.33203125" style="1" customWidth="1"/>
-    <col min="7686" max="7686" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7687" max="7687" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7688" max="7688" width="12.109375" style="1" customWidth="1"/>
-    <col min="7689" max="7936" width="9" style="1" customWidth="1"/>
-    <col min="7937" max="7937" width="9.33203125" style="1" customWidth="1"/>
-    <col min="7938" max="7938" width="6.33203125" style="1" customWidth="1"/>
-    <col min="7939" max="7939" width="47" style="1" customWidth="1"/>
-    <col min="7940" max="7940" width="43.33203125" style="1" customWidth="1"/>
-    <col min="7941" max="7941" width="13.33203125" style="1" customWidth="1"/>
-    <col min="7942" max="7942" width="10.6640625" style="1" customWidth="1"/>
-    <col min="7943" max="7943" width="12.44140625" style="1" customWidth="1"/>
-    <col min="7944" max="7944" width="12.109375" style="1" customWidth="1"/>
-    <col min="7945" max="8192" width="9" style="1" customWidth="1"/>
-    <col min="8193" max="8193" width="9.33203125" style="1" customWidth="1"/>
-    <col min="8194" max="8194" width="6.33203125" style="1" customWidth="1"/>
-    <col min="8195" max="8195" width="47" style="1" customWidth="1"/>
-    <col min="8196" max="8196" width="43.33203125" style="1" customWidth="1"/>
-    <col min="8197" max="8197" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8198" max="8198" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8199" max="8199" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8200" max="8200" width="12.109375" style="1" customWidth="1"/>
-    <col min="8201" max="8448" width="9" style="1" customWidth="1"/>
-    <col min="8449" max="8449" width="9.33203125" style="1" customWidth="1"/>
-    <col min="8450" max="8450" width="6.33203125" style="1" customWidth="1"/>
-    <col min="8451" max="8451" width="47" style="1" customWidth="1"/>
-    <col min="8452" max="8452" width="43.33203125" style="1" customWidth="1"/>
-    <col min="8453" max="8453" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8454" max="8454" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8455" max="8455" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8456" max="8456" width="12.109375" style="1" customWidth="1"/>
-    <col min="8457" max="8704" width="9" style="1" customWidth="1"/>
-    <col min="8705" max="8705" width="9.33203125" style="1" customWidth="1"/>
-    <col min="8706" max="8706" width="6.33203125" style="1" customWidth="1"/>
-    <col min="8707" max="8707" width="47" style="1" customWidth="1"/>
-    <col min="8708" max="8708" width="43.33203125" style="1" customWidth="1"/>
-    <col min="8709" max="8709" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8710" max="8710" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8711" max="8711" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8712" max="8712" width="12.109375" style="1" customWidth="1"/>
-    <col min="8713" max="8960" width="9" style="1" customWidth="1"/>
-    <col min="8961" max="8961" width="9.33203125" style="1" customWidth="1"/>
-    <col min="8962" max="8962" width="6.33203125" style="1" customWidth="1"/>
-    <col min="8963" max="8963" width="47" style="1" customWidth="1"/>
-    <col min="8964" max="8964" width="43.33203125" style="1" customWidth="1"/>
-    <col min="8965" max="8965" width="13.33203125" style="1" customWidth="1"/>
-    <col min="8966" max="8966" width="10.6640625" style="1" customWidth="1"/>
-    <col min="8967" max="8967" width="12.44140625" style="1" customWidth="1"/>
-    <col min="8968" max="8968" width="12.109375" style="1" customWidth="1"/>
-    <col min="8969" max="9216" width="9" style="1" customWidth="1"/>
-    <col min="9217" max="9217" width="9.33203125" style="1" customWidth="1"/>
-    <col min="9218" max="9218" width="6.33203125" style="1" customWidth="1"/>
-    <col min="9219" max="9219" width="47" style="1" customWidth="1"/>
-    <col min="9220" max="9220" width="43.33203125" style="1" customWidth="1"/>
-    <col min="9221" max="9221" width="13.33203125" style="1" customWidth="1"/>
-    <col min="9222" max="9222" width="10.6640625" style="1" customWidth="1"/>
-    <col min="9223" max="9223" width="12.44140625" style="1" customWidth="1"/>
-    <col min="9224" max="9224" width="12.109375" style="1" customWidth="1"/>
-    <col min="9225" max="9472" width="9" style="1" customWidth="1"/>
-    <col min="9473" max="9473" width="9.33203125" style="1" customWidth="1"/>
-    <col min="9474" max="9474" width="6.33203125" style="1" customWidth="1"/>
-    <col min="9475" max="9475" width="47" style="1" customWidth="1"/>
-    <col min="9476" max="9476" width="43.33203125" style="1" customWidth="1"/>
-    <col min="9477" max="9477" width="13.33203125" style="1" customWidth="1"/>
-    <col min="9478" max="9478" width="10.6640625" style="1" customWidth="1"/>
-    <col min="9479" max="9479" width="12.44140625" style="1" customWidth="1"/>
-    <col min="9480" max="9480" width="12.109375" style="1" customWidth="1"/>
-    <col min="9481" max="9728" width="9" style="1" customWidth="1"/>
-    <col min="9729" max="9729" width="9.33203125" style="1" customWidth="1"/>
-    <col min="9730" max="9730" width="6.33203125" style="1" customWidth="1"/>
-    <col min="9731" max="9731" width="47" style="1" customWidth="1"/>
-    <col min="9732" max="9732" width="43.33203125" style="1" customWidth="1"/>
-    <col min="9733" max="9733" width="13.33203125" style="1" customWidth="1"/>
-    <col min="9734" max="9734" width="10.6640625" style="1" customWidth="1"/>
-    <col min="9735" max="9735" width="12.44140625" style="1" customWidth="1"/>
-    <col min="9736" max="9736" width="12.109375" style="1" customWidth="1"/>
-    <col min="9737" max="9984" width="9" style="1" customWidth="1"/>
-    <col min="9985" max="9985" width="9.33203125" style="1" customWidth="1"/>
-    <col min="9986" max="9986" width="6.33203125" style="1" customWidth="1"/>
-    <col min="9987" max="9987" width="47" style="1" customWidth="1"/>
-    <col min="9988" max="9988" width="43.33203125" style="1" customWidth="1"/>
-    <col min="9989" max="9989" width="13.33203125" style="1" customWidth="1"/>
-    <col min="9990" max="9990" width="10.6640625" style="1" customWidth="1"/>
-    <col min="9991" max="9991" width="12.44140625" style="1" customWidth="1"/>
-    <col min="9992" max="9992" width="12.109375" style="1" customWidth="1"/>
-    <col min="9993" max="10240" width="9" style="1" customWidth="1"/>
-    <col min="10241" max="10241" width="9.33203125" style="1" customWidth="1"/>
-    <col min="10242" max="10242" width="6.33203125" style="1" customWidth="1"/>
-    <col min="10243" max="10243" width="47" style="1" customWidth="1"/>
-    <col min="10244" max="10244" width="43.33203125" style="1" customWidth="1"/>
-    <col min="10245" max="10245" width="13.33203125" style="1" customWidth="1"/>
-    <col min="10246" max="10246" width="10.6640625" style="1" customWidth="1"/>
-    <col min="10247" max="10247" width="12.44140625" style="1" customWidth="1"/>
-    <col min="10248" max="10248" width="12.109375" style="1" customWidth="1"/>
-    <col min="10249" max="10496" width="9" style="1" customWidth="1"/>
-    <col min="10497" max="10497" width="9.33203125" style="1" customWidth="1"/>
-    <col min="10498" max="10498" width="6.33203125" style="1" customWidth="1"/>
-    <col min="10499" max="10499" width="47" style="1" customWidth="1"/>
-    <col min="10500" max="10500" width="43.33203125" style="1" customWidth="1"/>
-    <col min="10501" max="10501" width="13.33203125" style="1" customWidth="1"/>
-    <col min="10502" max="10502" width="10.6640625" style="1" customWidth="1"/>
-    <col min="10503" max="10503" width="12.44140625" style="1" customWidth="1"/>
-    <col min="10504" max="10504" width="12.109375" style="1" customWidth="1"/>
-    <col min="10505" max="10752" width="9" style="1" customWidth="1"/>
-    <col min="10753" max="10753" width="9.33203125" style="1" customWidth="1"/>
-    <col min="10754" max="10754" width="6.33203125" style="1" customWidth="1"/>
-    <col min="10755" max="10755" width="47" style="1" customWidth="1"/>
-    <col min="10756" max="10756" width="43.33203125" style="1" customWidth="1"/>
-    <col min="10757" max="10757" width="13.33203125" style="1" customWidth="1"/>
-    <col min="10758" max="10758" width="10.6640625" style="1" customWidth="1"/>
-    <col min="10759" max="10759" width="12.44140625" style="1" customWidth="1"/>
-    <col min="10760" max="10760" width="12.109375" style="1" customWidth="1"/>
-    <col min="10761" max="11008" width="9" style="1" customWidth="1"/>
-    <col min="11009" max="11009" width="9.33203125" style="1" customWidth="1"/>
-    <col min="11010" max="11010" width="6.33203125" style="1" customWidth="1"/>
-    <col min="11011" max="11011" width="47" style="1" customWidth="1"/>
-    <col min="11012" max="11012" width="43.33203125" style="1" customWidth="1"/>
-    <col min="11013" max="11013" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11014" max="11014" width="10.6640625" style="1" customWidth="1"/>
-    <col min="11015" max="11015" width="12.44140625" style="1" customWidth="1"/>
-    <col min="11016" max="11016" width="12.109375" style="1" customWidth="1"/>
-    <col min="11017" max="11264" width="9" style="1" customWidth="1"/>
-    <col min="11265" max="11265" width="9.33203125" style="1" customWidth="1"/>
-    <col min="11266" max="11266" width="6.33203125" style="1" customWidth="1"/>
-    <col min="11267" max="11267" width="47" style="1" customWidth="1"/>
-    <col min="11268" max="11268" width="43.33203125" style="1" customWidth="1"/>
-    <col min="11269" max="11269" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11270" max="11270" width="10.6640625" style="1" customWidth="1"/>
-    <col min="11271" max="11271" width="12.44140625" style="1" customWidth="1"/>
-    <col min="11272" max="11272" width="12.109375" style="1" customWidth="1"/>
-    <col min="11273" max="11520" width="9" style="1" customWidth="1"/>
-    <col min="11521" max="11521" width="9.33203125" style="1" customWidth="1"/>
-    <col min="11522" max="11522" width="6.33203125" style="1" customWidth="1"/>
-    <col min="11523" max="11523" width="47" style="1" customWidth="1"/>
-    <col min="11524" max="11524" width="43.33203125" style="1" customWidth="1"/>
-    <col min="11525" max="11525" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11526" max="11526" width="10.6640625" style="1" customWidth="1"/>
-    <col min="11527" max="11527" width="12.44140625" style="1" customWidth="1"/>
-    <col min="11528" max="11528" width="12.109375" style="1" customWidth="1"/>
-    <col min="11529" max="11776" width="9" style="1" customWidth="1"/>
-    <col min="11777" max="11777" width="9.33203125" style="1" customWidth="1"/>
-    <col min="11778" max="11778" width="6.33203125" style="1" customWidth="1"/>
-    <col min="11779" max="11779" width="47" style="1" customWidth="1"/>
-    <col min="11780" max="11780" width="43.33203125" style="1" customWidth="1"/>
-    <col min="11781" max="11781" width="13.33203125" style="1" customWidth="1"/>
-    <col min="11782" max="11782" width="10.6640625" style="1" customWidth="1"/>
-    <col min="11783" max="11783" width="12.44140625" style="1" customWidth="1"/>
-    <col min="11784" max="11784" width="12.109375" style="1" customWidth="1"/>
-    <col min="11785" max="12032" width="9" style="1" customWidth="1"/>
-    <col min="12033" max="12033" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12034" max="12034" width="6.33203125" style="1" customWidth="1"/>
-    <col min="12035" max="12035" width="47" style="1" customWidth="1"/>
-    <col min="12036" max="12036" width="43.33203125" style="1" customWidth="1"/>
-    <col min="12037" max="12037" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12038" max="12038" width="10.6640625" style="1" customWidth="1"/>
-    <col min="12039" max="12039" width="12.44140625" style="1" customWidth="1"/>
-    <col min="12040" max="12040" width="12.109375" style="1" customWidth="1"/>
-    <col min="12041" max="12288" width="9" style="1" customWidth="1"/>
-    <col min="12289" max="12289" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12290" max="12290" width="6.33203125" style="1" customWidth="1"/>
-    <col min="12291" max="12291" width="47" style="1" customWidth="1"/>
-    <col min="12292" max="12292" width="43.33203125" style="1" customWidth="1"/>
-    <col min="12293" max="12293" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12294" max="12294" width="10.6640625" style="1" customWidth="1"/>
-    <col min="12295" max="12295" width="12.44140625" style="1" customWidth="1"/>
-    <col min="12296" max="12296" width="12.109375" style="1" customWidth="1"/>
-    <col min="12297" max="12544" width="9" style="1" customWidth="1"/>
-    <col min="12545" max="12545" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12546" max="12546" width="6.33203125" style="1" customWidth="1"/>
-    <col min="12547" max="12547" width="47" style="1" customWidth="1"/>
-    <col min="12548" max="12548" width="43.33203125" style="1" customWidth="1"/>
-    <col min="12549" max="12549" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12550" max="12550" width="10.6640625" style="1" customWidth="1"/>
-    <col min="12551" max="12551" width="12.44140625" style="1" customWidth="1"/>
-    <col min="12552" max="12552" width="12.109375" style="1" customWidth="1"/>
-    <col min="12553" max="12800" width="9" style="1" customWidth="1"/>
-    <col min="12801" max="12801" width="9.33203125" style="1" customWidth="1"/>
-    <col min="12802" max="12802" width="6.33203125" style="1" customWidth="1"/>
-    <col min="12803" max="12803" width="47" style="1" customWidth="1"/>
-    <col min="12804" max="12804" width="43.33203125" style="1" customWidth="1"/>
-    <col min="12805" max="12805" width="13.33203125" style="1" customWidth="1"/>
-    <col min="12806" max="12806" width="10.6640625" style="1" customWidth="1"/>
-    <col min="12807" max="12807" width="12.44140625" style="1" customWidth="1"/>
-    <col min="12808" max="12808" width="12.109375" style="1" customWidth="1"/>
-    <col min="12809" max="13056" width="9" style="1" customWidth="1"/>
-    <col min="13057" max="13057" width="9.33203125" style="1" customWidth="1"/>
-    <col min="13058" max="13058" width="6.33203125" style="1" customWidth="1"/>
-    <col min="13059" max="13059" width="47" style="1" customWidth="1"/>
-    <col min="13060" max="13060" width="43.33203125" style="1" customWidth="1"/>
-    <col min="13061" max="13061" width="13.33203125" style="1" customWidth="1"/>
-    <col min="13062" max="13062" width="10.6640625" style="1" customWidth="1"/>
-    <col min="13063" max="13063" width="12.44140625" style="1" customWidth="1"/>
-    <col min="13064" max="13064" width="12.109375" style="1" customWidth="1"/>
-    <col min="13065" max="13312" width="9" style="1" customWidth="1"/>
-    <col min="13313" max="13313" width="9.33203125" style="1" customWidth="1"/>
-    <col min="13314" max="13314" width="6.33203125" style="1" customWidth="1"/>
-    <col min="13315" max="13315" width="47" style="1" customWidth="1"/>
-    <col min="13316" max="13316" width="43.33203125" style="1" customWidth="1"/>
-    <col min="13317" max="13317" width="13.33203125" style="1" customWidth="1"/>
-    <col min="13318" max="13318" width="10.6640625" style="1" customWidth="1"/>
-    <col min="13319" max="13319" width="12.44140625" style="1" customWidth="1"/>
-    <col min="13320" max="13320" width="12.109375" style="1" customWidth="1"/>
-    <col min="13321" max="13568" width="9" style="1" customWidth="1"/>
-    <col min="13569" max="13569" width="9.33203125" style="1" customWidth="1"/>
-    <col min="13570" max="13570" width="6.33203125" style="1" customWidth="1"/>
-    <col min="13571" max="13571" width="47" style="1" customWidth="1"/>
-    <col min="13572" max="13572" width="43.33203125" style="1" customWidth="1"/>
-    <col min="13573" max="13573" width="13.33203125" style="1" customWidth="1"/>
-    <col min="13574" max="13574" width="10.6640625" style="1" customWidth="1"/>
-    <col min="13575" max="13575" width="12.44140625" style="1" customWidth="1"/>
-    <col min="13576" max="13576" width="12.109375" style="1" customWidth="1"/>
-    <col min="13577" max="13824" width="9" style="1" customWidth="1"/>
-    <col min="13825" max="13825" width="9.33203125" style="1" customWidth="1"/>
-    <col min="13826" max="13826" width="6.33203125" style="1" customWidth="1"/>
-    <col min="13827" max="13827" width="47" style="1" customWidth="1"/>
-    <col min="13828" max="13828" width="43.33203125" style="1" customWidth="1"/>
-    <col min="13829" max="13829" width="13.33203125" style="1" customWidth="1"/>
-    <col min="13830" max="13830" width="10.6640625" style="1" customWidth="1"/>
-    <col min="13831" max="13831" width="12.44140625" style="1" customWidth="1"/>
-    <col min="13832" max="13832" width="12.109375" style="1" customWidth="1"/>
-    <col min="13833" max="14080" width="9" style="1" customWidth="1"/>
-    <col min="14081" max="14081" width="9.33203125" style="1" customWidth="1"/>
-    <col min="14082" max="14082" width="6.33203125" style="1" customWidth="1"/>
-    <col min="14083" max="14083" width="47" style="1" customWidth="1"/>
-    <col min="14084" max="14084" width="43.33203125" style="1" customWidth="1"/>
-    <col min="14085" max="14085" width="13.33203125" style="1" customWidth="1"/>
-    <col min="14086" max="14086" width="10.6640625" style="1" customWidth="1"/>
-    <col min="14087" max="14087" width="12.44140625" style="1" customWidth="1"/>
-    <col min="14088" max="14088" width="12.109375" style="1" customWidth="1"/>
-    <col min="14089" max="14336" width="9" style="1" customWidth="1"/>
-    <col min="14337" max="14337" width="9.33203125" style="1" customWidth="1"/>
-    <col min="14338" max="14338" width="6.33203125" style="1" customWidth="1"/>
-    <col min="14339" max="14339" width="47" style="1" customWidth="1"/>
-    <col min="14340" max="14340" width="43.33203125" style="1" customWidth="1"/>
-    <col min="14341" max="14341" width="13.33203125" style="1" customWidth="1"/>
-    <col min="14342" max="14342" width="10.6640625" style="1" customWidth="1"/>
-    <col min="14343" max="14343" width="12.44140625" style="1" customWidth="1"/>
-    <col min="14344" max="14344" width="12.109375" style="1" customWidth="1"/>
-    <col min="14345" max="14592" width="9" style="1" customWidth="1"/>
-    <col min="14593" max="14593" width="9.33203125" style="1" customWidth="1"/>
-    <col min="14594" max="14594" width="6.33203125" style="1" customWidth="1"/>
-    <col min="14595" max="14595" width="47" style="1" customWidth="1"/>
-    <col min="14596" max="14596" width="43.33203125" style="1" customWidth="1"/>
-    <col min="14597" max="14597" width="13.33203125" style="1" customWidth="1"/>
-    <col min="14598" max="14598" width="10.6640625" style="1" customWidth="1"/>
-    <col min="14599" max="14599" width="12.44140625" style="1" customWidth="1"/>
-    <col min="14600" max="14600" width="12.109375" style="1" customWidth="1"/>
-    <col min="14601" max="14848" width="9" style="1" customWidth="1"/>
-    <col min="14849" max="14849" width="9.33203125" style="1" customWidth="1"/>
-    <col min="14850" max="14850" width="6.33203125" style="1" customWidth="1"/>
-    <col min="14851" max="14851" width="47" style="1" customWidth="1"/>
-    <col min="14852" max="14852" width="43.33203125" style="1" customWidth="1"/>
-    <col min="14853" max="14853" width="13.33203125" style="1" customWidth="1"/>
-    <col min="14854" max="14854" width="10.6640625" style="1" customWidth="1"/>
-    <col min="14855" max="14855" width="12.44140625" style="1" customWidth="1"/>
-    <col min="14856" max="14856" width="12.109375" style="1" customWidth="1"/>
-    <col min="14857" max="15104" width="9" style="1" customWidth="1"/>
-    <col min="15105" max="15105" width="9.33203125" style="1" customWidth="1"/>
-    <col min="15106" max="15106" width="6.33203125" style="1" customWidth="1"/>
-    <col min="15107" max="15107" width="47" style="1" customWidth="1"/>
-    <col min="15108" max="15108" width="43.33203125" style="1" customWidth="1"/>
-    <col min="15109" max="15109" width="13.33203125" style="1" customWidth="1"/>
-    <col min="15110" max="15110" width="10.6640625" style="1" customWidth="1"/>
-    <col min="15111" max="15111" width="12.44140625" style="1" customWidth="1"/>
-    <col min="15112" max="15112" width="12.109375" style="1" customWidth="1"/>
-    <col min="15113" max="15360" width="9" style="1" customWidth="1"/>
-    <col min="15361" max="15361" width="9.33203125" style="1" customWidth="1"/>
-    <col min="15362" max="15362" width="6.33203125" style="1" customWidth="1"/>
-    <col min="15363" max="15363" width="47" style="1" customWidth="1"/>
-    <col min="15364" max="15364" width="43.33203125" style="1" customWidth="1"/>
-    <col min="15365" max="15365" width="13.33203125" style="1" customWidth="1"/>
-    <col min="15366" max="15366" width="10.6640625" style="1" customWidth="1"/>
-    <col min="15367" max="15367" width="12.44140625" style="1" customWidth="1"/>
-    <col min="15368" max="15368" width="12.109375" style="1" customWidth="1"/>
-    <col min="15369" max="15616" width="9" style="1" customWidth="1"/>
-    <col min="15617" max="15617" width="9.33203125" style="1" customWidth="1"/>
-    <col min="15618" max="15618" width="6.33203125" style="1" customWidth="1"/>
-    <col min="15619" max="15619" width="47" style="1" customWidth="1"/>
-    <col min="15620" max="15620" width="43.33203125" style="1" customWidth="1"/>
-    <col min="15621" max="15621" width="13.33203125" style="1" customWidth="1"/>
-    <col min="15622" max="15622" width="10.6640625" style="1" customWidth="1"/>
-    <col min="15623" max="15623" width="12.44140625" style="1" customWidth="1"/>
-    <col min="15624" max="15624" width="12.109375" style="1" customWidth="1"/>
-    <col min="15625" max="15872" width="9" style="1" customWidth="1"/>
-    <col min="15873" max="15873" width="9.33203125" style="1" customWidth="1"/>
-    <col min="15874" max="15874" width="6.33203125" style="1" customWidth="1"/>
-    <col min="15875" max="15875" width="47" style="1" customWidth="1"/>
-    <col min="15876" max="15876" width="43.33203125" style="1" customWidth="1"/>
-    <col min="15877" max="15877" width="13.33203125" style="1" customWidth="1"/>
-    <col min="15878" max="15878" width="10.6640625" style="1" customWidth="1"/>
-    <col min="15879" max="15879" width="12.44140625" style="1" customWidth="1"/>
-    <col min="15880" max="15880" width="12.109375" style="1" customWidth="1"/>
-    <col min="15881" max="16128" width="9" style="1" customWidth="1"/>
-    <col min="16129" max="16129" width="9.33203125" style="1" customWidth="1"/>
-    <col min="16130" max="16130" width="6.33203125" style="1" customWidth="1"/>
-    <col min="16131" max="16131" width="47" style="1" customWidth="1"/>
-    <col min="16132" max="16132" width="43.33203125" style="1" customWidth="1"/>
-    <col min="16133" max="16133" width="13.33203125" style="1" customWidth="1"/>
-    <col min="16134" max="16134" width="10.6640625" style="1" customWidth="1"/>
-    <col min="16135" max="16135" width="12.44140625" style="1" customWidth="1"/>
-    <col min="16136" max="16136" width="12.109375" style="1" customWidth="1"/>
-    <col min="16137" max="16384" width="9" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33" customWidth="1"/>
+    <col min="2" max="2" width="6.33" customWidth="1"/>
+    <col min="3" max="3" width="37.44" customWidth="1"/>
+    <col min="4" max="4" width="41.11" customWidth="1"/>
+    <col min="5" max="5" width="13.33" customWidth="1"/>
+    <col min="6" max="6" width="10.66" customWidth="1"/>
+    <col min="7" max="7" width="12.44" customWidth="1"/>
+    <col min="8" max="8" width="12.11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -9490,7 +8397,7 @@
     </row>
     <row r="5" ht="20.25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -9527,119 +8434,122 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="108" t="s">
-        <v>249</v>
-      </c>
-      <c r="B7" s="21"/>
-      <c r="C7" s="68"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="31"/>
+      <c r="A7" s="103" t="s">
+        <v>215</v>
+      </c>
+      <c r="B7" s="104"/>
+      <c r="C7" s="105"/>
+      <c r="D7" s="106"/>
+      <c r="E7" s="107"/>
+      <c r="F7" s="107"/>
+      <c r="G7" s="104"/>
+      <c r="H7" s="108"/>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="108" t="s">
-        <v>250</v>
-      </c>
-      <c r="B8" s="21"/>
-      <c r="C8" s="68"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="21"/>
-      <c r="H8" s="31"/>
+      <c r="A8" s="103" t="s">
+        <v>216</v>
+      </c>
+      <c r="B8" s="104"/>
+      <c r="C8" s="105"/>
+      <c r="D8" s="106"/>
+      <c r="E8" s="107"/>
+      <c r="F8" s="107"/>
+      <c r="G8" s="104"/>
+      <c r="H8" s="108"/>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="108" t="s">
-        <v>251</v>
-      </c>
-      <c r="B9" s="21" t="s">
+      <c r="A9" s="103" t="s">
+        <v>217</v>
+      </c>
+      <c r="B9" s="104"/>
+      <c r="C9" s="105"/>
+      <c r="D9" s="106"/>
+      <c r="E9" s="107"/>
+      <c r="F9" s="107"/>
+      <c r="G9" s="104"/>
+      <c r="H9" s="108"/>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="103" t="s">
+        <v>218</v>
+      </c>
+      <c r="B10" s="104" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="109" t="s">
+        <v>219</v>
+      </c>
+      <c r="D10" s="110" t="s">
+        <v>220</v>
+      </c>
+      <c r="E10" s="111" t="s">
+        <v>221</v>
+      </c>
+      <c r="F10" s="111" t="s">
+        <v>222</v>
+      </c>
+      <c r="G10" s="112" t="s">
+        <v>223</v>
+      </c>
+      <c r="H10" s="113" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="103"/>
+      <c r="B11" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="68" t="s">
-        <v>252</v>
-      </c>
-      <c r="D9" s="68" t="s">
-        <v>253</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>253</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>253</v>
-      </c>
-      <c r="G9" s="21" t="s">
-        <v>253</v>
-      </c>
-      <c r="H9" s="31"/>
-    </row>
-    <row r="10" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="108" t="s">
-        <v>254</v>
-      </c>
-      <c r="B10" s="21"/>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
-      <c r="H10" s="31"/>
-    </row>
-    <row r="11" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="108" t="s">
-        <v>255</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="68" t="s">
-        <v>252</v>
-      </c>
-      <c r="D11" s="68" t="s">
-        <v>253</v>
-      </c>
-      <c r="E11" s="21" t="s">
-        <v>253</v>
-      </c>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21" t="s">
-        <v>253</v>
-      </c>
-      <c r="H11" s="31" t="s">
-        <v>253</v>
-      </c>
+      <c r="C11" s="105"/>
+      <c r="D11" s="106"/>
+      <c r="E11" s="107"/>
+      <c r="F11" s="107"/>
+      <c r="G11" s="104"/>
+      <c r="H11" s="108"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="108" t="s">
-        <v>256</v>
-      </c>
-      <c r="B12" s="21"/>
-      <c r="C12" s="68"/>
-      <c r="D12" s="68"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
-      <c r="H12" s="31"/>
+      <c r="A12" s="103" t="s">
+        <v>224</v>
+      </c>
+      <c r="B12" s="104"/>
+      <c r="C12" s="105"/>
+      <c r="D12" s="106"/>
+      <c r="E12" s="107"/>
+      <c r="F12" s="107"/>
+      <c r="G12" s="104"/>
+      <c r="H12" s="108"/>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="108" t="s">
-        <v>257</v>
-      </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="68"/>
-      <c r="D13" s="68"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="31"/>
+      <c r="A13" s="103" t="s">
+        <v>225</v>
+      </c>
+      <c r="B13" s="104"/>
+      <c r="C13" s="105"/>
+      <c r="D13" s="106"/>
+      <c r="E13" s="107"/>
+      <c r="F13" s="107"/>
+      <c r="G13" s="104"/>
+      <c r="H13" s="108"/>
+    </row>
+    <row r="14" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="114" t="s">
+        <v>226</v>
+      </c>
+      <c r="B14" s="115"/>
+      <c r="C14" s="116"/>
+      <c r="D14" s="117"/>
+      <c r="E14" s="118"/>
+      <c r="F14" s="118"/>
+      <c r="G14" s="115"/>
+      <c r="H14" s="119"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A10:A11"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2362204724409449" right="0" top="0.2362204724409449" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>

<commit_message>
sua excel va loi lech ngay
</commit_message>
<xml_diff>
--- a/backend/public/lichmau.xlsx
+++ b/backend/public/lichmau.xlsx
@@ -15,6 +15,7 @@
     <sheet sheetId="7" name="09_02-15_02" state="visible" r:id="rId9"/>
     <sheet sheetId="8" name="23_02-01_03" state="visible" r:id="rId10"/>
     <sheet sheetId="5" name="26_01-01_02" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="09_03-15_03" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'29_12-04_01'!$6:$6</definedName>
@@ -25,13 +26,14 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'09_02-15_02'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'23_02-01_03'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'26_01-01_02'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'09_03-15_03'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="274">
   <si>
     <t>TRƯỜNG ĐẠI HỌC THÁI BÌNH</t>
   </si>
@@ -944,6 +946,37 @@
   <si>
     <t xml:space="preserve">Chủ Nhật
  ngày 01/02</t>
+  </si>
+  <si>
+    <t>(Từ ngày 09/03/2026 đến ngày 15/03/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Hai
+ ngày 09/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Ba
+ ngày 10/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Tư
+ ngày 11/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Năm
+ ngày 12/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Sáu
+ ngày 13/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thứ Bảy
+ ngày 14/03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ Nhật
+ ngày 15/03</t>
   </si>
 </sst>
 </file>
@@ -8555,4 +8588,184 @@
   <pageMargins left="0.2362204724409449" right="0" top="0.2362204724409449" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="9.33" customWidth="1"/>
+    <col min="2" max="2" width="6.33" customWidth="1"/>
+    <col min="3" max="3" width="37.44" customWidth="1"/>
+    <col min="4" max="4" width="41.11" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="7" max="8" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+    </row>
+    <row r="2" ht="18" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" ht="8.1" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+    </row>
+    <row r="4" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" ht="20.25" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="B5" s="10"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+    </row>
+    <row r="6" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="103" t="s">
+        <v>267</v>
+      </c>
+      <c r="B7" s="104"/>
+      <c r="C7" s="105"/>
+      <c r="D7" s="106"/>
+      <c r="E7" s="107"/>
+      <c r="F7" s="107"/>
+      <c r="G7" s="104"/>
+      <c r="H7" s="108"/>
+    </row>
+    <row r="8" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="103" t="s">
+        <v>268</v>
+      </c>
+      <c r="B8" s="104"/>
+      <c r="C8" s="105"/>
+      <c r="D8" s="106"/>
+      <c r="E8" s="107"/>
+      <c r="F8" s="107"/>
+      <c r="G8" s="104"/>
+      <c r="H8" s="108"/>
+    </row>
+    <row r="9" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="103" t="s">
+        <v>269</v>
+      </c>
+      <c r="B9" s="104"/>
+      <c r="C9" s="105"/>
+      <c r="D9" s="106"/>
+      <c r="E9" s="107"/>
+      <c r="F9" s="107"/>
+      <c r="G9" s="104"/>
+      <c r="H9" s="108"/>
+    </row>
+    <row r="10" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="103" t="s">
+        <v>270</v>
+      </c>
+      <c r="B10" s="104"/>
+      <c r="C10" s="105"/>
+      <c r="D10" s="106"/>
+      <c r="E10" s="107"/>
+      <c r="F10" s="107"/>
+      <c r="G10" s="104"/>
+      <c r="H10" s="108"/>
+    </row>
+    <row r="11" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="103" t="s">
+        <v>271</v>
+      </c>
+      <c r="B11" s="104"/>
+      <c r="C11" s="105"/>
+      <c r="D11" s="106"/>
+      <c r="E11" s="107"/>
+      <c r="F11" s="107"/>
+      <c r="G11" s="104"/>
+      <c r="H11" s="108"/>
+    </row>
+    <row r="12" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="103" t="s">
+        <v>272</v>
+      </c>
+      <c r="B12" s="104"/>
+      <c r="C12" s="105"/>
+      <c r="D12" s="106"/>
+      <c r="E12" s="107"/>
+      <c r="F12" s="107"/>
+      <c r="G12" s="104"/>
+      <c r="H12" s="108"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="114" t="s">
+        <v>273</v>
+      </c>
+      <c r="B13" s="115"/>
+      <c r="C13" s="116"/>
+      <c r="D13" s="117"/>
+      <c r="E13" s="118"/>
+      <c r="F13" s="118"/>
+      <c r="G13" s="115"/>
+      <c r="H13" s="119"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A5:H5"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.2362204724409449" right="0" top="0.2362204724409449" bottom="0" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="0" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
 </file>
</xml_diff>